<commit_message>
Hoàn tất kiểm thử TC-21-03
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{195810EC-F29C-45B9-A5AB-57217BF5235C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BF80EFA-055A-482C-859C-E36E662DCB38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1238" uniqueCount="770">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="772">
   <si>
     <t>TEST PLAN – Hệ thống quản lý quán cà phê Làn Mây (Nhóm 5)</t>
   </si>
@@ -2382,6 +2382,12 @@
   </si>
   <si>
     <t>KQ-test\TC-21-02.pdf</t>
+  </si>
+  <si>
+    <t>success: false, "data": null, "maLoi": "SAI_THONG_TIN", "message": "Sai tên đăng nhập hoặc mật khẩu" } ở lại trang đăng nhập</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-21-03.png</t>
   </si>
 </sst>
 </file>
@@ -2588,6 +2594,9 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2596,9 +2605,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2943,66 +2949,66 @@
       <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
     </row>
     <row r="6" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
     </row>
     <row r="7" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
     </row>
     <row r="8" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
     </row>
     <row r="9" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
@@ -3245,79 +3251,79 @@
       <c r="A23" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
     </row>
     <row r="24" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
     </row>
     <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
     </row>
     <row r="26" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
     </row>
     <row r="27" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
     </row>
     <row r="28" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
@@ -3337,13 +3343,13 @@
       <c r="B31" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="C31" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
     </row>
     <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
@@ -3352,13 +3358,13 @@
       <c r="B32" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
     </row>
     <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
@@ -3367,13 +3373,13 @@
       <c r="B33" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="C33" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
     </row>
     <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
@@ -3382,13 +3388,13 @@
       <c r="B34" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C34" s="21" t="s">
+      <c r="C34" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
     </row>
     <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
@@ -3397,13 +3403,13 @@
       <c r="B35" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C35" s="21" t="s">
+      <c r="C35" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-      <c r="G35" s="21"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
     </row>
     <row r="36" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
@@ -3412,13 +3418,13 @@
       <c r="B36" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="21" t="s">
+      <c r="C36" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="21"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="22"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="22"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
@@ -3435,53 +3441,53 @@
       <c r="A39" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B39" s="21" t="s">
+      <c r="B39" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="C39" s="21"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
-      <c r="G39" s="21"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="22"/>
     </row>
     <row r="40" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C40" s="21"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
-      <c r="G40" s="21"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="22"/>
     </row>
     <row r="41" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B41" s="21" t="s">
+      <c r="B41" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="C41" s="21"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
-      <c r="G41" s="21"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
     </row>
     <row r="42" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="B42" s="21" t="s">
+      <c r="B42" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="C42" s="21"/>
-      <c r="D42" s="21"/>
-      <c r="E42" s="21"/>
-      <c r="F42" s="21"/>
-      <c r="G42" s="21"/>
+      <c r="C42" s="22"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="22"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
@@ -3498,53 +3504,53 @@
       <c r="A45" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B45" s="21" t="s">
+      <c r="B45" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="C45" s="21"/>
-      <c r="D45" s="21"/>
-      <c r="E45" s="21"/>
-      <c r="F45" s="21"/>
-      <c r="G45" s="21"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="22"/>
     </row>
     <row r="46" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B46" s="21" t="s">
+      <c r="B46" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="21"/>
-      <c r="G46" s="21"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
     </row>
     <row r="47" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B47" s="21" t="s">
+      <c r="B47" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="C47" s="21"/>
-      <c r="D47" s="21"/>
-      <c r="E47" s="21"/>
-      <c r="F47" s="21"/>
-      <c r="G47" s="21"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
     </row>
     <row r="48" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B48" s="21" t="s">
+      <c r="B48" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="C48" s="21"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="21"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="22"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
@@ -3561,113 +3567,113 @@
       <c r="A51" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B51" s="21" t="s">
+      <c r="B51" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="C51" s="21"/>
-      <c r="D51" s="21"/>
-      <c r="E51" s="21"/>
-      <c r="F51" s="21"/>
-      <c r="G51" s="21"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
     </row>
     <row r="52" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="B52" s="21" t="s">
+      <c r="B52" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="C52" s="21"/>
-      <c r="D52" s="21"/>
-      <c r="E52" s="21"/>
-      <c r="F52" s="21"/>
-      <c r="G52" s="21"/>
+      <c r="C52" s="22"/>
+      <c r="D52" s="22"/>
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="22"/>
     </row>
     <row r="53" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B53" s="21" t="s">
+      <c r="B53" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="C53" s="21"/>
-      <c r="D53" s="21"/>
-      <c r="E53" s="21"/>
-      <c r="F53" s="21"/>
-      <c r="G53" s="21"/>
+      <c r="C53" s="22"/>
+      <c r="D53" s="22"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="22"/>
     </row>
     <row r="54" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B54" s="21" t="s">
+      <c r="B54" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="C54" s="21"/>
-      <c r="D54" s="21"/>
-      <c r="E54" s="21"/>
-      <c r="F54" s="21"/>
-      <c r="G54" s="21"/>
+      <c r="C54" s="22"/>
+      <c r="D54" s="22"/>
+      <c r="E54" s="22"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="22"/>
     </row>
     <row r="55" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B55" s="21" t="s">
+      <c r="B55" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="C55" s="21"/>
-      <c r="D55" s="21"/>
-      <c r="E55" s="21"/>
-      <c r="F55" s="21"/>
-      <c r="G55" s="21"/>
+      <c r="C55" s="22"/>
+      <c r="D55" s="22"/>
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="22"/>
     </row>
     <row r="56" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B56" s="21" t="s">
+      <c r="B56" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="C56" s="21"/>
-      <c r="D56" s="21"/>
-      <c r="E56" s="21"/>
-      <c r="F56" s="21"/>
-      <c r="G56" s="21"/>
+      <c r="C56" s="22"/>
+      <c r="D56" s="22"/>
+      <c r="E56" s="22"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B9:G9"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="B39:G39"/>
-    <mergeCell ref="B40:G40"/>
-    <mergeCell ref="B41:G41"/>
-    <mergeCell ref="B42:G42"/>
-    <mergeCell ref="B45:G45"/>
-    <mergeCell ref="B46:G46"/>
-    <mergeCell ref="B47:G47"/>
-    <mergeCell ref="B48:G48"/>
     <mergeCell ref="B56:G56"/>
     <mergeCell ref="B51:G51"/>
     <mergeCell ref="B52:G52"/>
     <mergeCell ref="B53:G53"/>
     <mergeCell ref="B54:G54"/>
     <mergeCell ref="B55:G55"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B46:G46"/>
+    <mergeCell ref="B47:G47"/>
+    <mergeCell ref="B48:G48"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B9:G9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4230,7 +4236,7 @@
       <c r="L2" s="10" t="s">
         <v>766</v>
       </c>
-      <c r="M2" s="24" t="s">
+      <c r="M2" s="21" t="s">
         <v>767</v>
       </c>
       <c r="N2" s="2"/>
@@ -4272,7 +4278,7 @@
       <c r="L3" s="10" t="s">
         <v>766</v>
       </c>
-      <c r="M3" s="24" t="s">
+      <c r="M3" s="21" t="s">
         <v>769</v>
       </c>
       <c r="N3" s="2" t="s">
@@ -4310,11 +4316,15 @@
       <c r="J4" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="K4" s="2"/>
+      <c r="K4" s="2" t="s">
+        <v>770</v>
+      </c>
       <c r="L4" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="M4" s="2"/>
+        <v>766</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>771</v>
+      </c>
       <c r="N4" s="2"/>
     </row>
     <row r="5" spans="1:14" ht="51" x14ac:dyDescent="0.25">
@@ -6865,6 +6875,7 @@
   <hyperlinks>
     <hyperlink ref="M2" r:id="rId1" xr:uid="{50F66AAF-B0D6-4015-AE81-202020A4C517}"/>
     <hyperlink ref="M3" r:id="rId2" xr:uid="{A82CC3A9-D097-4E0D-BC9C-E140A8961EB2}"/>
+    <hyperlink ref="M4" r:id="rId3" xr:uid="{08D47271-6BFF-47CF-A4E0-50C3B7CBE0C6}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -7094,11 +7105,11 @@
       </c>
       <c r="E5" s="10">
         <f t="shared" ref="E5:E12" si="0">F5+G5</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" s="10">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"PASS")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="10">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"FAIL")</f>
@@ -7106,7 +7117,7 @@
       </c>
       <c r="H5" s="10">
         <f t="shared" ref="H5:H12" si="1">D5-E5</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I5" s="15">
         <f t="shared" ref="I5:I13" si="2">IF(E5=0,"-",F5/E5)</f>
@@ -7404,11 +7415,11 @@
       </c>
       <c r="E13" s="16">
         <f>SUM(E5:E12)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" s="16">
         <f>SUM(F5:F12)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G13" s="16">
         <f>SUM(G5:G12)</f>
@@ -7416,7 +7427,7 @@
       </c>
       <c r="H13" s="16">
         <f>SUM(H5:H12)</f>
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I13" s="18">
         <f t="shared" si="2"/>
@@ -7479,7 +7490,7 @@
       </c>
       <c r="E18" s="10">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"PASS")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" s="10">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"FAIL")</f>
@@ -7649,74 +7660,74 @@
       <c r="A32" s="7" t="s">
         <v>689</v>
       </c>
-      <c r="B32" s="21" t="str">
+      <c r="B32" s="22" t="str">
         <f>"Đã chạy "&amp;E13&amp;" / "&amp;D13&amp;" TC; PASS "&amp;F13&amp;"; FAIL "&amp;G13&amp;"; tỉ lệ pass "&amp;IF(E13=0,"-",TEXT(F13/E13,"0.0%"))</f>
-        <v>Đã chạy 2 / 68 TC; PASS 2; FAIL 0; tỉ lệ pass 100.0%</v>
-      </c>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
+        <v>Đã chạy 3 / 68 TC; PASS 3; FAIL 0; tỉ lệ pass 100.0%</v>
+      </c>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="22"/>
     </row>
     <row r="33" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>690</v>
       </c>
-      <c r="B33" s="22"/>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="22"/>
-      <c r="H33" s="22"/>
-      <c r="I33" s="22"/>
-      <c r="J33" s="22"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="23"/>
+      <c r="J33" s="23"/>
     </row>
     <row r="34" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>691</v>
       </c>
-      <c r="B34" s="22"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="22"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="23"/>
     </row>
     <row r="35" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>692</v>
       </c>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="22"/>
-      <c r="I35" s="22"/>
-      <c r="J35" s="22"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="23"/>
     </row>
     <row r="36" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>693</v>
       </c>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="22"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Hoàn thành kiểm thử TC-21-05
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BF80EFA-055A-482C-859C-E36E662DCB38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4E6AA0-618D-4515-9DE8-0952BE3CD280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="772">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1242" uniqueCount="774">
   <si>
     <t>TEST PLAN – Hệ thống quản lý quán cà phê Làn Mây (Nhóm 5)</t>
   </si>
@@ -849,9 +849,6 @@
   <si>
     <t>(a) username rỗng, password = 123456
 (b) username = phucvu01, password rỗng</t>
-  </si>
-  <si>
-    <t>Cả (a) và (b): HTTP 400, maLoi=THIEU_THONG_TIN. Lỗi hiện ngay dưới ô còn thiếu; không đăng nhập.</t>
   </si>
   <si>
     <t>Giả định: bỏ trống ô không tính vào so_lan_sai [X03].</t>
@@ -2384,10 +2381,19 @@
     <t>KQ-test\TC-21-02.pdf</t>
   </si>
   <si>
-    <t>success: false, "data": null, "maLoi": "SAI_THONG_TIN", "message": "Sai tên đăng nhập hoặc mật khẩu" } ở lại trang đăng nhập</t>
-  </si>
-  <si>
     <t>KQ-test\TC-21-03.png</t>
+  </si>
+  <si>
+    <t>success: false, "data": null, "maLoi": "SAI_THONG_TIN", "message": "Sai tên đăng nhập hoặc mật khẩu" } ở lại trang đăng nhập, solansai có tăng lên 1 và khi đăng nhập đúng thì solansai về lại 0</t>
+  </si>
+  <si>
+    <t>Lỗi hiện ngay dưới ô còn thiếu; không đăng nhập.</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-21-05.png</t>
+  </si>
+  <si>
+    <t>hiển thị lỗi màu đỏ trực tiếp dưới ô input ("Vui lòng nhập tên đăng nhập" / "Vui lòng nhập mật khẩu"), và không tính số lần sai</t>
   </si>
 </sst>
 </file>
@@ -3643,37 +3649,37 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B46:G46"/>
+    <mergeCell ref="B47:G47"/>
+    <mergeCell ref="B48:G48"/>
     <mergeCell ref="B56:G56"/>
     <mergeCell ref="B51:G51"/>
     <mergeCell ref="B52:G52"/>
     <mergeCell ref="B53:G53"/>
     <mergeCell ref="B54:G54"/>
     <mergeCell ref="B55:G55"/>
-    <mergeCell ref="B42:G42"/>
-    <mergeCell ref="B45:G45"/>
-    <mergeCell ref="B46:G46"/>
-    <mergeCell ref="B47:G47"/>
-    <mergeCell ref="B48:G48"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="B39:G39"/>
-    <mergeCell ref="B40:G40"/>
-    <mergeCell ref="B41:G41"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B9:G9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4231,13 +4237,13 @@
         <v>239</v>
       </c>
       <c r="K2" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="L2" s="10" t="s">
         <v>765</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="M2" s="21" t="s">
         <v>766</v>
-      </c>
-      <c r="M2" s="21" t="s">
-        <v>767</v>
       </c>
       <c r="N2" s="2"/>
     </row>
@@ -4273,13 +4279,13 @@
         <v>246</v>
       </c>
       <c r="K3" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="L3" s="10" t="s">
+        <v>765</v>
+      </c>
+      <c r="M3" s="21" t="s">
         <v>768</v>
-      </c>
-      <c r="L3" s="10" t="s">
-        <v>766</v>
-      </c>
-      <c r="M3" s="21" t="s">
-        <v>769</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>247</v>
@@ -4320,10 +4326,10 @@
         <v>770</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="M4" s="21" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="N4" s="2"/>
     </row>
@@ -4356,35 +4362,39 @@
         <v>266</v>
       </c>
       <c r="J5" s="2" t="s">
+        <v>771</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>773</v>
+      </c>
+      <c r="L5" s="10" t="s">
+        <v>765</v>
+      </c>
+      <c r="M5" s="21" t="s">
+        <v>772</v>
+      </c>
+      <c r="N5" s="2" t="s">
         <v>267</v>
-      </c>
-      <c r="K5" s="2"/>
-      <c r="L5" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>272</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>273</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>236</v>
@@ -4393,10 +4403,10 @@
         <v>253</v>
       </c>
       <c r="I6" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>274</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>275</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="10" t="s">
@@ -4404,27 +4414,27 @@
       </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>279</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>236</v>
@@ -4433,10 +4443,10 @@
         <v>253</v>
       </c>
       <c r="I7" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>281</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>282</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="10" t="s">
@@ -4444,39 +4454,39 @@
       </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>295</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>296</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H8" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>298</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>299</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="10" t="s">
@@ -4484,18 +4494,18 @@
       </c>
       <c r="M8" s="2"/>
       <c r="N8" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>233</v>
@@ -4504,19 +4514,19 @@
         <v>234</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H9" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="I9" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>321</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>322</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="10" t="s">
@@ -4527,34 +4537,34 @@
     </row>
     <row r="10" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>325</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>326</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I10" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>327</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>328</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="10" t="s">
@@ -4565,34 +4575,34 @@
     </row>
     <row r="11" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>331</v>
-      </c>
       <c r="F11" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I11" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>332</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>333</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="10" t="s">
@@ -4603,34 +4613,34 @@
     </row>
     <row r="12" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E12" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>336</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>337</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I12" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>338</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>339</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="10" t="s">
@@ -4641,34 +4651,34 @@
     </row>
     <row r="13" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I13" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>343</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>344</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="10" t="s">
@@ -4679,34 +4689,34 @@
     </row>
     <row r="14" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>347</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>348</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I14" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>349</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>350</v>
       </c>
       <c r="K14" s="2"/>
       <c r="L14" s="10" t="s">
@@ -4717,34 +4727,34 @@
     </row>
     <row r="15" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>353</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>354</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H15" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>356</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>357</v>
       </c>
       <c r="K15" s="2"/>
       <c r="L15" s="10" t="s">
@@ -4752,39 +4762,39 @@
       </c>
       <c r="M15" s="2"/>
       <c r="N15" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H16" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>363</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>364</v>
       </c>
       <c r="K16" s="2"/>
       <c r="L16" s="10" t="s">
@@ -4795,34 +4805,34 @@
     </row>
     <row r="17" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>375</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>376</v>
       </c>
       <c r="G17" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H17" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>378</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>379</v>
       </c>
       <c r="K17" s="2"/>
       <c r="L17" s="10" t="s">
@@ -4830,18 +4840,18 @@
       </c>
       <c r="M17" s="2"/>
       <c r="N17" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>233</v>
@@ -4850,19 +4860,19 @@
         <v>234</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G18" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H18" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>391</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>392</v>
       </c>
       <c r="K18" s="2"/>
       <c r="L18" s="10" t="s">
@@ -4873,13 +4883,13 @@
     </row>
     <row r="19" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>233</v>
@@ -4888,19 +4898,19 @@
         <v>234</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="G19" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H19" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>397</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>398</v>
       </c>
       <c r="K19" s="2"/>
       <c r="L19" s="10" t="s">
@@ -4911,13 +4921,13 @@
     </row>
     <row r="20" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>233</v>
@@ -4926,19 +4936,19 @@
         <v>234</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G20" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I20" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="J20" s="2" t="s">
         <v>402</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>403</v>
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="10" t="s">
@@ -4949,34 +4959,34 @@
     </row>
     <row r="21" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>405</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>406</v>
       </c>
       <c r="G21" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I21" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>407</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>408</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="10" t="s">
@@ -4987,34 +4997,34 @@
     </row>
     <row r="22" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G22" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I22" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J22" s="2" t="s">
         <v>411</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>412</v>
       </c>
       <c r="K22" s="2"/>
       <c r="L22" s="10" t="s">
@@ -5025,34 +5035,34 @@
     </row>
     <row r="23" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G23" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I23" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="J23" s="2" t="s">
         <v>416</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>417</v>
       </c>
       <c r="K23" s="2"/>
       <c r="L23" s="10" t="s">
@@ -5063,34 +5073,34 @@
     </row>
     <row r="24" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I24" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="J24" s="2" t="s">
         <v>420</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>421</v>
       </c>
       <c r="K24" s="2"/>
       <c r="L24" s="10" t="s">
@@ -5101,34 +5111,34 @@
     </row>
     <row r="25" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E25" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>424</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>425</v>
       </c>
       <c r="G25" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H25" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="I25" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="J25" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>428</v>
       </c>
       <c r="K25" s="2"/>
       <c r="L25" s="10" t="s">
@@ -5136,18 +5146,18 @@
       </c>
       <c r="M25" s="2"/>
       <c r="N25" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>233</v>
@@ -5156,19 +5166,19 @@
         <v>234</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H26" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="I26" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="J26" s="2" t="s">
         <v>462</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>463</v>
       </c>
       <c r="K26" s="2"/>
       <c r="L26" s="10" t="s">
@@ -5176,39 +5186,39 @@
       </c>
       <c r="M26" s="2"/>
       <c r="N26" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E27" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>467</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>468</v>
       </c>
       <c r="G27" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I27" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="J27" s="2" t="s">
         <v>469</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>470</v>
       </c>
       <c r="K27" s="2"/>
       <c r="L27" s="10" t="s">
@@ -5216,39 +5226,39 @@
       </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C28" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E28" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>473</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>474</v>
       </c>
       <c r="G28" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I28" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="J28" s="2" t="s">
         <v>475</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>476</v>
       </c>
       <c r="K28" s="2"/>
       <c r="L28" s="10" t="s">
@@ -5259,34 +5269,34 @@
     </row>
     <row r="29" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E29" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>492</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>493</v>
       </c>
       <c r="G29" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I29" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="J29" s="2" t="s">
         <v>494</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>495</v>
       </c>
       <c r="K29" s="2"/>
       <c r="L29" s="10" t="s">
@@ -5294,39 +5304,39 @@
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E30" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>499</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>500</v>
       </c>
       <c r="G30" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I30" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="J30" s="2" t="s">
         <v>501</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>502</v>
       </c>
       <c r="K30" s="2"/>
       <c r="L30" s="10" t="s">
@@ -5334,39 +5344,39 @@
       </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="G31" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H31" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="I31" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="J31" s="2" t="s">
         <v>507</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>508</v>
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="10" t="s">
@@ -5383,28 +5393,28 @@
         <v>32</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E32" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>510</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>511</v>
       </c>
       <c r="G32" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H32" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>512</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="J32" s="2" t="s">
         <v>513</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>514</v>
       </c>
       <c r="K32" s="2"/>
       <c r="L32" s="10" t="s">
@@ -5412,39 +5422,39 @@
       </c>
       <c r="M32" s="2"/>
       <c r="N32" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E33" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>518</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>519</v>
       </c>
       <c r="G33" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H33" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="I33" s="2" t="s">
+      <c r="J33" s="2" t="s">
         <v>521</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>522</v>
       </c>
       <c r="K33" s="2"/>
       <c r="L33" s="10" t="s">
@@ -5452,39 +5462,39 @@
       </c>
       <c r="M33" s="2"/>
       <c r="N33" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E34" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>534</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>535</v>
       </c>
       <c r="G34" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H34" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="I34" s="2" t="s">
         <v>536</v>
       </c>
-      <c r="I34" s="2" t="s">
+      <c r="J34" s="2" t="s">
         <v>537</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>538</v>
       </c>
       <c r="K34" s="2"/>
       <c r="L34" s="10" t="s">
@@ -5495,34 +5505,34 @@
     </row>
     <row r="35" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="G35" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H35" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="J35" s="2" t="s">
         <v>553</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>554</v>
       </c>
       <c r="K35" s="2"/>
       <c r="L35" s="10" t="s">
@@ -5533,34 +5543,34 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E36" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>557</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>558</v>
       </c>
       <c r="G36" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H36" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="I36" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="J36" s="2" t="s">
         <v>560</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>561</v>
       </c>
       <c r="K36" s="2"/>
       <c r="L36" s="10" t="s">
@@ -5571,34 +5581,34 @@
     </row>
     <row r="37" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>40</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="G37" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H37" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="J37" s="2" t="s">
         <v>565</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>566</v>
       </c>
       <c r="K37" s="2"/>
       <c r="L37" s="10" t="s">
@@ -5609,34 +5619,34 @@
     </row>
     <row r="38" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>40</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="G38" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H38" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="J38" s="2" t="s">
         <v>569</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>570</v>
       </c>
       <c r="K38" s="2"/>
       <c r="L38" s="10" t="s">
@@ -5647,34 +5657,34 @@
     </row>
     <row r="39" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>40</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="G39" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H39" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="J39" s="2" t="s">
         <v>574</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="J39" s="2" t="s">
-        <v>575</v>
       </c>
       <c r="K39" s="2"/>
       <c r="L39" s="10" t="s">
@@ -5685,34 +5695,34 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>40</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="G40" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H40" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="J40" s="2" t="s">
         <v>578</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>579</v>
       </c>
       <c r="K40" s="2"/>
       <c r="L40" s="10" t="s">
@@ -5720,39 +5730,39 @@
       </c>
       <c r="M40" s="2"/>
       <c r="N40" s="2" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B41" s="10" t="s">
         <v>42</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="G41" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="I41" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="J41" s="2" t="s">
         <v>593</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>594</v>
       </c>
       <c r="K41" s="2"/>
       <c r="L41" s="10" t="s">
@@ -5763,34 +5773,34 @@
     </row>
     <row r="42" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B42" s="10" t="s">
         <v>42</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E42" s="2" t="s">
         <v>596</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>597</v>
-      </c>
       <c r="F42" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="G42" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="I42" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="J42" s="2" t="s">
         <v>598</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>599</v>
       </c>
       <c r="K42" s="2"/>
       <c r="L42" s="10" t="s">
@@ -5798,39 +5808,39 @@
       </c>
       <c r="M42" s="2"/>
       <c r="N42" s="2" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B43" s="10" t="s">
         <v>42</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="G43" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="I43" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="J43" s="2" t="s">
         <v>604</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>605</v>
       </c>
       <c r="K43" s="2"/>
       <c r="L43" s="10" t="s">
@@ -5841,34 +5851,34 @@
     </row>
     <row r="44" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>42</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="G44" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H44" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="I44" s="2" t="s">
         <v>614</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="J44" s="2" t="s">
         <v>615</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>616</v>
       </c>
       <c r="K44" s="2"/>
       <c r="L44" s="10" t="s">
@@ -5876,39 +5886,39 @@
       </c>
       <c r="M44" s="2"/>
       <c r="N44" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="G45" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H45" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>621</v>
       </c>
-      <c r="I45" s="2" t="s">
+      <c r="J45" s="2" t="s">
         <v>622</v>
-      </c>
-      <c r="J45" s="2" t="s">
-        <v>623</v>
       </c>
       <c r="K45" s="2"/>
       <c r="L45" s="10" t="s">
@@ -5919,34 +5929,34 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="G46" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H46" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="I46" s="2" t="s">
         <v>627</v>
       </c>
-      <c r="I46" s="2" t="s">
+      <c r="J46" s="2" t="s">
         <v>628</v>
-      </c>
-      <c r="J46" s="2" t="s">
-        <v>629</v>
       </c>
       <c r="K46" s="2"/>
       <c r="L46" s="10" t="s">
@@ -5957,34 +5967,34 @@
     </row>
     <row r="47" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="G47" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H47" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="I47" s="2" t="s">
         <v>632</v>
       </c>
-      <c r="I47" s="2" t="s">
+      <c r="J47" s="2" t="s">
         <v>633</v>
-      </c>
-      <c r="J47" s="2" t="s">
-        <v>634</v>
       </c>
       <c r="K47" s="2"/>
       <c r="L47" s="10" t="s">
@@ -5995,34 +6005,34 @@
     </row>
     <row r="48" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="G48" s="10" t="s">
         <v>236</v>
       </c>
       <c r="H48" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="J48" s="2" t="s">
         <v>649</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="J48" s="2" t="s">
-        <v>650</v>
       </c>
       <c r="K48" s="2"/>
       <c r="L48" s="10" t="s">
@@ -6033,34 +6043,34 @@
     </row>
     <row r="49" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E49" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="F49" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="G49" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="G49" s="10" t="s">
+      <c r="H49" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="H49" s="2" t="s">
+      <c r="I49" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="I49" s="2" t="s">
+      <c r="J49" s="2" t="s">
         <v>290</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>291</v>
       </c>
       <c r="K49" s="2"/>
       <c r="L49" s="10" t="s">
@@ -6068,39 +6078,39 @@
       </c>
       <c r="M49" s="2"/>
       <c r="N49" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E50" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="G50" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="H50" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="G50" s="10" t="s">
-        <v>288</v>
-      </c>
-      <c r="H50" s="2" t="s">
+      <c r="I50" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="I50" s="2" t="s">
+      <c r="J50" s="2" t="s">
         <v>306</v>
-      </c>
-      <c r="J50" s="2" t="s">
-        <v>307</v>
       </c>
       <c r="K50" s="2"/>
       <c r="L50" s="10" t="s">
@@ -6108,39 +6118,39 @@
       </c>
       <c r="M50" s="2"/>
       <c r="N50" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="51" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B51" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E51" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="F51" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="F51" s="2" t="s">
+      <c r="G51" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="I51" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="G51" s="10" t="s">
-        <v>288</v>
-      </c>
-      <c r="H51" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="I51" s="2" t="s">
+      <c r="J51" s="2" t="s">
         <v>385</v>
-      </c>
-      <c r="J51" s="2" t="s">
-        <v>386</v>
       </c>
       <c r="K51" s="2"/>
       <c r="L51" s="10" t="s">
@@ -6151,34 +6161,34 @@
     </row>
     <row r="52" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B52" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F52" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="G52" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="H52" s="2" t="s">
         <v>541</v>
       </c>
-      <c r="G52" s="10" t="s">
-        <v>288</v>
-      </c>
-      <c r="H52" s="2" t="s">
+      <c r="I52" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="I52" s="2" t="s">
+      <c r="J52" s="2" t="s">
         <v>543</v>
-      </c>
-      <c r="J52" s="2" t="s">
-        <v>544</v>
       </c>
       <c r="K52" s="2"/>
       <c r="L52" s="10" t="s">
@@ -6189,34 +6199,34 @@
     </row>
     <row r="53" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B53" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C53" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="F53" s="2" t="s">
         <v>642</v>
       </c>
-      <c r="D53" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>597</v>
-      </c>
-      <c r="F53" s="2" t="s">
+      <c r="G53" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="H53" s="2" t="s">
         <v>643</v>
       </c>
-      <c r="G53" s="10" t="s">
-        <v>288</v>
-      </c>
-      <c r="H53" s="2" t="s">
+      <c r="I53" s="2" t="s">
         <v>644</v>
       </c>
-      <c r="I53" s="2" t="s">
+      <c r="J53" s="2" t="s">
         <v>645</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>646</v>
       </c>
       <c r="K53" s="2"/>
       <c r="L53" s="10" t="s">
@@ -6265,34 +6275,34 @@
     </row>
     <row r="55" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B55" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E55" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>312</v>
       </c>
       <c r="G55" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H55" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="I55" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="I55" s="2" t="s">
+      <c r="J55" s="2" t="s">
         <v>314</v>
-      </c>
-      <c r="J55" s="2" t="s">
-        <v>315</v>
       </c>
       <c r="K55" s="2"/>
       <c r="L55" s="10" t="s">
@@ -6300,39 +6310,39 @@
       </c>
       <c r="M55" s="2"/>
       <c r="N55" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="56" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E56" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="F56" s="2" t="s">
         <v>367</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>368</v>
       </c>
       <c r="G56" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H56" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="I56" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="I56" s="2" t="s">
+      <c r="J56" s="2" t="s">
         <v>370</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>371</v>
       </c>
       <c r="K56" s="2"/>
       <c r="L56" s="10" t="s">
@@ -6340,39 +6350,39 @@
       </c>
       <c r="M56" s="2"/>
       <c r="N56" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="57" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G57" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="I57" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="J57" s="2" t="s">
         <v>432</v>
-      </c>
-      <c r="J57" s="2" t="s">
-        <v>433</v>
       </c>
       <c r="K57" s="2"/>
       <c r="L57" s="10" t="s">
@@ -6383,34 +6393,34 @@
     </row>
     <row r="58" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A58" s="9" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B58" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G58" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H58" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="I58" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="I58" s="2" t="s">
+      <c r="J58" s="2" t="s">
         <v>437</v>
-      </c>
-      <c r="J58" s="2" t="s">
-        <v>438</v>
       </c>
       <c r="K58" s="2"/>
       <c r="L58" s="10" t="s">
@@ -6421,34 +6431,34 @@
     </row>
     <row r="59" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B59" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="G59" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H59" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="I59" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="I59" s="2" t="s">
+      <c r="J59" s="2" t="s">
         <v>443</v>
-      </c>
-      <c r="J59" s="2" t="s">
-        <v>444</v>
       </c>
       <c r="K59" s="2"/>
       <c r="L59" s="10" t="s">
@@ -6459,34 +6469,34 @@
     </row>
     <row r="60" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B60" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E60" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>448</v>
       </c>
       <c r="G60" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H60" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="I60" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="I60" s="2" t="s">
+      <c r="J60" s="2" t="s">
         <v>450</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>451</v>
       </c>
       <c r="K60" s="2"/>
       <c r="L60" s="10" t="s">
@@ -6497,34 +6507,34 @@
     </row>
     <row r="61" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B61" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E61" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="F61" s="2" t="s">
         <v>454</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>455</v>
       </c>
       <c r="G61" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I61" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="J61" s="2" t="s">
         <v>456</v>
-      </c>
-      <c r="J61" s="2" t="s">
-        <v>457</v>
       </c>
       <c r="K61" s="2"/>
       <c r="L61" s="10" t="s">
@@ -6535,34 +6545,34 @@
     </row>
     <row r="62" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E62" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>479</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>480</v>
       </c>
       <c r="G62" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I62" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="J62" s="2" t="s">
         <v>481</v>
-      </c>
-      <c r="J62" s="2" t="s">
-        <v>482</v>
       </c>
       <c r="K62" s="2"/>
       <c r="L62" s="10" t="s">
@@ -6570,39 +6580,39 @@
       </c>
       <c r="M62" s="2"/>
       <c r="N62" s="2" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="63" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A63" s="9" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E63" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="F63" s="2" t="s">
         <v>486</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>487</v>
       </c>
       <c r="G63" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I63" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="J63" s="2" t="s">
         <v>488</v>
-      </c>
-      <c r="J63" s="2" t="s">
-        <v>489</v>
       </c>
       <c r="K63" s="2"/>
       <c r="L63" s="10" t="s">
@@ -6613,34 +6623,34 @@
     </row>
     <row r="64" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>525</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="E64" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="F64" s="2" t="s">
         <v>527</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>528</v>
       </c>
       <c r="G64" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I64" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="J64" s="2" t="s">
         <v>529</v>
-      </c>
-      <c r="J64" s="2" t="s">
-        <v>530</v>
       </c>
       <c r="K64" s="2"/>
       <c r="L64" s="10" t="s">
@@ -6648,39 +6658,39 @@
       </c>
       <c r="M64" s="2"/>
       <c r="N64" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="65" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B65" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E65" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="F65" s="2" t="s">
         <v>534</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>535</v>
       </c>
       <c r="G65" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H65" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="I65" s="2" t="s">
         <v>547</v>
       </c>
-      <c r="I65" s="2" t="s">
+      <c r="J65" s="2" t="s">
         <v>548</v>
-      </c>
-      <c r="J65" s="2" t="s">
-        <v>549</v>
       </c>
       <c r="K65" s="2"/>
       <c r="L65" s="10" t="s">
@@ -6691,34 +6701,34 @@
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="9" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>40</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="G66" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H66" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="J66" s="2" t="s">
         <v>583</v>
-      </c>
-      <c r="I66" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="J66" s="2" t="s">
-        <v>584</v>
       </c>
       <c r="K66" s="2"/>
       <c r="L66" s="10" t="s">
@@ -6729,34 +6739,34 @@
     </row>
     <row r="67" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>40</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="G67" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H67" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="J67" s="2" t="s">
         <v>588</v>
-      </c>
-      <c r="I67" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="J67" s="2" t="s">
-        <v>589</v>
       </c>
       <c r="K67" s="2"/>
       <c r="L67" s="10" t="s">
@@ -6767,34 +6777,34 @@
     </row>
     <row r="68" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A68" s="9" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>42</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>250</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="G68" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="I68" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="J68" s="2" t="s">
         <v>609</v>
-      </c>
-      <c r="J68" s="2" t="s">
-        <v>610</v>
       </c>
       <c r="K68" s="2"/>
       <c r="L68" s="10" t="s">
@@ -6805,34 +6815,34 @@
     </row>
     <row r="69" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A69" s="9" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="G69" s="10" t="s">
         <v>259</v>
       </c>
       <c r="H69" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="I69" s="2" t="s">
         <v>638</v>
       </c>
-      <c r="I69" s="2" t="s">
+      <c r="J69" s="2" t="s">
         <v>639</v>
-      </c>
-      <c r="J69" s="2" t="s">
-        <v>640</v>
       </c>
       <c r="K69" s="2"/>
       <c r="L69" s="10" t="s">
@@ -6876,6 +6886,7 @@
     <hyperlink ref="M2" r:id="rId1" xr:uid="{50F66AAF-B0D6-4015-AE81-202020A4C517}"/>
     <hyperlink ref="M3" r:id="rId2" xr:uid="{A82CC3A9-D097-4E0D-BC9C-E140A8961EB2}"/>
     <hyperlink ref="M4" r:id="rId3" xr:uid="{08D47271-6BFF-47CF-A4E0-50C3B7CBE0C6}"/>
+    <hyperlink ref="M5" r:id="rId4" xr:uid="{9F651E7B-E02C-482C-A9C3-B48CE366708D}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6902,68 +6913,68 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>652</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>654</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="E2" s="8" t="s">
         <v>655</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>656</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="H2" s="12" t="s">
         <v>658</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="I2" s="12" t="s">
         <v>659</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="J2" s="12" t="s">
         <v>660</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="51" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
+        <v>661</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>350</v>
+      </c>
+      <c r="C3" s="14" t="s">
         <v>662</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>351</v>
-      </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" s="14" t="s">
         <v>663</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="E3" s="14" t="s">
         <v>664</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="F3" s="14" t="s">
         <v>665</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="G3" s="13" t="s">
         <v>666</v>
-      </c>
-      <c r="G3" s="13" t="s">
-        <v>667</v>
       </c>
       <c r="H3" s="13" t="s">
         <v>29</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="J3" s="14"/>
     </row>
@@ -7049,12 +7060,12 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -7065,28 +7076,28 @@
         <v>15</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>670</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>671</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="E4" s="8" t="s">
         <v>672</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="F4" s="8" t="s">
         <v>673</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="G4" s="8" t="s">
         <v>674</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>675</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>240</v>
       </c>
       <c r="I4" s="8" t="s">
+        <v>675</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>676</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -7105,11 +7116,11 @@
       </c>
       <c r="E5" s="10">
         <f t="shared" ref="E5:E12" si="0">F5+G5</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="10">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"PASS")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5" s="10">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"FAIL")</f>
@@ -7117,7 +7128,7 @@
       </c>
       <c r="H5" s="10">
         <f t="shared" ref="H5:H12" si="1">D5-E5</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I5" s="15">
         <f t="shared" ref="I5:I13" si="2">IF(E5=0,"-",F5/E5)</f>
@@ -7403,10 +7414,10 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
+        <v>677</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>678</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>679</v>
       </c>
       <c r="C13" s="17"/>
       <c r="D13" s="16">
@@ -7415,11 +7426,11 @@
       </c>
       <c r="E13" s="16">
         <f>SUM(E5:E12)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F13" s="16">
         <f>SUM(F5:F12)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" s="16">
         <f>SUM(G5:G12)</f>
@@ -7427,7 +7438,7 @@
       </c>
       <c r="H13" s="16">
         <f>SUM(H5:H12)</f>
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I13" s="18">
         <f t="shared" si="2"/>
@@ -7440,7 +7451,7 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -7450,13 +7461,13 @@
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="E16" s="8" t="s">
+        <v>673</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>674</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>675</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -7490,7 +7501,7 @@
       </c>
       <c r="E18" s="10">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"PASS")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="10">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"FAIL")</f>
@@ -7499,7 +7510,7 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -7537,7 +7548,7 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -7556,28 +7567,28 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="E25" s="8" t="s">
+        <v>682</v>
+      </c>
+      <c r="F25" s="8" t="s">
         <v>683</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>684</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -7596,7 +7607,7 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -7615,7 +7626,7 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -7634,7 +7645,7 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -7653,16 +7664,16 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="B32" s="22" t="str">
         <f>"Đã chạy "&amp;E13&amp;" / "&amp;D13&amp;" TC; PASS "&amp;F13&amp;"; FAIL "&amp;G13&amp;"; tỉ lệ pass "&amp;IF(E13=0,"-",TEXT(F13/E13,"0.0%"))</f>
-        <v>Đã chạy 3 / 68 TC; PASS 3; FAIL 0; tỉ lệ pass 100.0%</v>
+        <v>Đã chạy 4 / 68 TC; PASS 4; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
       <c r="C32" s="22"/>
       <c r="D32" s="22"/>
@@ -7675,7 +7686,7 @@
     </row>
     <row r="33" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B33" s="23"/>
       <c r="C33" s="23"/>
@@ -7689,7 +7700,7 @@
     </row>
     <row r="34" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B34" s="23"/>
       <c r="C34" s="23"/>
@@ -7703,7 +7714,7 @@
     </row>
     <row r="35" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B35" s="23"/>
       <c r="C35" s="23"/>
@@ -7717,7 +7728,7 @@
     </row>
     <row r="36" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B36" s="23"/>
       <c r="C36" s="23"/>
@@ -7762,95 +7773,95 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="8" t="s">
+        <v>695</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>696</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="E2" s="8" t="s">
         <v>697</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>698</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="12" t="s">
         <v>699</v>
       </c>
-      <c r="G2" s="12" t="s">
-        <v>700</v>
-      </c>
       <c r="H2" s="12" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>702</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>703</v>
       </c>
       <c r="E3" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>706</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>707</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>709</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>710</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>711</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>24</v>
@@ -7860,319 +7871,319 @@
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>713</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="10" t="s">
         <v>714</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="F6" s="2" t="s">
         <v>715</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>716</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>716</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>717</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="C7" s="2" t="s">
         <v>718</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>719</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="10" t="s">
         <v>720</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="F7" s="2" t="s">
         <v>721</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>722</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="20" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>725</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>726</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>729</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>730</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
+        <v>730</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>717</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>731</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>718</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>732</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>733</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>738</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>739</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>741</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>742</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="10" t="s">
         <v>743</v>
       </c>
-      <c r="E13" s="10" t="s">
-        <v>744</v>
-      </c>
       <c r="F13" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>23</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>745</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>746</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="10" t="s">
         <v>747</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="F14" s="2" t="s">
         <v>748</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>749</v>
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>750</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>751</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>752</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>207</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>755</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>756</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>26</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
+        <v>759</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>760</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="C18" s="2" t="s">
         <v>761</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>762</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="10" t="s">
+        <v>714</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>763</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>715</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>764</v>
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="20" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Hoàn thành kiểm thử TC-21-06
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4E6AA0-618D-4515-9DE8-0952BE3CD280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E16B451B-556A-4310-9182-CDEB3E4ADA36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1242" uniqueCount="774">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1244" uniqueCount="776">
   <si>
     <t>TEST PLAN – Hệ thống quản lý quán cà phê Làn Mây (Nhóm 5)</t>
   </si>
@@ -2394,6 +2394,12 @@
   </si>
   <si>
     <t>hiển thị lỗi màu đỏ trực tiếp dưới ô input ("Vui lòng nhập tên đăng nhập" / "Vui lòng nhập mật khẩu"), và không tính số lần sai</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-21-06.png</t>
+  </si>
+  <si>
+    <t>4 lần đầu đăng nhập sai vẫn chưa bị khóa đến lần 5 đăng nhập đúng vào đúng màn hình. Và solansai cũng về 0.</t>
   </si>
 </sst>
 </file>
@@ -3649,37 +3655,37 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B9:G9"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="B39:G39"/>
-    <mergeCell ref="B40:G40"/>
-    <mergeCell ref="B41:G41"/>
-    <mergeCell ref="B42:G42"/>
-    <mergeCell ref="B45:G45"/>
-    <mergeCell ref="B46:G46"/>
-    <mergeCell ref="B47:G47"/>
-    <mergeCell ref="B48:G48"/>
     <mergeCell ref="B56:G56"/>
     <mergeCell ref="B51:G51"/>
     <mergeCell ref="B52:G52"/>
     <mergeCell ref="B53:G53"/>
     <mergeCell ref="B54:G54"/>
     <mergeCell ref="B55:G55"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B46:G46"/>
+    <mergeCell ref="B47:G47"/>
+    <mergeCell ref="B48:G48"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B9:G9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4408,11 +4414,15 @@
       <c r="J6" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="K6" s="2"/>
+      <c r="K6" s="2" t="s">
+        <v>775</v>
+      </c>
       <c r="L6" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="M6" s="2"/>
+        <v>765</v>
+      </c>
+      <c r="M6" s="21" t="s">
+        <v>774</v>
+      </c>
       <c r="N6" s="2" t="s">
         <v>275</v>
       </c>
@@ -6887,6 +6897,7 @@
     <hyperlink ref="M3" r:id="rId2" xr:uid="{A82CC3A9-D097-4E0D-BC9C-E140A8961EB2}"/>
     <hyperlink ref="M4" r:id="rId3" xr:uid="{08D47271-6BFF-47CF-A4E0-50C3B7CBE0C6}"/>
     <hyperlink ref="M5" r:id="rId4" xr:uid="{9F651E7B-E02C-482C-A9C3-B48CE366708D}"/>
+    <hyperlink ref="M6" r:id="rId5" xr:uid="{A864ECE4-9FCB-49E2-B4CA-C451B08DAD6B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -7116,11 +7127,11 @@
       </c>
       <c r="E5" s="10">
         <f t="shared" ref="E5:E12" si="0">F5+G5</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F5" s="10">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"PASS")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5" s="10">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"FAIL")</f>
@@ -7128,7 +7139,7 @@
       </c>
       <c r="H5" s="10">
         <f t="shared" ref="H5:H12" si="1">D5-E5</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I5" s="15">
         <f t="shared" ref="I5:I13" si="2">IF(E5=0,"-",F5/E5)</f>
@@ -7426,11 +7437,11 @@
       </c>
       <c r="E13" s="16">
         <f>SUM(E5:E12)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F13" s="16">
         <f>SUM(F5:F12)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G13" s="16">
         <f>SUM(G5:G12)</f>
@@ -7438,7 +7449,7 @@
       </c>
       <c r="H13" s="16">
         <f>SUM(H5:H12)</f>
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I13" s="18">
         <f t="shared" si="2"/>
@@ -7520,7 +7531,7 @@
       </c>
       <c r="E19" s="10">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"PASS")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="10">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"FAIL")</f>
@@ -7673,7 +7684,7 @@
       </c>
       <c r="B32" s="22" t="str">
         <f>"Đã chạy "&amp;E13&amp;" / "&amp;D13&amp;" TC; PASS "&amp;F13&amp;"; FAIL "&amp;G13&amp;"; tỉ lệ pass "&amp;IF(E13=0,"-",TEXT(F13/E13,"0.0%"))</f>
-        <v>Đã chạy 4 / 68 TC; PASS 4; FAIL 0; tỉ lệ pass 100.0%</v>
+        <v>Đã chạy 5 / 68 TC; PASS 5; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
       <c r="C32" s="22"/>
       <c r="D32" s="22"/>

</xml_diff>

<commit_message>
Hoàn tất kiêm thử TC-01-01
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA179AD-E711-4667-96E4-50C4828CA584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F877A3C-8A05-47A1-BBEF-43DAD686AE71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="506">
   <si>
     <t>UC</t>
   </si>
@@ -1574,6 +1574,15 @@
   </si>
   <si>
     <t>KQ-test\TC-21-07.png</t>
+  </si>
+  <si>
+    <t>HTTP 403 Forbidden, thông báo đỏ tài khoản đã bị vô hiệu hóa, vui lòng liên hệ chủ quán</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-21-09.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-01-01.png</t>
   </si>
 </sst>
 </file>
@@ -2401,11 +2410,15 @@
       <c r="J8" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="K8" s="1"/>
+      <c r="K8" s="1" t="s">
+        <v>503</v>
+      </c>
       <c r="L8" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M8" s="1"/>
+        <v>490</v>
+      </c>
+      <c r="M8" s="14" t="s">
+        <v>504</v>
+      </c>
       <c r="N8" s="1" t="s">
         <v>103</v>
       </c>
@@ -2441,11 +2454,15 @@
       <c r="J9" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="K9" s="1"/>
+      <c r="K9" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="L9" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M9" s="1"/>
+        <v>490</v>
+      </c>
+      <c r="M9" s="14" t="s">
+        <v>505</v>
+      </c>
       <c r="N9" s="1"/>
     </row>
     <row r="10" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
@@ -4802,6 +4819,8 @@
     <hyperlink ref="M5" r:id="rId4" xr:uid="{9F651E7B-E02C-482C-A9C3-B48CE366708D}"/>
     <hyperlink ref="M6" r:id="rId5" xr:uid="{A864ECE4-9FCB-49E2-B4CA-C451B08DAD6B}"/>
     <hyperlink ref="M7" r:id="rId6" xr:uid="{A93B080E-95D8-407A-B7EF-3EF80B22C84E}"/>
+    <hyperlink ref="M8" r:id="rId7" xr:uid="{6B3DF791-B948-4A8E-A3AC-C8A2DC934749}"/>
+    <hyperlink ref="M9" r:id="rId8" xr:uid="{54F1630E-C33A-44D8-AF37-43D154BB6BAD}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4991,11 +5010,11 @@
       </c>
       <c r="E4" s="6">
         <f t="shared" ref="E4:E11" si="0">F4+G4</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F4" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A4,'Test Case'!$L:$L,"PASS")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G4" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A4,'Test Case'!$L:$L,"FAIL")</f>
@@ -5003,7 +5022,7 @@
       </c>
       <c r="H4" s="6">
         <f t="shared" ref="H4:H11" si="1">D4-E4</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I4" s="9">
         <f t="shared" ref="I4:I12" si="2">IF(E4=0,"-",F4/E4)</f>
@@ -5030,11 +5049,11 @@
       </c>
       <c r="E5" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"PASS")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"FAIL")</f>
@@ -5042,11 +5061,11 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="1"/>
-        <v>11</v>
-      </c>
-      <c r="I5" s="9" t="str">
+        <v>10</v>
+      </c>
+      <c r="I5" s="9">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>1</v>
       </c>
       <c r="J5" s="6">
         <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A5,2)&amp;"-*")</f>
@@ -5301,11 +5320,11 @@
       </c>
       <c r="E12" s="10">
         <f>SUM(E4:E11)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F12" s="10">
         <f>SUM(F4:F11)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G12" s="10">
         <f>SUM(G4:G11)</f>
@@ -5313,7 +5332,7 @@
       </c>
       <c r="H12" s="10">
         <f>SUM(H4:H11)</f>
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" si="2"/>
@@ -5357,7 +5376,7 @@
       </c>
       <c r="E16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"PASS")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"FAIL")</f>
@@ -5414,7 +5433,7 @@
       </c>
       <c r="E19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"PASS")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"FAIL")</f>
@@ -5548,7 +5567,7 @@
       </c>
       <c r="B31" s="15" t="str">
         <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
-        <v>Đã chạy 6 / 68 TC; PASS 6; FAIL 0; tỉ lệ pass 100.0%</v>
+        <v>Đã chạy 8 / 68 TC; PASS 8; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>

</xml_diff>

<commit_message>
hoàn thành kiểm thử TC-01-02
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F877A3C-8A05-47A1-BBEF-43DAD686AE71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1126C25F-724C-407C-9BCB-2E92C75F72BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="507">
   <si>
     <t>UC</t>
   </si>
@@ -1583,6 +1583,9 @@
   </si>
   <si>
     <t>KQ-test\TC-01-01.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-01-02.png</t>
   </si>
 </sst>
 </file>
@@ -2496,11 +2499,15 @@
       <c r="J10" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="K10" s="1"/>
+      <c r="K10" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="L10" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M10" s="1"/>
+        <v>490</v>
+      </c>
+      <c r="M10" s="14" t="s">
+        <v>506</v>
+      </c>
       <c r="N10" s="1"/>
     </row>
     <row r="11" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
@@ -4821,6 +4828,7 @@
     <hyperlink ref="M7" r:id="rId6" xr:uid="{A93B080E-95D8-407A-B7EF-3EF80B22C84E}"/>
     <hyperlink ref="M8" r:id="rId7" xr:uid="{6B3DF791-B948-4A8E-A3AC-C8A2DC934749}"/>
     <hyperlink ref="M9" r:id="rId8" xr:uid="{54F1630E-C33A-44D8-AF37-43D154BB6BAD}"/>
+    <hyperlink ref="M10" r:id="rId9" xr:uid="{23368E01-5C93-453F-9C9A-97753332BDA4}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5049,11 +5057,11 @@
       </c>
       <c r="E5" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"PASS")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"FAIL")</f>
@@ -5061,7 +5069,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" si="2"/>
@@ -5320,11 +5328,11 @@
       </c>
       <c r="E12" s="10">
         <f>SUM(E4:E11)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F12" s="10">
         <f>SUM(F4:F11)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G12" s="10">
         <f>SUM(G4:G11)</f>
@@ -5332,7 +5340,7 @@
       </c>
       <c r="H12" s="10">
         <f>SUM(H4:H11)</f>
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" si="2"/>
@@ -5414,7 +5422,7 @@
       </c>
       <c r="E18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"PASS")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"FAIL")</f>
@@ -5567,7 +5575,7 @@
       </c>
       <c r="B31" s="15" t="str">
         <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
-        <v>Đã chạy 8 / 68 TC; PASS 8; FAIL 0; tỉ lệ pass 100.0%</v>
+        <v>Đã chạy 9 / 68 TC; PASS 9; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>

</xml_diff>

<commit_message>
hoàn thành kiểm thử TC-01-03
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1126C25F-724C-407C-9BCB-2E92C75F72BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4271788D-A2C1-406D-86A0-DD9A3CE75B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="508">
   <si>
     <t>UC</t>
   </si>
@@ -1586,6 +1586,9 @@
   </si>
   <si>
     <t>KQ-test\TC-01-02.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-01-03.png</t>
   </si>
 </sst>
 </file>
@@ -2541,11 +2544,15 @@
       <c r="J11" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="K11" s="1"/>
+      <c r="K11" s="1" t="s">
+        <v>136</v>
+      </c>
       <c r="L11" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M11" s="1"/>
+        <v>490</v>
+      </c>
+      <c r="M11" s="14" t="s">
+        <v>507</v>
+      </c>
       <c r="N11" s="1"/>
     </row>
     <row r="12" spans="1:14" ht="51" x14ac:dyDescent="0.25">
@@ -4829,6 +4836,7 @@
     <hyperlink ref="M8" r:id="rId7" xr:uid="{6B3DF791-B948-4A8E-A3AC-C8A2DC934749}"/>
     <hyperlink ref="M9" r:id="rId8" xr:uid="{54F1630E-C33A-44D8-AF37-43D154BB6BAD}"/>
     <hyperlink ref="M10" r:id="rId9" xr:uid="{23368E01-5C93-453F-9C9A-97753332BDA4}"/>
+    <hyperlink ref="M11" r:id="rId10" xr:uid="{052C7473-5CF6-451A-BECC-1E425E96FDD2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5057,11 +5065,11 @@
       </c>
       <c r="E5" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"PASS")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"FAIL")</f>
@@ -5069,7 +5077,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" si="2"/>
@@ -5328,11 +5336,11 @@
       </c>
       <c r="E12" s="10">
         <f>SUM(E4:E11)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F12" s="10">
         <f>SUM(F4:F11)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G12" s="10">
         <f>SUM(G4:G11)</f>
@@ -5340,7 +5348,7 @@
       </c>
       <c r="H12" s="10">
         <f>SUM(H4:H11)</f>
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" si="2"/>
@@ -5422,7 +5430,7 @@
       </c>
       <c r="E18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"PASS")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"FAIL")</f>
@@ -5575,7 +5583,7 @@
       </c>
       <c r="B31" s="15" t="str">
         <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
-        <v>Đã chạy 9 / 68 TC; PASS 9; FAIL 0; tỉ lệ pass 100.0%</v>
+        <v>Đã chạy 10 / 68 TC; PASS 10; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>

</xml_diff>

<commit_message>
hoàn tất kiểm thử TC-01-08
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4271788D-A2C1-406D-86A0-DD9A3CE75B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518F2332-A5C1-437F-826A-9022B3EA2E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="512">
   <si>
     <t>UC</t>
   </si>
@@ -1589,6 +1589,18 @@
   </si>
   <si>
     <t>KQ-test\TC-01-03.png</t>
+  </si>
+  <si>
+    <t>Giao diện chỉ có cho số lượng 1 ấn dấu - số lượng không bị thay đổi</t>
+  </si>
+  <si>
+    <t>Giao diện chỉ có cho số lượng 100 ấn dấu + số lượng không bị thay đổi</t>
+  </si>
+  <si>
+    <t>Giao diện: món hiện xám, không chọn được. message: bạc xĩu đã hết nguyên liệu và  bàn vẫn trống</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-01-07.png</t>
   </si>
 </sst>
 </file>
@@ -2586,9 +2598,11 @@
       <c r="J12" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="K12" s="1"/>
+      <c r="K12" s="1" t="s">
+        <v>508</v>
+      </c>
       <c r="L12" s="6" t="s">
-        <v>44</v>
+        <v>490</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
@@ -2624,9 +2638,11 @@
       <c r="J13" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="K13" s="1"/>
+      <c r="K13" s="1" t="s">
+        <v>508</v>
+      </c>
       <c r="L13" s="6" t="s">
-        <v>44</v>
+        <v>490</v>
       </c>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
@@ -2662,9 +2678,11 @@
       <c r="J14" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="K14" s="1"/>
+      <c r="K14" s="1" t="s">
+        <v>509</v>
+      </c>
       <c r="L14" s="6" t="s">
-        <v>44</v>
+        <v>490</v>
       </c>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
@@ -2700,11 +2718,15 @@
       <c r="J15" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="K15" s="1"/>
+      <c r="K15" s="1" t="s">
+        <v>510</v>
+      </c>
       <c r="L15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M15" s="1"/>
+        <v>490</v>
+      </c>
+      <c r="M15" s="14" t="s">
+        <v>511</v>
+      </c>
       <c r="N15" s="1" t="s">
         <v>161</v>
       </c>
@@ -4837,6 +4859,7 @@
     <hyperlink ref="M9" r:id="rId8" xr:uid="{54F1630E-C33A-44D8-AF37-43D154BB6BAD}"/>
     <hyperlink ref="M10" r:id="rId9" xr:uid="{23368E01-5C93-453F-9C9A-97753332BDA4}"/>
     <hyperlink ref="M11" r:id="rId10" xr:uid="{052C7473-5CF6-451A-BECC-1E425E96FDD2}"/>
+    <hyperlink ref="M15" r:id="rId11" xr:uid="{0DC140F7-DC54-47D0-8FE4-B05287842DF7}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5065,11 +5088,11 @@
       </c>
       <c r="E5" s="6">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"PASS")</f>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"FAIL")</f>
@@ -5077,7 +5100,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" si="2"/>
@@ -5336,11 +5359,11 @@
       </c>
       <c r="E12" s="10">
         <f>SUM(E4:E11)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F12" s="10">
         <f>SUM(F4:F11)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G12" s="10">
         <f>SUM(G4:G11)</f>
@@ -5348,7 +5371,7 @@
       </c>
       <c r="H12" s="10">
         <f>SUM(H4:H11)</f>
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" si="2"/>
@@ -5411,7 +5434,7 @@
       </c>
       <c r="E17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"PASS")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"FAIL")</f>
@@ -5430,7 +5453,7 @@
       </c>
       <c r="E18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"PASS")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"FAIL")</f>
@@ -5449,7 +5472,7 @@
       </c>
       <c r="E19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"PASS")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"FAIL")</f>
@@ -5583,7 +5606,7 @@
       </c>
       <c r="B31" s="15" t="str">
         <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
-        <v>Đã chạy 10 / 68 TC; PASS 10; FAIL 0; tỉ lệ pass 100.0%</v>
+        <v>Đã chạy 14 / 68 TC; PASS 14; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>

</xml_diff>

<commit_message>
Hoàn thành kiểm thử TC-01-08
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518F2332-A5C1-437F-826A-9022B3EA2E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C0AFB6-A0BC-431F-BC26-9578666FE0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="514">
   <si>
     <t>UC</t>
   </si>
@@ -1601,6 +1601,12 @@
   </si>
   <si>
     <t>KQ-test\TC-01-07.png</t>
+  </si>
+  <si>
+    <t>bàn cân dọn không gọi món được, hiện message cần dọn bàn</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-01-08.png</t>
   </si>
 </sst>
 </file>
@@ -2762,11 +2768,15 @@
       <c r="J16" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="K16" s="1"/>
+      <c r="K16" s="1" t="s">
+        <v>512</v>
+      </c>
       <c r="L16" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M16" s="1"/>
+        <v>490</v>
+      </c>
+      <c r="M16" s="14" t="s">
+        <v>513</v>
+      </c>
       <c r="N16" s="1"/>
     </row>
     <row r="17" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
@@ -4860,6 +4870,7 @@
     <hyperlink ref="M10" r:id="rId9" xr:uid="{23368E01-5C93-453F-9C9A-97753332BDA4}"/>
     <hyperlink ref="M11" r:id="rId10" xr:uid="{052C7473-5CF6-451A-BECC-1E425E96FDD2}"/>
     <hyperlink ref="M15" r:id="rId11" xr:uid="{0DC140F7-DC54-47D0-8FE4-B05287842DF7}"/>
+    <hyperlink ref="M16" r:id="rId12" xr:uid="{4D3489F9-5D17-474D-9677-E57F0217832E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5088,11 +5099,11 @@
       </c>
       <c r="E5" s="6">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"PASS")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"FAIL")</f>
@@ -5100,7 +5111,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" si="2"/>
@@ -5359,11 +5370,11 @@
       </c>
       <c r="E12" s="10">
         <f>SUM(E4:E11)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" s="10">
         <f>SUM(F4:F11)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G12" s="10">
         <f>SUM(G4:G11)</f>
@@ -5371,7 +5382,7 @@
       </c>
       <c r="H12" s="10">
         <f>SUM(H4:H11)</f>
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" si="2"/>
@@ -5472,7 +5483,7 @@
       </c>
       <c r="E19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"PASS")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"FAIL")</f>
@@ -5606,7 +5617,7 @@
       </c>
       <c r="B31" s="15" t="str">
         <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
-        <v>Đã chạy 14 / 68 TC; PASS 14; FAIL 0; tỉ lệ pass 100.0%</v>
+        <v>Đã chạy 15 / 68 TC; PASS 15; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>

</xml_diff>

<commit_message>
Hoàn thành kiểm thử TC-04-01
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C0AFB6-A0BC-431F-BC26-9578666FE0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A35D55-0AF0-4FC9-9B3C-F1807116C953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Tổng hợp" sheetId="6" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Case'!$A$1:$N$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Case'!$A$1:$N$68</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="508">
   <si>
     <t>UC</t>
   </si>
@@ -584,31 +584,6 @@
     <t>Đề xuất của Tuấn trong contract, chưa chốt [X01]. Nếu chốt khác thì sửa Expected.</t>
   </si>
   <si>
-    <t>TC-01-10</t>
-  </si>
-  <si>
-    <t>Bếp không phản hồi sau 5 giây: đơn vẫn lưu, isSynced=false</t>
-  </si>
-  <si>
-    <t>Black-box theo UC Spec (EF: bếp không phản hồi)</t>
-  </si>
-  <si>
-    <t>SD Tạo order (msg 2–25); api-contract §3 UC01 (POST /orders); BPC T3 (guiOrderDenKDS, danhDauChuaDongBo)</t>
-  </si>
-  <si>
-    <t>Đã nạp lại schema.sql rồi seed.sql; đã đăng nhập phucvu01. ban-01 (B01) đang TRONG; bếp (KDS) được giả lập không phản hồi quá 5 giây.</t>
-  </si>
-  <si>
-    <t>banId = ban-01 (B01); mon-02 (Cà phê sữa) soLuong = 1; KDS_TIMEOUT_MS = 5000</t>
-  </si>
-  <si>
-    <t>Sau khoảng 5 giây hệ thống vẫn trả kết quả: HTTP 201, isSynced=false.
-Đơn vẫn được lưu; bàn chuyển DANG_PHUC_VU. Giao diện không bị treo.</t>
-  </si>
-  <si>
-    <t>Cách giả lập bếp [X06]; giả định HTTP 201 khi isSynced=false. Đơn tạo ra ở đây dùng làm dh-004 cho TC-10-09.</t>
-  </si>
-  <si>
     <t>TC-01-11</t>
   </si>
   <si>
@@ -1607,6 +1582,12 @@
   </si>
   <si>
     <t>KQ-test\TC-01-08.png</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-04-01.png</t>
   </si>
 </sst>
 </file>
@@ -2080,7 +2061,7 @@
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
   </sheetPr>
-  <dimension ref="A1:N69"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2175,13 +2156,13 @@
         <v>43</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>489</v>
+        <v>481</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>491</v>
+        <v>483</v>
       </c>
       <c r="N2" s="1"/>
     </row>
@@ -2217,13 +2198,13 @@
         <v>50</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>492</v>
+        <v>484</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M3" s="14" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>51</v>
@@ -2261,13 +2242,13 @@
         <v>59</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>494</v>
+        <v>486</v>
       </c>
       <c r="N4" s="1"/>
     </row>
@@ -2300,16 +2281,16 @@
         <v>70</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>497</v>
+        <v>489</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>71</v>
@@ -2347,13 +2328,13 @@
         <v>78</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>500</v>
+        <v>492</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M6" s="14" t="s">
-        <v>499</v>
+        <v>491</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>79</v>
@@ -2391,13 +2372,13 @@
         <v>85</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>86</v>
@@ -2435,13 +2416,13 @@
         <v>102</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M8" s="14" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>103</v>
@@ -2482,10 +2463,10 @@
         <v>125</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="N9" s="1"/>
     </row>
@@ -2524,10 +2505,10 @@
         <v>131</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>506</v>
+        <v>498</v>
       </c>
       <c r="N10" s="1"/>
     </row>
@@ -2566,10 +2547,10 @@
         <v>136</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M11" s="14" t="s">
-        <v>507</v>
+        <v>499</v>
       </c>
       <c r="N11" s="1"/>
     </row>
@@ -2605,10 +2586,10 @@
         <v>142</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>508</v>
+        <v>500</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
@@ -2645,10 +2626,10 @@
         <v>147</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>508</v>
+        <v>500</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
@@ -2685,10 +2666,10 @@
         <v>153</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>509</v>
+        <v>501</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
@@ -2725,13 +2706,13 @@
         <v>160</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M15" s="14" t="s">
-        <v>511</v>
+        <v>503</v>
       </c>
       <c r="N15" s="1" t="s">
         <v>161</v>
@@ -2769,65 +2750,67 @@
         <v>167</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>512</v>
+        <v>504</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="M16" s="14" t="s">
-        <v>513</v>
+        <v>505</v>
       </c>
       <c r="N16" s="1"/>
     </row>
-    <row r="17" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>178</v>
+        <v>38</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="K17" s="1"/>
+        <v>187</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>187</v>
+      </c>
       <c r="L17" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+        <v>506</v>
+      </c>
+      <c r="M17" s="14" t="s">
+        <v>507</v>
+      </c>
+      <c r="N17" s="1"/>
+    </row>
+    <row r="18" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>37</v>
@@ -2836,19 +2819,19 @@
         <v>38</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="J18" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="K18" s="1"/>
       <c r="L18" s="6" t="s">
@@ -2859,13 +2842,13 @@
     </row>
     <row r="19" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>37</v>
@@ -2874,19 +2857,19 @@
         <v>38</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="K19" s="1"/>
       <c r="L19" s="6" t="s">
@@ -2897,34 +2880,34 @@
     </row>
     <row r="20" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>38</v>
+        <v>128</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" s="6" t="s">
@@ -2935,34 +2918,34 @@
     </row>
     <row r="21" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>74</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="6" t="s">
@@ -2973,34 +2956,34 @@
     </row>
     <row r="22" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="6" t="s">
@@ -3011,34 +2994,34 @@
     </row>
     <row r="23" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="K23" s="1"/>
       <c r="L23" s="6" t="s">
@@ -3047,74 +3030,76 @@
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>150</v>
+        <v>219</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>199</v>
+        <v>221</v>
       </c>
       <c r="I24" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="J24" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>224</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-    </row>
-    <row r="25" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+      <c r="N24" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>225</v>
+        <v>253</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>226</v>
+        <v>254</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>227</v>
+        <v>38</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>228</v>
+        <v>255</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>229</v>
+        <v>256</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>230</v>
+        <v>257</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>231</v>
+        <v>258</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="6" t="s">
@@ -3122,24 +3107,24 @@
       </c>
       <c r="M25" s="1"/>
       <c r="N25" s="1" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>262</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>263</v>
@@ -3148,13 +3133,13 @@
         <v>40</v>
       </c>
       <c r="H26" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="I26" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>266</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" s="6" t="s">
@@ -3162,117 +3147,117 @@
       </c>
       <c r="M26" s="1"/>
       <c r="N26" s="1" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>74</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M27" s="1"/>
-      <c r="N27" s="1" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="N27" s="1"/>
+    </row>
+    <row r="28" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>274</v>
+        <v>285</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>277</v>
+        <v>288</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M28" s="1"/>
-      <c r="N28" s="1"/>
+      <c r="N28" s="1" t="s">
+        <v>291</v>
+      </c>
     </row>
     <row r="29" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>295</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>296</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="I29" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="J29" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>298</v>
       </c>
       <c r="K29" s="1"/>
       <c r="L29" s="6" t="s">
@@ -3280,90 +3265,90 @@
       </c>
       <c r="M29" s="1"/>
       <c r="N29" s="1" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>302</v>
+        <v>242</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="G30" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>264</v>
+        <v>301</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="K30" s="1"/>
       <c r="L30" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M30" s="1"/>
-      <c r="N30" s="1" t="s">
-        <v>267</v>
-      </c>
+      <c r="N30" s="1"/>
     </row>
     <row r="31" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>306</v>
+        <v>21</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>250</v>
+        <v>305</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H31" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J31" s="1" t="s">
         <v>309</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>311</v>
       </c>
       <c r="K31" s="1"/>
       <c r="L31" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-    </row>
-    <row r="32" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="N31" s="1" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>21</v>
+        <v>311</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>9</v>
@@ -3401,76 +3386,74 @@
         <v>318</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="K33" s="1"/>
       <c r="L33" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M33" s="1"/>
-      <c r="N33" s="1" t="s">
-        <v>326</v>
-      </c>
+      <c r="N33" s="1"/>
     </row>
     <row r="34" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>37</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="G34" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>339</v>
+        <v>348</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="K34" s="1"/>
       <c r="L34" s="6" t="s">
@@ -3479,36 +3462,36 @@
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H35" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="J35" s="1" t="s">
         <v>356</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>346</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>357</v>
       </c>
       <c r="K35" s="1"/>
       <c r="L35" s="6" t="s">
@@ -3517,36 +3500,36 @@
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C36" s="1" t="s">
+      <c r="D36" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="F36" s="1" t="s">
         <v>359</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>360</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>361</v>
       </c>
       <c r="G36" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>363</v>
+        <v>338</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="K36" s="1"/>
       <c r="L36" s="6" t="s">
@@ -3557,34 +3540,34 @@
     </row>
     <row r="37" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>37</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="K37" s="1"/>
       <c r="L37" s="6" t="s">
@@ -3595,34 +3578,34 @@
     </row>
     <row r="38" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="K38" s="1"/>
       <c r="L38" s="6" t="s">
@@ -3631,270 +3614,270 @@
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
     </row>
-    <row r="39" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="K39" s="1"/>
       <c r="L39" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M39" s="1"/>
-      <c r="N39" s="1"/>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N39" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>376</v>
+        <v>387</v>
       </c>
       <c r="G40" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>381</v>
+        <v>331</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>346</v>
+        <v>388</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="K40" s="1"/>
       <c r="L40" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M40" s="1"/>
-      <c r="N40" s="1" t="s">
-        <v>383</v>
-      </c>
+      <c r="N40" s="1"/>
     </row>
     <row r="41" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>337</v>
+        <v>392</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="G41" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="K41" s="1"/>
       <c r="L41" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M41" s="1"/>
-      <c r="N41" s="1"/>
+      <c r="N41" s="1" t="s">
+        <v>395</v>
+      </c>
     </row>
     <row r="42" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K42" s="1"/>
       <c r="L42" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M42" s="1"/>
-      <c r="N42" s="1" t="s">
-        <v>403</v>
-      </c>
+      <c r="N42" s="1"/>
     </row>
     <row r="43" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>400</v>
+        <v>329</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>339</v>
+        <v>409</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="K43" s="1"/>
       <c r="L43" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M43" s="1"/>
-      <c r="N43" s="1"/>
+      <c r="N43" s="1" t="s">
+        <v>412</v>
+      </c>
     </row>
     <row r="44" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C44" s="1" t="s">
+      <c r="D44" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>415</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>416</v>
       </c>
       <c r="G44" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H44" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="I44" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="I44" s="1" t="s">
+      <c r="J44" s="1" t="s">
         <v>418</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>419</v>
       </c>
       <c r="K44" s="1"/>
       <c r="L44" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M44" s="1"/>
-      <c r="N44" s="1" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="N44" s="1"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>337</v>
+        <v>403</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="G45" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H45" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="J45" s="1" t="s">
         <v>424</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>425</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>426</v>
       </c>
       <c r="K45" s="1"/>
       <c r="L45" s="6" t="s">
@@ -3903,36 +3886,36 @@
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>411</v>
+        <v>329</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="G46" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="6" t="s">
@@ -3943,34 +3926,34 @@
     </row>
     <row r="47" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>433</v>
+        <v>442</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>434</v>
+        <v>443</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>429</v>
+        <v>415</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>435</v>
+        <v>444</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>436</v>
+        <v>338</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="K47" s="1"/>
       <c r="L47" s="6" t="s">
@@ -3979,74 +3962,76 @@
       <c r="M47" s="1"/>
       <c r="N47" s="1"/>
     </row>
-    <row r="48" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>450</v>
+        <v>87</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>451</v>
+        <v>88</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>337</v>
+        <v>89</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>423</v>
+        <v>90</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>452</v>
+        <v>92</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>346</v>
+        <v>93</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>453</v>
+        <v>94</v>
       </c>
       <c r="K48" s="1"/>
       <c r="L48" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M48" s="1"/>
-      <c r="N48" s="1"/>
+      <c r="N48" s="1" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="49" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="G49" s="6" t="s">
         <v>91</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="K49" s="1"/>
       <c r="L49" s="6" t="s">
@@ -4054,79 +4039,77 @@
       </c>
       <c r="M49" s="1"/>
       <c r="N49" s="1" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>104</v>
+        <v>176</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>105</v>
+        <v>177</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>107</v>
+        <v>179</v>
       </c>
       <c r="G50" s="6" t="s">
         <v>91</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>109</v>
+        <v>180</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>110</v>
+        <v>181</v>
       </c>
       <c r="K50" s="1"/>
       <c r="L50" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M50" s="1"/>
-      <c r="N50" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="N50" s="1"/>
+    </row>
+    <row r="51" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>184</v>
+        <v>334</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>185</v>
+        <v>335</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>186</v>
+        <v>329</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>187</v>
+        <v>336</v>
       </c>
       <c r="G51" s="6" t="s">
         <v>91</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>123</v>
+        <v>337</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>188</v>
+        <v>338</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>189</v>
+        <v>339</v>
       </c>
       <c r="K51" s="1"/>
       <c r="L51" s="6" t="s">
@@ -4137,34 +4120,34 @@
     </row>
     <row r="52" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>342</v>
+        <v>436</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>343</v>
+        <v>437</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>337</v>
+        <v>392</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>344</v>
+        <v>438</v>
       </c>
       <c r="G52" s="6" t="s">
         <v>91</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>345</v>
+        <v>439</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>346</v>
+        <v>440</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>347</v>
+        <v>441</v>
       </c>
       <c r="K52" s="1"/>
       <c r="L52" s="6" t="s">
@@ -4173,36 +4156,36 @@
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
     </row>
-    <row r="53" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>444</v>
+        <v>60</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>445</v>
+        <v>61</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>400</v>
+        <v>62</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>446</v>
+        <v>56</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>447</v>
+        <v>48</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>448</v>
+        <v>64</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>449</v>
+        <v>65</v>
       </c>
       <c r="K53" s="1"/>
       <c r="L53" s="6" t="s">
@@ -4213,72 +4196,74 @@
     </row>
     <row r="54" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>60</v>
+        <v>112</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>61</v>
+        <v>113</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>62</v>
+        <v>114</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>56</v>
+        <v>115</v>
       </c>
       <c r="G54" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>48</v>
+        <v>116</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="K54" s="1"/>
       <c r="L54" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M54" s="1"/>
-      <c r="N54" s="1"/>
-    </row>
-    <row r="55" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="N54" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>112</v>
+        <v>168</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>113</v>
+        <v>169</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>114</v>
+        <v>170</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>115</v>
+        <v>171</v>
       </c>
       <c r="G55" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>116</v>
+        <v>172</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>117</v>
+        <v>173</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>118</v>
+        <v>174</v>
       </c>
       <c r="K55" s="1"/>
       <c r="L55" s="6" t="s">
@@ -4286,79 +4271,77 @@
       </c>
       <c r="M55" s="1"/>
       <c r="N55" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>168</v>
+        <v>225</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>169</v>
+        <v>226</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>170</v>
+        <v>219</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="G56" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>172</v>
+        <v>221</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>173</v>
+        <v>227</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>174</v>
+        <v>228</v>
       </c>
       <c r="K56" s="1"/>
       <c r="L56" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M56" s="1"/>
-      <c r="N56" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="57" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+      <c r="N56" s="1"/>
+    </row>
+    <row r="57" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="G57" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K57" s="1"/>
       <c r="L57" s="6" t="s">
@@ -4367,36 +4350,36 @@
       <c r="M57" s="1"/>
       <c r="N57" s="1"/>
     </row>
-    <row r="58" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>227</v>
+        <v>156</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>209</v>
+        <v>236</v>
       </c>
       <c r="G58" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H58" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="J58" s="1" t="s">
         <v>239</v>
-      </c>
-      <c r="I58" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="J58" s="1" t="s">
-        <v>241</v>
       </c>
       <c r="K58" s="1"/>
       <c r="L58" s="6" t="s">
@@ -4405,36 +4388,36 @@
       <c r="M58" s="1"/>
       <c r="N58" s="1"/>
     </row>
-    <row r="59" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>156</v>
+        <v>242</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G59" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H59" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="I59" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="I59" s="1" t="s">
+      <c r="J59" s="1" t="s">
         <v>246</v>
-      </c>
-      <c r="J59" s="1" t="s">
-        <v>247</v>
       </c>
       <c r="K59" s="1"/>
       <c r="L59" s="6" t="s">
@@ -4443,36 +4426,36 @@
       <c r="M59" s="1"/>
       <c r="N59" s="1"/>
     </row>
-    <row r="60" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C60" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E60" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="D60" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E60" s="1" t="s">
+      <c r="F60" s="1" t="s">
         <v>250</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>251</v>
       </c>
       <c r="G60" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H60" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="J60" s="1" t="s">
         <v>252</v>
-      </c>
-      <c r="I60" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>254</v>
       </c>
       <c r="K60" s="1"/>
       <c r="L60" s="6" t="s">
@@ -4481,192 +4464,192 @@
       <c r="M60" s="1"/>
       <c r="N60" s="1"/>
     </row>
-    <row r="61" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>255</v>
+        <v>272</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>257</v>
+        <v>274</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>258</v>
+        <v>275</v>
       </c>
       <c r="G61" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>199</v>
+        <v>256</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>259</v>
+        <v>276</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>260</v>
+        <v>277</v>
       </c>
       <c r="K61" s="1"/>
       <c r="L61" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M61" s="1"/>
-      <c r="N61" s="1"/>
+      <c r="N61" s="1" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="62" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E62" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>283</v>
       </c>
       <c r="G62" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="I62" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="J62" s="1" t="s">
         <v>284</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>285</v>
       </c>
       <c r="K62" s="1"/>
       <c r="L62" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M62" s="1"/>
-      <c r="N62" s="1" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="63" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="N62" s="1"/>
+    </row>
+    <row r="63" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>288</v>
+        <v>320</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>54</v>
+        <v>321</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>289</v>
+        <v>322</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="G63" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>291</v>
+        <v>324</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>292</v>
+        <v>325</v>
       </c>
       <c r="K63" s="1"/>
       <c r="L63" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M63" s="1"/>
-      <c r="N63" s="1"/>
-    </row>
-    <row r="64" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="N63" s="1" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>328</v>
+        <v>341</v>
       </c>
       <c r="D64" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="F64" s="1" t="s">
         <v>330</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>331</v>
       </c>
       <c r="G64" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>264</v>
+        <v>342</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>333</v>
+        <v>344</v>
       </c>
       <c r="K64" s="1"/>
       <c r="L64" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M64" s="1"/>
-      <c r="N64" s="1" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="65" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="N64" s="1"/>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>348</v>
+        <v>376</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>349</v>
+        <v>377</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>338</v>
+        <v>368</v>
       </c>
       <c r="G65" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>350</v>
+        <v>378</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>352</v>
+        <v>379</v>
       </c>
       <c r="K65" s="1"/>
       <c r="L65" s="6" t="s">
@@ -4675,36 +4658,36 @@
       <c r="M65" s="1"/>
       <c r="N65" s="1"/>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="G66" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="K66" s="1"/>
       <c r="L66" s="6" t="s">
@@ -4715,34 +4698,34 @@
     </row>
     <row r="67" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>388</v>
+        <v>401</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>389</v>
+        <v>402</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>337</v>
+        <v>403</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="G67" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>391</v>
+        <v>331</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>346</v>
+        <v>404</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>392</v>
+        <v>405</v>
       </c>
       <c r="K67" s="1"/>
       <c r="L67" s="6" t="s">
@@ -4753,34 +4736,34 @@
     </row>
     <row r="68" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>409</v>
+        <v>430</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>410</v>
+        <v>431</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>411</v>
+        <v>329</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>406</v>
+        <v>432</v>
       </c>
       <c r="G68" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>339</v>
+        <v>433</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>412</v>
+        <v>434</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>413</v>
+        <v>435</v>
       </c>
       <c r="K68" s="1"/>
       <c r="L68" s="6" t="s">
@@ -4789,51 +4772,13 @@
       <c r="M68" s="1"/>
       <c r="N68" s="1"/>
     </row>
-    <row r="69" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A69" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="B69" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E69" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="F69" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="G69" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H69" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="I69" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="J69" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="K69" s="1"/>
-      <c r="L69" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M69" s="1"/>
-      <c r="N69" s="1"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N69" xr:uid="{00000000-0009-0000-0000-000003000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N69">
-      <sortCondition ref="G1:G69"/>
+  <autoFilter ref="A1:N68" xr:uid="{00000000-0009-0000-0000-000003000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N68">
+      <sortCondition ref="G1:G68"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="L2:L399">
+  <conditionalFormatting sqref="L2:L398">
     <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"PASS"</formula>
     </cfRule>
@@ -4845,15 +4790,15 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="D2:D399" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D398" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Happy path,Negative,Boundary,Alternative flow,Phi chức năng"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G399" xr:uid="{00000000-0002-0000-0300-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G398" xr:uid="{00000000-0002-0000-0300-000001000000}">
       <formula1>"Cao,Trung,Thấp"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L2:L399" xr:uid="{00000000-0002-0000-0300-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="L2:L398" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>"Chưa chạy,PASS,FAIL"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4871,6 +4816,7 @@
     <hyperlink ref="M11" r:id="rId10" xr:uid="{052C7473-5CF6-451A-BECC-1E425E96FDD2}"/>
     <hyperlink ref="M15" r:id="rId11" xr:uid="{0DC140F7-DC54-47D0-8FE4-B05287842DF7}"/>
     <hyperlink ref="M16" r:id="rId12" xr:uid="{4D3489F9-5D17-474D-9677-E57F0217832E}"/>
+    <hyperlink ref="M17" r:id="rId13" xr:uid="{3C114A65-7E2A-4CB9-BDE4-077F5E538DB2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4897,34 +4843,34 @@
   <sheetData>
     <row r="1" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>454</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="J1" s="8" t="s">
         <v>455</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>456</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>457</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>458</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>459</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>460</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>461</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>462</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -5009,7 +4955,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5020,28 +4966,28 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>468</v>
+        <v>460</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>44</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>471</v>
+        <v>463</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -5095,7 +5041,7 @@
       </c>
       <c r="D5" s="6">
         <f>COUNTIF('Test Case'!$B:$B,$A5)</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E5" s="6">
         <f t="shared" si="0"/>
@@ -5111,7 +5057,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" si="2"/>
@@ -5138,11 +5084,11 @@
       </c>
       <c r="E6" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A6,'Test Case'!$L:$L,"PASS")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A6,'Test Case'!$L:$L,"FAIL")</f>
@@ -5150,11 +5096,11 @@
       </c>
       <c r="H6" s="6">
         <f t="shared" si="1"/>
-        <v>13</v>
-      </c>
-      <c r="I6" s="9" t="str">
+        <v>12</v>
+      </c>
+      <c r="I6" s="9">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>1</v>
       </c>
       <c r="J6" s="6">
         <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A6,2)&amp;"-*")</f>
@@ -5358,23 +5304,23 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>473</v>
+        <v>465</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="10">
         <f>SUM(D4:D11)</f>
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E12" s="10">
         <f>SUM(E4:E11)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F12" s="10">
         <f>SUM(F4:F11)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G12" s="10">
         <f>SUM(G4:G11)</f>
@@ -5382,7 +5328,7 @@
       </c>
       <c r="H12" s="10">
         <f>SUM(H4:H11)</f>
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" si="2"/>
@@ -5395,7 +5341,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>475</v>
+        <v>467</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5405,13 +5351,13 @@
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -5426,7 +5372,7 @@
       </c>
       <c r="E16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"PASS")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"FAIL")</f>
@@ -5479,7 +5425,7 @@
       <c r="C19" s="1"/>
       <c r="D19" s="6">
         <f>COUNTIF('Test Case'!$D:$D,$A19)</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"PASS")</f>
@@ -5492,7 +5438,7 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -5511,28 +5457,28 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>476</v>
+        <v>468</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>477</v>
+        <v>469</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>478</v>
+        <v>470</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>479</v>
+        <v>471</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>480</v>
+        <v>472</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -5551,7 +5497,7 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -5570,7 +5516,7 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>481</v>
+        <v>473</v>
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -5589,7 +5535,7 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>482</v>
+        <v>474</v>
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -5608,16 +5554,16 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>483</v>
+        <v>475</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
       <c r="B31" s="15" t="str">
         <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
-        <v>Đã chạy 15 / 68 TC; PASS 15; FAIL 0; tỉ lệ pass 100.0%</v>
+        <v>Đã chạy 16 / 67 TC; PASS 16; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>
@@ -5630,7 +5576,7 @@
     </row>
     <row r="32" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>485</v>
+        <v>477</v>
       </c>
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
@@ -5644,7 +5590,7 @@
     </row>
     <row r="33" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>486</v>
+        <v>478</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
@@ -5658,7 +5604,7 @@
     </row>
     <row r="34" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>487</v>
+        <v>479</v>
       </c>
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
@@ -5672,7 +5618,7 @@
     </row>
     <row r="35" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>488</v>
+        <v>480</v>
       </c>
       <c r="B35" s="16"/>
       <c r="C35" s="16"/>

</xml_diff>

<commit_message>
Hoàn thành kiểm thử các test case của UC1, UC4, UC 10, UC21
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A35D55-0AF0-4FC9-9B3C-F1807116C953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648A381E-8F35-4D57-8F56-BCEEEE8A6FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Tổng hợp" sheetId="6" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Case'!$A$1:$N$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Case'!$A$1:$N$65</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="518">
   <si>
     <t>UC</t>
   </si>
@@ -584,9 +584,6 @@
     <t>Đề xuất của Tuấn trong contract, chưa chốt [X01]. Nếu chốt khác thì sửa Expected.</t>
   </si>
   <si>
-    <t>TC-01-11</t>
-  </si>
-  <si>
     <t>Gửi order khi giỏ hàng rỗng</t>
   </si>
   <si>
@@ -798,24 +795,6 @@
   </si>
   <si>
     <t>Cả ba: HTTP 409, maLoi=DON_DA_THANH_TOAN. Đơn không thay đổi.</t>
-  </si>
-  <si>
-    <t>TC-04-13</t>
-  </si>
-  <si>
-    <t>Sửa món với chiTietId không tồn tại</t>
-  </si>
-  <si>
-    <t>EP (invalid class: id không tồn tại)</t>
-  </si>
-  <si>
-    <t>CD_CapNhat (themMon/suaMon/huyMon); api-contract §3 UC04; mã lỗi MON_TRONG_DON_KHONG_TON_TAI</t>
-  </si>
-  <si>
-    <t>chiTietId = "ct-khongco"</t>
-  </si>
-  <si>
-    <t>HTTP 404, maLoi=MON_TRONG_DON_KHONG_TON_TAI. Đơn không thay đổi.</t>
   </si>
   <si>
     <t>TC-10-01</t>
@@ -853,9 +832,6 @@
     <t>SD_ThanhToan; api-contract §3 UC10 (POST /payments); BPC T6 (tinhTienThoi)</t>
   </si>
   <si>
-    <t>phuongThuc = TIEN_MAT; tienKhachDua = 100.000; maGiaoDich mới</t>
-  </si>
-  <si>
     <t>HTTP 200; thanhCong=true; tienThoi=0; trangThaiDon=DA_THANH_TOAN; trangThaiBan=CAN_DON.</t>
   </si>
   <si>
@@ -941,26 +917,6 @@
     <t>TC-10-07</t>
   </si>
   <si>
-    <t>Bấm xác nhận 2 lần với cùng mã giao dịch</t>
-  </si>
-  <si>
-    <t>Black-box theo UC Spec (EF: thanh toán trùng)</t>
-  </si>
-  <si>
-    <t>SD_ThanhToan; api-contract §3 UC10 (POST /payments); BPC T6 (findByMaGiaoDich), mục 2 (chặn thanh toán trùng mã)</t>
-  </si>
-  <si>
-    <t>maGiaoDich = "gd-test-0001"; phuongThuc = TIEN_MAT; tienKhachDua = 100.000</t>
-  </si>
-  <si>
-    <t>Lần 1: HTTP 200, daXuLyTruoc=false.
-Lần 2: HTTP 200, daXuLyTruoc=true, kết quả giống lần 1; không thu tiền lần hai.
-CSDL chỉ có 1 bản ghi thanh_toan với maGiaoDich = gd-test-0001.</t>
-  </si>
-  <si>
-    <t>TC-10-08</t>
-  </si>
-  <si>
     <t>Thanh toán đơn đã thanh toán (mã giao dịch khác)</t>
   </si>
   <si>
@@ -974,30 +930,6 @@
   </si>
   <si>
     <t>HTTP 409, maLoi=DON_DA_THANH_TOAN. Không thêm bản ghi thanh_toan; đơn và bàn giữ nguyên.</t>
-  </si>
-  <si>
-    <t>Thanh toán đơn chưa gửi bếp</t>
-  </si>
-  <si>
-    <t>Black-box theo UC Spec (EF: đơn chưa gửi bếp)</t>
-  </si>
-  <si>
-    <t>SD_ThanhToan; api-contract §3 UC10 (POST /payments); mã lỗi DON_CHUA_GUI_BEP</t>
-  </si>
-  <si>
-    <t>Đã đăng nhập thungan01; dh-004 là đơn có isSynced=false (chạy SQL: UPDATE don_hang SET is_synced = FALSE WHERE id = 'dh-004';).</t>
-  </si>
-  <si>
-    <t>donHangId = dh-004; phuongThuc = TIEN_MAT; tienKhachDua đủ; maGiaoDich mới</t>
-  </si>
-  <si>
-    <t>HTTP 409, maLoi=DON_CHUA_GUI_BEP. Không ghi dữ liệu; đơn dh-004 vẫn DANG_PHUC_VU; trạng thái bàn ban-06 giữ nguyên (seed đang để CAN_DON).</t>
-  </si>
-  <si>
-    <t>Có thể tạo đơn chưa đồng bộ từ TC-01-10 [X06]. Lưu ý seed: dh-004 có tong_tien 70.000 gồm cả món DA_HUY 30.000 [X16].</t>
-  </si>
-  <si>
-    <t>TC-10-10</t>
   </si>
   <si>
     <t>Lỗi giữa chừng: rollback cả 3 thao tác ghi</t>
@@ -1022,9 +954,6 @@
     <t>Cách ép lỗi [X07]. Nạp lại schema.sql + seed.sql trước TC này (đơn dh-002 chỉ thanh toán được một lần).</t>
   </si>
   <si>
-    <t>TC-10-11</t>
-  </si>
-  <si>
     <t>Nút "Xác nhận" bị khóa khi đang xử lý (chống bấm 2 lần)</t>
   </si>
   <si>
@@ -1588,6 +1517,105 @@
   </si>
   <si>
     <t>KQ-test\TC-04-01.png</t>
+  </si>
+  <si>
+    <t>HTTP 200. soLuong=3; tongTien = 85.000 + 4×40.000 = 245000; món vẫn CHO_PHA_CHE.</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-04-02.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-04-03.png</t>
+  </si>
+  <si>
+    <t>Hệ thống không cho chỉnh số lượng về 0</t>
+  </si>
+  <si>
+    <t>Hệ thống không cho chỉnh số lượng về 100</t>
+  </si>
+  <si>
+    <t>hệ thống không hiện nút hủy với món đang làm</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-10-01.png</t>
+  </si>
+  <si>
+    <t>phuongThuc = TIEN_MAT; tienKhachDua = 85.000; maGiaoDich mới</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập thungan01; đơn dh-001 (ban-03/B03, HOAN_THANH, tổng 85.000, mọi món DA_XONG) chưa thanh toán (vừa nạp lại DB).</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-10-02.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-10-03.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-10-06.png</t>
+  </si>
+  <si>
+    <t>đơn đã thanh toán thì hệ thống sẽ không hiện nữa</t>
+  </si>
+  <si>
+    <t>Khi bàn đang phục vụ thì màn hình tạo hóa đơn chỉ có gọi thêm chứ không còn tạo thêm đơn nữa</t>
+  </si>
+  <si>
+    <t>Hệ thống báo lỗi chưa chọn món nào</t>
+  </si>
+  <si>
+    <t>TC-01-10</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-01-10.png</t>
+  </si>
+  <si>
+    <t>TC-10-8</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-10-07.png</t>
+  </si>
+  <si>
+    <t>Màn hình không cho phép thay đổi số lượng khi món đang làm</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-04-09.png</t>
+  </si>
+  <si>
+    <t>Màn hình không cho phép thay đổi số lượng khi món đã xong</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-04-10.png</t>
+  </si>
+  <si>
+    <t>Giao diện: món hiện xám, không chọn được.</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-04-11.png</t>
+  </si>
+  <si>
+    <t>Khi bàn đã thanh toán thì tự động chuyển sang cần dọn không cho phép thêm sửa xóa</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-04-12.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-21-04.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-21-08.png</t>
+  </si>
+  <si>
+    <t>HTTP 401 Unauthorized, success=false, maLoi="CHUA_DANG_NHAP", message="Vui lòng đăng nhập". Server chặn thành công truy cập trái phép khi thiếu token Authorization</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-21-10.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-21-11.png</t>
+  </si>
+  <si>
+    <t>HTTP 403 Forbidden, success=false, maLoi="KHONG_CO_QUYEN", message="Bạn không có quyền thực hiện thao tác này". Hệ thống phân quyền chặt chẽ, chặn thành công khi tài khoản Phuc vu gọi API thanh toán của Thu ngan. Dữ liệu đơn hàng giữ nguyên</t>
   </si>
 </sst>
 </file>
@@ -2061,7 +2089,7 @@
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
   </sheetPr>
-  <dimension ref="A1:N68"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2126,13 +2154,13 @@
     </row>
     <row r="2" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>36</v>
+        <v>121</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>37</v>
@@ -2141,1045 +2169,1045 @@
         <v>38</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>39</v>
+        <v>122</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>41</v>
+        <v>123</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>42</v>
+        <v>124</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>43</v>
+        <v>125</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>481</v>
+        <v>125</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>482</v>
+        <v>459</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>483</v>
+        <v>474</v>
       </c>
       <c r="N2" s="1"/>
     </row>
     <row r="3" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>45</v>
+        <v>126</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>46</v>
+        <v>127</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>38</v>
+        <v>128</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>47</v>
+        <v>129</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>48</v>
+        <v>123</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>49</v>
+        <v>130</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>50</v>
+        <v>131</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>484</v>
+        <v>131</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>482</v>
+        <v>459</v>
       </c>
       <c r="M3" s="14" t="s">
-        <v>485</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>51</v>
-      </c>
+        <v>475</v>
+      </c>
+      <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>52</v>
+        <v>132</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>53</v>
+        <v>133</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>55</v>
+        <v>134</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>56</v>
+        <v>129</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>57</v>
+        <v>123</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>58</v>
+        <v>135</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>59</v>
+        <v>136</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>487</v>
+        <v>136</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>482</v>
+        <v>459</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>486</v>
+        <v>476</v>
       </c>
       <c r="N4" s="1"/>
     </row>
     <row r="5" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>66</v>
+        <v>137</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>67</v>
+        <v>138</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>68</v>
+        <v>139</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>69</v>
+        <v>140</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>48</v>
+        <v>123</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>70</v>
+        <v>141</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>488</v>
+        <v>142</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>490</v>
+        <v>477</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="M5" s="14" t="s">
-        <v>489</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>71</v>
-      </c>
+        <v>459</v>
+      </c>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
     </row>
     <row r="6" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>72</v>
+        <v>143</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>73</v>
+        <v>144</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>75</v>
+        <v>145</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>76</v>
+        <v>140</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>57</v>
+        <v>123</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>77</v>
+        <v>146</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>78</v>
+        <v>147</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>492</v>
+        <v>477</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="M6" s="14" t="s">
-        <v>491</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>79</v>
-      </c>
+        <v>459</v>
+      </c>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
     </row>
     <row r="7" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>80</v>
+        <v>148</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>81</v>
+        <v>149</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>74</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>82</v>
+        <v>150</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>83</v>
+        <v>151</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>57</v>
+        <v>123</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>84</v>
+        <v>152</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>85</v>
+        <v>153</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>493</v>
+        <v>478</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="M7" s="14" t="s">
-        <v>494</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>86</v>
-      </c>
+        <v>459</v>
+      </c>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
     </row>
     <row r="8" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>96</v>
+        <v>154</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>97</v>
+        <v>155</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>98</v>
+        <v>156</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>99</v>
+        <v>157</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>100</v>
+        <v>158</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>101</v>
+        <v>159</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>102</v>
+        <v>160</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>495</v>
+        <v>479</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>482</v>
+        <v>459</v>
       </c>
       <c r="M8" s="14" t="s">
-        <v>496</v>
+        <v>480</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>103</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>120</v>
+        <v>162</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>121</v>
+        <v>163</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>38</v>
+        <v>164</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>123</v>
+        <v>165</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>124</v>
+        <v>166</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>125</v>
+        <v>167</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>125</v>
+        <v>481</v>
       </c>
       <c r="L9" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="M9" s="14" t="s">
         <v>482</v>
       </c>
-      <c r="M9" s="14" t="s">
-        <v>497</v>
-      </c>
       <c r="N9" s="1"/>
     </row>
-    <row r="10" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>126</v>
+        <v>168</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>127</v>
+        <v>169</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>128</v>
+        <v>170</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>129</v>
+        <v>171</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>123</v>
+        <v>172</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>130</v>
+        <v>173</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>131</v>
+        <v>174</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>131</v>
+        <v>498</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="M10" s="14" t="s">
-        <v>498</v>
-      </c>
-      <c r="N10" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="11" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>132</v>
+        <v>500</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>133</v>
+        <v>176</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>134</v>
+        <v>177</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>129</v>
+        <v>178</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>135</v>
+        <v>179</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>136</v>
+        <v>180</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>136</v>
+        <v>499</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>482</v>
+        <v>459</v>
       </c>
       <c r="M11" s="14" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="N11" s="1"/>
     </row>
     <row r="12" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>137</v>
+        <v>181</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>138</v>
+        <v>182</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>139</v>
+        <v>38</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>123</v>
+        <v>184</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>141</v>
+        <v>185</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>142</v>
+        <v>186</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>500</v>
+        <v>186</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="M12" s="1"/>
+        <v>483</v>
+      </c>
+      <c r="M12" s="14" t="s">
+        <v>484</v>
+      </c>
       <c r="N12" s="1"/>
     </row>
     <row r="13" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>143</v>
+        <v>187</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>144</v>
+        <v>188</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>145</v>
+        <v>38</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>140</v>
+        <v>189</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>123</v>
+        <v>190</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>146</v>
+        <v>191</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>147</v>
+        <v>192</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>500</v>
+        <v>485</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="M13" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M13" s="14" t="s">
+        <v>486</v>
+      </c>
       <c r="N13" s="1"/>
     </row>
     <row r="14" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>148</v>
+        <v>193</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>149</v>
+        <v>194</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>150</v>
+        <v>38</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>151</v>
+        <v>195</v>
       </c>
       <c r="G14" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>123</v>
+        <v>190</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>152</v>
+        <v>196</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>153</v>
+        <v>197</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>501</v>
+        <v>197</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="M14" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M14" s="14" t="s">
+        <v>487</v>
+      </c>
       <c r="N14" s="1"/>
     </row>
     <row r="15" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>154</v>
+        <v>198</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>155</v>
+        <v>199</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>156</v>
+        <v>128</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>157</v>
+        <v>200</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>158</v>
+        <v>190</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>159</v>
+        <v>201</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>160</v>
+        <v>202</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>502</v>
+        <v>202</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="M15" s="14" t="s">
-        <v>503</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>161</v>
-      </c>
+        <v>459</v>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
     </row>
     <row r="16" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>162</v>
+        <v>203</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>163</v>
+        <v>204</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>164</v>
+        <v>134</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>157</v>
+        <v>200</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>165</v>
+        <v>190</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>166</v>
+        <v>205</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>167</v>
+        <v>206</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>504</v>
+        <v>206</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="M16" s="14" t="s">
-        <v>505</v>
-      </c>
+        <v>459</v>
+      </c>
+      <c r="M16" s="1"/>
       <c r="N16" s="1"/>
     </row>
     <row r="17" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>183</v>
+        <v>208</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>38</v>
+        <v>139</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>184</v>
+        <v>209</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>187</v>
+        <v>211</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>187</v>
+        <v>488</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>506</v>
-      </c>
-      <c r="M17" s="14" t="s">
-        <v>507</v>
-      </c>
+        <v>459</v>
+      </c>
+      <c r="M17" s="1"/>
       <c r="N17" s="1"/>
     </row>
     <row r="18" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>188</v>
+        <v>212</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>189</v>
+        <v>213</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>38</v>
+        <v>150</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="K18" s="1"/>
+        <v>215</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>489</v>
+      </c>
       <c r="L18" s="6" t="s">
-        <v>44</v>
+        <v>459</v>
       </c>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
     <row r="19" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>195</v>
+        <v>217</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>38</v>
+        <v>218</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>196</v>
+        <v>219</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>197</v>
+        <v>221</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="K19" s="1"/>
+        <v>222</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>490</v>
+      </c>
       <c r="L19" s="6" t="s">
-        <v>44</v>
+        <v>459</v>
       </c>
       <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-    </row>
-    <row r="20" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="N19" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="G20" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="K20" s="1"/>
+        <v>227</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>504</v>
+      </c>
       <c r="L20" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M20" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M20" s="14" t="s">
+        <v>505</v>
+      </c>
       <c r="N20" s="1"/>
     </row>
-    <row r="21" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>205</v>
+        <v>229</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>134</v>
+        <v>218</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>191</v>
+        <v>230</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>206</v>
+        <v>231</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="K21" s="1"/>
+        <v>232</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>506</v>
+      </c>
       <c r="L21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M21" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M21" s="14" t="s">
+        <v>507</v>
+      </c>
       <c r="N21" s="1"/>
     </row>
-    <row r="22" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>208</v>
+        <v>233</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>209</v>
+        <v>234</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>210</v>
+        <v>235</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>191</v>
+        <v>236</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="K22" s="1"/>
+        <v>238</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>508</v>
+      </c>
       <c r="L22" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M22" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M22" s="14" t="s">
+        <v>509</v>
+      </c>
       <c r="N22" s="1"/>
     </row>
-    <row r="23" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>213</v>
+        <v>239</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>214</v>
+        <v>240</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>150</v>
+        <v>241</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>210</v>
+        <v>242</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>191</v>
+        <v>243</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>215</v>
+        <v>244</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="K23" s="1"/>
+        <v>245</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>510</v>
+      </c>
       <c r="L23" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M23" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M23" s="14" t="s">
+        <v>511</v>
+      </c>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>217</v>
+        <v>390</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>218</v>
+        <v>391</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>219</v>
+        <v>306</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>220</v>
+        <v>392</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>221</v>
+        <v>393</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>222</v>
+        <v>394</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>223</v>
+        <v>395</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M24" s="1"/>
-      <c r="N24" s="1" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="N24" s="1"/>
+    </row>
+    <row r="25" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>253</v>
+        <v>396</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>254</v>
+        <v>397</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>38</v>
+        <v>380</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>255</v>
+        <v>398</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>256</v>
+        <v>399</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>257</v>
+        <v>400</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>258</v>
+        <v>401</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M25" s="1"/>
-      <c r="N25" s="1" t="s">
-        <v>259</v>
-      </c>
+      <c r="N25" s="1"/>
     </row>
     <row r="26" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>260</v>
+        <v>402</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>261</v>
+        <v>403</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>262</v>
+        <v>306</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>263</v>
+        <v>398</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>256</v>
+        <v>404</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>264</v>
+        <v>405</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>265</v>
+        <v>406</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M26" s="1"/>
-      <c r="N26" s="1" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="N26" s="1"/>
+    </row>
+    <row r="27" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>266</v>
+        <v>407</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>267</v>
+        <v>408</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>268</v>
+        <v>306</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>269</v>
+        <v>409</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>256</v>
+        <v>410</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>270</v>
+        <v>411</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>271</v>
+        <v>412</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="6" t="s">
@@ -3188,272 +3216,282 @@
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
     </row>
-    <row r="28" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>285</v>
+        <v>413</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>286</v>
+        <v>414</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>287</v>
+        <v>369</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>288</v>
+        <v>415</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>256</v>
+        <v>416</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>289</v>
+        <v>417</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>290</v>
+        <v>418</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M28" s="1"/>
-      <c r="N28" s="1" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="N28" s="1"/>
+    </row>
+    <row r="29" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>292</v>
+        <v>419</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>293</v>
+        <v>420</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>295</v>
+        <v>392</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>256</v>
+        <v>421</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>297</v>
+        <v>422</v>
       </c>
       <c r="K29" s="1"/>
       <c r="L29" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M29" s="1"/>
-      <c r="N29" s="1" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="N29" s="1"/>
+    </row>
+    <row r="30" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>298</v>
+        <v>246</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>299</v>
+        <v>247</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>242</v>
+        <v>38</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>300</v>
+        <v>248</v>
       </c>
       <c r="G30" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>301</v>
+        <v>249</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>302</v>
+        <v>250</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="K30" s="1"/>
+        <v>251</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>251</v>
+      </c>
       <c r="L30" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-    </row>
-    <row r="31" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+        <v>459</v>
+      </c>
+      <c r="M30" s="14" t="s">
+        <v>491</v>
+      </c>
+      <c r="N30" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>21</v>
+        <v>253</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>304</v>
+        <v>254</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>305</v>
+        <v>255</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>306</v>
+        <v>256</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>307</v>
+        <v>493</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>308</v>
+        <v>492</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>309</v>
-      </c>
-      <c r="K31" s="1"/>
+        <v>257</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>257</v>
+      </c>
       <c r="L31" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M31" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M31" s="14" t="s">
+        <v>494</v>
+      </c>
       <c r="N31" s="1" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>311</v>
+        <v>258</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>312</v>
+        <v>259</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>313</v>
+        <v>260</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>314</v>
+        <v>261</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>315</v>
+        <v>249</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>316</v>
+        <v>262</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="K32" s="1"/>
+        <v>263</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>263</v>
+      </c>
       <c r="L32" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M32" s="1"/>
-      <c r="N32" s="1" t="s">
-        <v>318</v>
-      </c>
+        <v>459</v>
+      </c>
+      <c r="M32" s="14" t="s">
+        <v>495</v>
+      </c>
+      <c r="N32" s="1"/>
     </row>
     <row r="33" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>327</v>
+        <v>264</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>328</v>
+        <v>265</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>329</v>
+        <v>266</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>330</v>
+        <v>267</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>331</v>
+        <v>249</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>332</v>
+        <v>268</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>333</v>
+        <v>269</v>
       </c>
       <c r="K33" s="1"/>
       <c r="L33" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M33" s="1"/>
-      <c r="N33" s="1"/>
+      <c r="N33" s="1" t="s">
+        <v>270</v>
+      </c>
     </row>
     <row r="34" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>345</v>
+        <v>271</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>346</v>
+        <v>272</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>329</v>
+        <v>273</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>347</v>
+        <v>274</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>348</v>
+        <v>249</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>338</v>
+        <v>275</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>349</v>
+        <v>276</v>
       </c>
       <c r="K34" s="1"/>
       <c r="L34" s="6" t="s">
@@ -3462,228 +3500,240 @@
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>350</v>
+        <v>277</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>351</v>
+        <v>278</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>352</v>
+        <v>279</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>353</v>
+        <v>280</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>354</v>
+        <v>249</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>355</v>
+        <v>281</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>356</v>
-      </c>
-      <c r="K35" s="1"/>
+        <v>282</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>282</v>
+      </c>
       <c r="L35" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M35" s="1"/>
-      <c r="N35" s="1"/>
-    </row>
-    <row r="36" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+        <v>459</v>
+      </c>
+      <c r="M35" s="14" t="s">
+        <v>496</v>
+      </c>
+      <c r="N35" s="1" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>357</v>
+        <v>284</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>358</v>
+        <v>285</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>329</v>
+        <v>241</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>359</v>
+        <v>286</v>
       </c>
       <c r="G36" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>360</v>
+        <v>287</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>338</v>
+        <v>288</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="K36" s="1"/>
+        <v>289</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>497</v>
+      </c>
       <c r="L36" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M36" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M36" s="14" t="s">
+        <v>503</v>
+      </c>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>362</v>
+        <v>502</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>363</v>
+        <v>290</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>329</v>
+        <v>291</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>359</v>
+        <v>292</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>364</v>
+        <v>293</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>338</v>
+        <v>294</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>365</v>
+        <v>295</v>
       </c>
       <c r="K37" s="1"/>
       <c r="L37" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M37" s="1"/>
-      <c r="N37" s="1"/>
-    </row>
-    <row r="38" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="N37" s="1" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>366</v>
+        <v>21</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>367</v>
+        <v>297</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>54</v>
+        <v>298</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>329</v>
+        <v>299</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>368</v>
+        <v>300</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>369</v>
+        <v>249</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>338</v>
+        <v>301</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>370</v>
+        <v>302</v>
       </c>
       <c r="K38" s="1"/>
       <c r="L38" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N38" s="1" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>371</v>
+        <v>304</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>372</v>
+        <v>305</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>329</v>
+        <v>306</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>368</v>
+        <v>307</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>373</v>
+        <v>308</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>338</v>
+        <v>309</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>374</v>
+        <v>310</v>
       </c>
       <c r="K39" s="1"/>
       <c r="L39" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M39" s="1"/>
-      <c r="N39" s="1" t="s">
-        <v>375</v>
-      </c>
+      <c r="N39" s="1"/>
     </row>
     <row r="40" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>385</v>
+        <v>311</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>386</v>
+        <v>312</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>329</v>
+        <v>306</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>387</v>
+        <v>313</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>331</v>
+        <v>314</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>388</v>
+        <v>315</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>389</v>
+        <v>316</v>
       </c>
       <c r="K40" s="1"/>
       <c r="L40" s="6" t="s">
@@ -3694,74 +3744,72 @@
     </row>
     <row r="41" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>390</v>
+        <v>317</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>391</v>
+        <v>318</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>392</v>
+        <v>306</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>387</v>
+        <v>307</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>393</v>
+        <v>320</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>394</v>
+        <v>321</v>
       </c>
       <c r="K41" s="1"/>
       <c r="L41" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M41" s="1"/>
-      <c r="N41" s="1" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="N41" s="1"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>396</v>
+        <v>322</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>397</v>
+        <v>323</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>392</v>
+        <v>306</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>398</v>
+        <v>324</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>399</v>
+        <v>315</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>400</v>
+        <v>326</v>
       </c>
       <c r="K42" s="1"/>
       <c r="L42" s="6" t="s">
@@ -3772,74 +3820,72 @@
     </row>
     <row r="43" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>406</v>
+        <v>327</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>407</v>
+        <v>328</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>329</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>408</v>
+        <v>330</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>409</v>
+        <v>331</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>410</v>
+        <v>332</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>411</v>
+        <v>333</v>
       </c>
       <c r="K43" s="1"/>
       <c r="L43" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M43" s="1"/>
-      <c r="N43" s="1" t="s">
-        <v>412</v>
-      </c>
+      <c r="N43" s="1"/>
     </row>
     <row r="44" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>413</v>
+        <v>334</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>414</v>
+        <v>335</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>37</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>329</v>
+        <v>306</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>415</v>
+        <v>336</v>
       </c>
       <c r="G44" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>416</v>
+        <v>337</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>417</v>
+        <v>315</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>418</v>
+        <v>338</v>
       </c>
       <c r="K44" s="1"/>
       <c r="L44" s="6" t="s">
@@ -3848,36 +3894,36 @@
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>419</v>
+        <v>339</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>420</v>
+        <v>340</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>403</v>
+        <v>306</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>421</v>
+        <v>336</v>
       </c>
       <c r="G45" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>422</v>
+        <v>341</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>423</v>
+        <v>315</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>424</v>
+        <v>342</v>
       </c>
       <c r="K45" s="1"/>
       <c r="L45" s="6" t="s">
@@ -3886,36 +3932,36 @@
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
     </row>
-    <row r="46" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>425</v>
+        <v>343</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>426</v>
+        <v>344</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>329</v>
+        <v>306</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>421</v>
+        <v>345</v>
       </c>
       <c r="G46" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>427</v>
+        <v>346</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>428</v>
+        <v>315</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>429</v>
+        <v>347</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="6" t="s">
@@ -3924,154 +3970,152 @@
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
     </row>
-    <row r="47" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>442</v>
+        <v>348</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>443</v>
+        <v>349</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>329</v>
+        <v>306</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>415</v>
+        <v>345</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>444</v>
+        <v>350</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>338</v>
+        <v>315</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>445</v>
+        <v>351</v>
       </c>
       <c r="K47" s="1"/>
       <c r="L47" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M47" s="1"/>
-      <c r="N47" s="1"/>
-    </row>
-    <row r="48" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="N47" s="1" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>87</v>
+        <v>353</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>88</v>
+        <v>354</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>89</v>
+        <v>306</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>90</v>
+        <v>345</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>92</v>
+        <v>355</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>93</v>
+        <v>315</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>94</v>
+        <v>356</v>
       </c>
       <c r="K48" s="1"/>
       <c r="L48" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M48" s="1"/>
-      <c r="N48" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="N48" s="1"/>
+    </row>
+    <row r="49" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>104</v>
+        <v>357</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>105</v>
+        <v>358</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>106</v>
+        <v>306</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>107</v>
+        <v>359</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>108</v>
+        <v>360</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>109</v>
+        <v>315</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>110</v>
+        <v>361</v>
       </c>
       <c r="K49" s="1"/>
       <c r="L49" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M49" s="1"/>
-      <c r="N49" s="1" t="s">
-        <v>111</v>
-      </c>
+      <c r="N49" s="1"/>
     </row>
     <row r="50" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>176</v>
+        <v>362</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>177</v>
+        <v>363</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>178</v>
+        <v>306</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>179</v>
+        <v>364</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>123</v>
+        <v>308</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>180</v>
+        <v>365</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>181</v>
+        <v>366</v>
       </c>
       <c r="K50" s="1"/>
       <c r="L50" s="6" t="s">
@@ -4080,74 +4124,76 @@
       <c r="M50" s="1"/>
       <c r="N50" s="1"/>
     </row>
-    <row r="51" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>334</v>
+        <v>367</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>335</v>
+        <v>368</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>329</v>
+        <v>369</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>336</v>
+        <v>364</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>337</v>
+        <v>308</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>338</v>
+        <v>370</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>339</v>
+        <v>371</v>
       </c>
       <c r="K51" s="1"/>
       <c r="L51" s="6" t="s">
         <v>44</v>
       </c>
       <c r="M51" s="1"/>
-      <c r="N51" s="1"/>
-    </row>
-    <row r="52" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="N51" s="1" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>436</v>
+        <v>373</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>437</v>
+        <v>374</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>392</v>
+        <v>369</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>438</v>
+        <v>375</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>439</v>
+        <v>308</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>440</v>
+        <v>376</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>441</v>
+        <v>377</v>
       </c>
       <c r="K52" s="1"/>
       <c r="L52" s="6" t="s">
@@ -4156,36 +4202,36 @@
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
     </row>
-    <row r="53" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>60</v>
+        <v>378</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>61</v>
+        <v>379</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>62</v>
+        <v>380</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>56</v>
+        <v>375</v>
       </c>
       <c r="G53" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>48</v>
+        <v>308</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>64</v>
+        <v>381</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>65</v>
+        <v>382</v>
       </c>
       <c r="K53" s="1"/>
       <c r="L53" s="6" t="s">
@@ -4194,36 +4240,36 @@
       <c r="M53" s="1"/>
       <c r="N53" s="1"/>
     </row>
-    <row r="54" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>112</v>
+        <v>383</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>113</v>
+        <v>384</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>114</v>
+        <v>306</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>115</v>
+        <v>385</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>116</v>
+        <v>386</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>117</v>
+        <v>387</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>118</v>
+        <v>388</v>
       </c>
       <c r="K54" s="1"/>
       <c r="L54" s="6" t="s">
@@ -4231,554 +4277,494 @@
       </c>
       <c r="M54" s="1"/>
       <c r="N54" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>168</v>
+        <v>35</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>169</v>
+        <v>36</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>170</v>
+        <v>38</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>171</v>
+        <v>39</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>172</v>
+        <v>41</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>173</v>
+        <v>42</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="K55" s="1"/>
+        <v>43</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>458</v>
+      </c>
       <c r="L55" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M55" s="1"/>
-      <c r="N55" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+        <v>459</v>
+      </c>
+      <c r="M55" s="14" t="s">
+        <v>460</v>
+      </c>
+      <c r="N55" s="1"/>
+    </row>
+    <row r="56" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>225</v>
+        <v>45</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>226</v>
+        <v>46</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>219</v>
+        <v>38</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>201</v>
+        <v>47</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>221</v>
+        <v>48</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>227</v>
+        <v>49</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="K56" s="1"/>
+        <v>50</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>461</v>
+      </c>
       <c r="L56" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M56" s="1"/>
-      <c r="N56" s="1"/>
-    </row>
-    <row r="57" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+        <v>459</v>
+      </c>
+      <c r="M56" s="14" t="s">
+        <v>462</v>
+      </c>
+      <c r="N56" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>229</v>
+        <v>52</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>230</v>
+        <v>53</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>219</v>
+        <v>55</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>201</v>
+        <v>56</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>231</v>
+        <v>57</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>232</v>
+        <v>58</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="K57" s="1"/>
+        <v>59</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>464</v>
+      </c>
       <c r="L57" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M57" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M57" s="14" t="s">
+        <v>463</v>
+      </c>
       <c r="N57" s="1"/>
     </row>
-    <row r="58" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>234</v>
+        <v>60</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>235</v>
+        <v>61</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>156</v>
+        <v>62</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>236</v>
+        <v>56</v>
       </c>
       <c r="G58" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>237</v>
+        <v>48</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>238</v>
+        <v>64</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="K58" s="1"/>
+        <v>65</v>
+      </c>
+      <c r="K58" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="L58" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M58" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M58" s="14" t="s">
+        <v>512</v>
+      </c>
       <c r="N58" s="1"/>
     </row>
     <row r="59" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>240</v>
+        <v>66</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>241</v>
+        <v>67</v>
       </c>
       <c r="D59" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="K59" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="L59" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="M59" s="14" t="s">
+        <v>466</v>
+      </c>
+      <c r="N59" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A60" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="K60" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="L60" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="M60" s="14" t="s">
+        <v>468</v>
+      </c>
+      <c r="N60" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I61" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="J61" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="K61" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="L61" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="M61" s="14" t="s">
+        <v>471</v>
+      </c>
+      <c r="N61" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A62" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E59" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="G59" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H59" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="I59" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="J59" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="K59" s="1"/>
-      <c r="L59" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M59" s="1"/>
-      <c r="N59" s="1"/>
-    </row>
-    <row r="60" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A60" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="D60" s="1" t="s">
+      <c r="E62" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I62" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J62" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K62" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L62" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="M62" s="14" t="s">
+        <v>513</v>
+      </c>
+      <c r="N62" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G63" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="J63" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K63" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="L63" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="M63" s="14" t="s">
+        <v>473</v>
+      </c>
+      <c r="N63" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A64" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E60" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="G60" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H60" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="I60" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="J60" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="K60" s="1"/>
-      <c r="L60" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M60" s="1"/>
-      <c r="N60" s="1"/>
-    </row>
-    <row r="61" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A61" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="G61" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H61" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="I61" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="J61" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="K61" s="1"/>
-      <c r="L61" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M61" s="1"/>
-      <c r="N61" s="1" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A62" s="5" t="s">
-        <v>279</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="G62" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H62" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="I62" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="J62" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="K62" s="1"/>
-      <c r="L62" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M62" s="1"/>
-      <c r="N62" s="1"/>
-    </row>
-    <row r="63" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A63" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="B63" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="G63" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H63" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="I63" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="J63" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="K63" s="1"/>
-      <c r="L63" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M63" s="1"/>
-      <c r="N63" s="1" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="64" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="B64" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="E64" s="1" t="s">
-        <v>329</v>
+        <v>106</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>330</v>
+        <v>107</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>342</v>
+        <v>108</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>343</v>
+        <v>109</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="K64" s="1"/>
+        <v>110</v>
+      </c>
+      <c r="K64" s="1" t="s">
+        <v>514</v>
+      </c>
       <c r="L64" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M64" s="1"/>
-      <c r="N64" s="1"/>
-    </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+        <v>459</v>
+      </c>
+      <c r="M64" s="14" t="s">
+        <v>515</v>
+      </c>
+      <c r="N64" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" ht="90.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>376</v>
+        <v>112</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>377</v>
+        <v>113</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>329</v>
+        <v>114</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>368</v>
+        <v>115</v>
       </c>
       <c r="G65" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>378</v>
+        <v>116</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>338</v>
+        <v>117</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="K65" s="1"/>
+        <v>118</v>
+      </c>
+      <c r="K65" s="1" t="s">
+        <v>517</v>
+      </c>
       <c r="L65" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M65" s="1"/>
-      <c r="N65" s="1"/>
-    </row>
-    <row r="66" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A66" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="B66" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>381</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>329</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="G66" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="I66" s="1" t="s">
-        <v>338</v>
-      </c>
-      <c r="J66" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="K66" s="1"/>
-      <c r="L66" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M66" s="1"/>
-      <c r="N66" s="1"/>
-    </row>
-    <row r="67" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A67" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="B67" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E67" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="G67" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>331</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="K67" s="1"/>
-      <c r="L67" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M67" s="1"/>
-      <c r="N67" s="1"/>
-    </row>
-    <row r="68" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A68" s="5" t="s">
-        <v>430</v>
-      </c>
-      <c r="B68" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E68" s="1" t="s">
-        <v>329</v>
-      </c>
-      <c r="F68" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="G68" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="I68" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="K68" s="1"/>
-      <c r="L68" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M68" s="1"/>
-      <c r="N68" s="1"/>
+        <v>459</v>
+      </c>
+      <c r="M65" s="14" t="s">
+        <v>516</v>
+      </c>
+      <c r="N65" s="1" t="s">
+        <v>119</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N68" xr:uid="{00000000-0009-0000-0000-000003000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N68">
-      <sortCondition ref="G1:G68"/>
+  <autoFilter ref="A1:N65" xr:uid="{00000000-0009-0000-0000-000003000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N65">
+      <sortCondition ref="A1:A65"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="L2:L398">
+  <conditionalFormatting sqref="L2:L395">
     <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"PASS"</formula>
     </cfRule>
@@ -4790,33 +4776,49 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="D2:D398" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D395" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Happy path,Negative,Boundary,Alternative flow,Phi chức năng"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G398" xr:uid="{00000000-0002-0000-0300-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G395" xr:uid="{00000000-0002-0000-0300-000001000000}">
       <formula1>"Cao,Trung,Thấp"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L2:L398" xr:uid="{00000000-0002-0000-0300-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="L2:L395" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>"Chưa chạy,PASS,FAIL"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="M2" r:id="rId1" xr:uid="{50F66AAF-B0D6-4015-AE81-202020A4C517}"/>
-    <hyperlink ref="M3" r:id="rId2" xr:uid="{A82CC3A9-D097-4E0D-BC9C-E140A8961EB2}"/>
-    <hyperlink ref="M4" r:id="rId3" xr:uid="{08D47271-6BFF-47CF-A4E0-50C3B7CBE0C6}"/>
-    <hyperlink ref="M5" r:id="rId4" xr:uid="{9F651E7B-E02C-482C-A9C3-B48CE366708D}"/>
-    <hyperlink ref="M6" r:id="rId5" xr:uid="{A864ECE4-9FCB-49E2-B4CA-C451B08DAD6B}"/>
-    <hyperlink ref="M7" r:id="rId6" xr:uid="{A93B080E-95D8-407A-B7EF-3EF80B22C84E}"/>
-    <hyperlink ref="M8" r:id="rId7" xr:uid="{6B3DF791-B948-4A8E-A3AC-C8A2DC934749}"/>
-    <hyperlink ref="M9" r:id="rId8" xr:uid="{54F1630E-C33A-44D8-AF37-43D154BB6BAD}"/>
-    <hyperlink ref="M10" r:id="rId9" xr:uid="{23368E01-5C93-453F-9C9A-97753332BDA4}"/>
-    <hyperlink ref="M11" r:id="rId10" xr:uid="{052C7473-5CF6-451A-BECC-1E425E96FDD2}"/>
-    <hyperlink ref="M15" r:id="rId11" xr:uid="{0DC140F7-DC54-47D0-8FE4-B05287842DF7}"/>
-    <hyperlink ref="M16" r:id="rId12" xr:uid="{4D3489F9-5D17-474D-9677-E57F0217832E}"/>
-    <hyperlink ref="M17" r:id="rId13" xr:uid="{3C114A65-7E2A-4CB9-BDE4-077F5E538DB2}"/>
+    <hyperlink ref="M55" r:id="rId1" xr:uid="{50F66AAF-B0D6-4015-AE81-202020A4C517}"/>
+    <hyperlink ref="M56" r:id="rId2" xr:uid="{A82CC3A9-D097-4E0D-BC9C-E140A8961EB2}"/>
+    <hyperlink ref="M57" r:id="rId3" xr:uid="{08D47271-6BFF-47CF-A4E0-50C3B7CBE0C6}"/>
+    <hyperlink ref="M59" r:id="rId4" xr:uid="{9F651E7B-E02C-482C-A9C3-B48CE366708D}"/>
+    <hyperlink ref="M60" r:id="rId5" xr:uid="{A864ECE4-9FCB-49E2-B4CA-C451B08DAD6B}"/>
+    <hyperlink ref="M61" r:id="rId6" xr:uid="{A93B080E-95D8-407A-B7EF-3EF80B22C84E}"/>
+    <hyperlink ref="M63" r:id="rId7" xr:uid="{6B3DF791-B948-4A8E-A3AC-C8A2DC934749}"/>
+    <hyperlink ref="M2" r:id="rId8" xr:uid="{54F1630E-C33A-44D8-AF37-43D154BB6BAD}"/>
+    <hyperlink ref="M3" r:id="rId9" xr:uid="{23368E01-5C93-453F-9C9A-97753332BDA4}"/>
+    <hyperlink ref="M4" r:id="rId10" xr:uid="{052C7473-5CF6-451A-BECC-1E425E96FDD2}"/>
+    <hyperlink ref="M8" r:id="rId11" xr:uid="{0DC140F7-DC54-47D0-8FE4-B05287842DF7}"/>
+    <hyperlink ref="M9" r:id="rId12" xr:uid="{4D3489F9-5D17-474D-9677-E57F0217832E}"/>
+    <hyperlink ref="M12" r:id="rId13" xr:uid="{3C114A65-7E2A-4CB9-BDE4-077F5E538DB2}"/>
+    <hyperlink ref="M13" r:id="rId14" xr:uid="{4051FF90-4DDE-45C7-9B35-C9EC983A64EB}"/>
+    <hyperlink ref="M14" r:id="rId15" xr:uid="{110BCE89-D2A5-455E-8067-5BD436DCF537}"/>
+    <hyperlink ref="M30" r:id="rId16" xr:uid="{71A0AEE4-3217-432A-8E55-341AEA509C97}"/>
+    <hyperlink ref="M31" r:id="rId17" xr:uid="{34ED325D-177A-4015-BC1E-E8EB6CA12D1E}"/>
+    <hyperlink ref="M32" r:id="rId18" xr:uid="{285250BE-5FDB-4B41-BDEE-17FF6DD89EF3}"/>
+    <hyperlink ref="M35" r:id="rId19" xr:uid="{293CF10D-69D5-48C8-9635-D73783E4072E}"/>
+    <hyperlink ref="M36" r:id="rId20" xr:uid="{6CBC592C-DD18-4821-8CB9-2097F3876169}"/>
+    <hyperlink ref="M11" r:id="rId21" xr:uid="{F04C9117-9C1E-4044-8F1D-E7B038BD9AB0}"/>
+    <hyperlink ref="M20" r:id="rId22" xr:uid="{F99C49CE-6294-484F-B479-CC14CB9FCE20}"/>
+    <hyperlink ref="M21" r:id="rId23" xr:uid="{80D4EF91-CE9C-4110-8AB1-EFE62AAAB626}"/>
+    <hyperlink ref="M22" r:id="rId24" xr:uid="{3EE94D8E-A41D-4531-8A33-6FE8222ED015}"/>
+    <hyperlink ref="M23" r:id="rId25" xr:uid="{75643E59-4472-4355-8654-FE4B15D48658}"/>
+    <hyperlink ref="M58" r:id="rId26" xr:uid="{AE7C3925-3134-4861-A4E6-C7B68DE91762}"/>
+    <hyperlink ref="M62" r:id="rId27" xr:uid="{3AA3DDD4-7123-4057-8041-CF1B902A3E1C}"/>
+    <hyperlink ref="M64" r:id="rId28" xr:uid="{9606907E-556D-4CCC-82F8-9F50D0A02BF1}"/>
+    <hyperlink ref="M65" r:id="rId29" xr:uid="{06E98682-1678-4789-922C-833F9D2B116B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4843,34 +4845,34 @@
   <sheetData>
     <row r="1" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>446</v>
+        <v>423</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>447</v>
+        <v>424</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>448</v>
+        <v>425</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>449</v>
+        <v>426</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>450</v>
+        <v>427</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>451</v>
+        <v>428</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>452</v>
+        <v>429</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>453</v>
+        <v>430</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>454</v>
+        <v>431</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>455</v>
+        <v>432</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -4955,7 +4957,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>457</v>
+        <v>434</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4966,28 +4968,28 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>458</v>
+        <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>459</v>
+        <v>436</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>460</v>
+        <v>437</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>461</v>
+        <v>438</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>462</v>
+        <v>439</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>44</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>463</v>
+        <v>440</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>464</v>
+        <v>441</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -5006,11 +5008,11 @@
       </c>
       <c r="E4" s="6">
         <f t="shared" ref="E4:E11" si="0">F4+G4</f>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F4" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A4,'Test Case'!$L:$L,"PASS")</f>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G4" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A4,'Test Case'!$L:$L,"FAIL")</f>
@@ -5018,7 +5020,7 @@
       </c>
       <c r="H4" s="6">
         <f t="shared" ref="H4:H11" si="1">D4-E4</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I4" s="9">
         <f t="shared" ref="I4:I12" si="2">IF(E4=0,"-",F4/E4)</f>
@@ -5045,11 +5047,11 @@
       </c>
       <c r="E5" s="6">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"PASS")</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A5,'Test Case'!$L:$L,"FAIL")</f>
@@ -5057,7 +5059,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" si="2"/>
@@ -5080,15 +5082,15 @@
       </c>
       <c r="D6" s="6">
         <f>COUNTIF('Test Case'!$B:$B,$A6)</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F6" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A6,'Test Case'!$L:$L,"PASS")</f>
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G6" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A6,'Test Case'!$L:$L,"FAIL")</f>
@@ -5096,7 +5098,7 @@
       </c>
       <c r="H6" s="6">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I6" s="9">
         <f t="shared" si="2"/>
@@ -5119,15 +5121,15 @@
       </c>
       <c r="D7" s="6">
         <f>COUNTIF('Test Case'!$B:$B,$A7)</f>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E7" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F7" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A7,'Test Case'!$L:$L,"PASS")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G7" s="6">
         <f>COUNTIFS('Test Case'!$B:$B,$A7,'Test Case'!$L:$L,"FAIL")</f>
@@ -5135,11 +5137,11 @@
       </c>
       <c r="H7" s="6">
         <f t="shared" si="1"/>
-        <v>11</v>
-      </c>
-      <c r="I7" s="9" t="str">
+        <v>4</v>
+      </c>
+      <c r="I7" s="9">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>1</v>
       </c>
       <c r="J7" s="6">
         <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A7,2)&amp;"-*")</f>
@@ -5304,23 +5306,23 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>465</v>
+        <v>442</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>466</v>
+        <v>443</v>
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="10">
         <f>SUM(D4:D11)</f>
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E12" s="10">
         <f>SUM(E4:E11)</f>
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="F12" s="10">
         <f>SUM(F4:F11)</f>
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="G12" s="10">
         <f>SUM(G4:G11)</f>
@@ -5328,7 +5330,7 @@
       </c>
       <c r="H12" s="10">
         <f>SUM(H4:H11)</f>
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="I12" s="12">
         <f t="shared" si="2"/>
@@ -5341,7 +5343,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>467</v>
+        <v>444</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5351,13 +5353,13 @@
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4" t="s">
-        <v>459</v>
+        <v>436</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>461</v>
+        <v>438</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>462</v>
+        <v>439</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -5372,7 +5374,7 @@
       </c>
       <c r="E16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"PASS")</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"FAIL")</f>
@@ -5387,11 +5389,11 @@
       <c r="C17" s="1"/>
       <c r="D17" s="6">
         <f>COUNTIF('Test Case'!$D:$D,$A17)</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"PASS")</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"FAIL")</f>
@@ -5410,7 +5412,7 @@
       </c>
       <c r="E18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"PASS")</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"FAIL")</f>
@@ -5425,11 +5427,11 @@
       <c r="C19" s="1"/>
       <c r="D19" s="6">
         <f>COUNTIF('Test Case'!$D:$D,$A19)</f>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"PASS")</f>
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="F19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"FAIL")</f>
@@ -5438,7 +5440,7 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>321</v>
+        <v>298</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -5457,28 +5459,28 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>468</v>
+        <v>445</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>469</v>
+        <v>446</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4" t="s">
-        <v>464</v>
+        <v>441</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>470</v>
+        <v>447</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>471</v>
+        <v>448</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>472</v>
+        <v>449</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -5497,7 +5499,7 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>456</v>
+        <v>433</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -5516,7 +5518,7 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>473</v>
+        <v>450</v>
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -5535,7 +5537,7 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>474</v>
+        <v>451</v>
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -5554,16 +5556,16 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>475</v>
+        <v>452</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>476</v>
+        <v>453</v>
       </c>
       <c r="B31" s="15" t="str">
         <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
-        <v>Đã chạy 16 / 67 TC; PASS 16; FAIL 0; tỉ lệ pass 100.0%</v>
+        <v>Đã chạy 38 / 64 TC; PASS 38; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>
@@ -5576,7 +5578,7 @@
     </row>
     <row r="32" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>477</v>
+        <v>454</v>
       </c>
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
@@ -5590,7 +5592,7 @@
     </row>
     <row r="33" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>478</v>
+        <v>455</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
@@ -5604,7 +5606,7 @@
     </row>
     <row r="34" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>479</v>
+        <v>456</v>
       </c>
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
@@ -5618,7 +5620,7 @@
     </row>
     <row r="35" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>480</v>
+        <v>457</v>
       </c>
       <c r="B35" s="16"/>
       <c r="C35" s="16"/>

</xml_diff>

<commit_message>
Thêm Testcase cho UC22 và UC24
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648A381E-8F35-4D57-8F56-BCEEEE8A6FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7589E0B-DD8E-480C-B14B-67FF0ED23B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="678">
   <si>
     <t>UC</t>
   </si>
@@ -1616,6 +1616,519 @@
   </si>
   <si>
     <t>HTTP 403 Forbidden, success=false, maLoi="KHONG_CO_QUYEN", message="Bạn không có quyền thực hiện thao tác này". Hệ thống phân quyền chặt chẽ, chặn thành công khi tài khoản Phuc vu gọi API thanh toán của Thu ngan. Dữ liệu đơn hàng giữ nguyên</t>
+  </si>
+  <si>
+    <t>UC22</t>
+  </si>
+  <si>
+    <t>UC24</t>
+  </si>
+  <si>
+    <t>TC-22-01</t>
+  </si>
+  <si>
+    <t>Xem danh sách thực đơn (Chủ quán xem được toàn bộ món)</t>
+  </si>
+  <si>
+    <t>UC22 Main Flow (bước 1); GET /api/menu-items</t>
+  </si>
+  <si>
+    <t>Đã nạp lại schema.sql rồi seed.sql; server đang chạy; đã đăng nhập tài khoản chutquan01 (vai trò CHU_QUAN).</t>
+  </si>
+  <si>
+    <t>GET /api/menu-items; Bearer token của chutquan01</t>
+  </si>
+  <si>
+    <t>HTTP 200, success=true. data chứa danh sách tất cả các món ăn gồm: id, tenMon, gia, trangThai (CON_HANG, TAM_HET). Bảng thực đơn trên giao diện hiển thị đầy đủ các món.</t>
+  </si>
+  <si>
+    <t>HTTP 200, success=true, trả về đầy đủ danh sách món kèm đơn giá và trạng thái bán. Giao diện vẽ bảng thực đơn chính xác.</t>
+  </si>
+  <si>
+    <t>Khớp TC-22-01 trong tests/uc22.test.js</t>
+  </si>
+  <si>
+    <t>TC-22-02</t>
+  </si>
+  <si>
+    <t>Thêm món mới hợp lệ thành công (tên được chuẩn hóa bỏ khoảng trắng thừa)</t>
+  </si>
+  <si>
+    <t>UC22 Main Flow (bước 2-6); POST /api/menu-items</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Món "Cà phê muối" chưa tồn tại trong thực đơn.</t>
+  </si>
+  <si>
+    <t>POST /api/menu-items; body: { tenMon: "  Cà   phê muối ", gia: 35000 }</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created. Tên món được tự động cắt gọn khoảng trắng thừa thành "Cà phê muối", gia = 35000, trangThai mặc định = "CON_HANG". Toast thông báo: "Đã thêm \"Cà phê muối\" vào thực đơn." và danh sách món được cập nhật ngay lập tức. CSDL có bản ghi mới trong bảng mon_an.</t>
+  </si>
+  <si>
+    <t>TC-22-03</t>
+  </si>
+  <si>
+    <t>Thêm món với tên trống hoặc chỉ chứa khoảng trắng (EF-1)</t>
+  </si>
+  <si>
+    <t>EP (invalid class: tên món rỗng / toàn khoảng trắng)</t>
+  </si>
+  <si>
+    <t>UC22 EF-1; POST /api/menu-items; mã lỗi TEN_MON_TRONG</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Server đang chạy.</t>
+  </si>
+  <si>
+    <t>(a) tenMon = "", gia = 35000
+(b) tenMon = "   ", gia = 35000
+(c) tenMon = undefined / null</t>
+  </si>
+  <si>
+    <t>Giao diện: Hiển thị lỗi màu đỏ "Vui lòng nhập tên món" dưới ô tên món, focus về ô tên món.
+API: HTTP 400 Bad Request, success=false, maLoi=TEN_MON_TRONG. Không ghi dữ liệu vào CSDL.</t>
+  </si>
+  <si>
+    <t>TC-22-04</t>
+  </si>
+  <si>
+    <t>Thêm món với tên vượt quá 100 ký tự (EF-2)</t>
+  </si>
+  <si>
+    <t>BVA (ngay trên biên 100 ký tự: 101 ký tự)</t>
+  </si>
+  <si>
+    <t>UC22 EF-2; POST /api/menu-items; mã lỗi TEN_MON_QUA_DAI</t>
+  </si>
+  <si>
+    <t>tenMon = chuỗi 101 ký tự "A" ("A"×101), gia = 35000</t>
+  </si>
+  <si>
+    <t>Giao diện: Thuộc tính maxlength="100" ngăn người dùng nhập quá 100 ký tự.
+API: HTTP 400 Bad Request, success=false, maLoi=TEN_MON_QUA_DAI, message="Tên món tối đa 100 ký tự". Không lưu CSDL.</t>
+  </si>
+  <si>
+    <t>TC-22-05</t>
+  </si>
+  <si>
+    <t>Thêm món trùng tên đã có trong thực đơn (không phân biệt hoa thường) (EF-3)</t>
+  </si>
+  <si>
+    <t>Black-box theo UC Spec (EF-3)</t>
+  </si>
+  <si>
+    <t>UC22 EF-3; POST /api/menu-items; mã lỗi TEN_MON_DA_TON_TAI</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Món "Cà phê đen" đã có sẵn trong thực đơn.</t>
+  </si>
+  <si>
+    <t>tenMon = "CÀ PHÊ ĐEN" (viết hoa toàn bộ), gia = 30000</t>
+  </si>
+  <si>
+    <t>HTTP 409 Conflict, success=false, maLoi=TEN_MON_DA_TON_TAI, message="Món \"Cà phê đen\" đã có trong thực đơn". Không tạo bản ghi trùng lặp trong CSDL.</t>
+  </si>
+  <si>
+    <t>TC-22-06</t>
+  </si>
+  <si>
+    <t>Giá món ở biên hợp lệ (1 đồng và 10.000.000 đồng)</t>
+  </si>
+  <si>
+    <t>BVA (biên dưới = 1; biên trên = 10.000.000)</t>
+  </si>
+  <si>
+    <t>UC22 Main Flow; POST /api/menu-items; BVA giá hợp lệ</t>
+  </si>
+  <si>
+    <t>(a) tenMon = "Món giá 1 đồng", gia = 1
+(b) tenMon = "Món giá 10 triệu", gia = 10000000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created cho cả 2 trường hợp. Món được lưu thành công vào CSDL với đúng giá trị biên 1đ và 10.000.000đ.</t>
+  </si>
+  <si>
+    <t>TC-22-07</t>
+  </si>
+  <si>
+    <t>Giá món không hợp lệ: 0, số âm, vượt 10 triệu, số thập phân, chuỗi, null (EF-4)</t>
+  </si>
+  <si>
+    <t>EP + BVA (invalid class &amp; ngoài biên)</t>
+  </si>
+  <si>
+    <t>UC22 EF-4; POST /api/menu-items; mã lỗi GIA_KHONG_HOP_LE</t>
+  </si>
+  <si>
+    <t>Thử các trường hợp gia:
+(a) gia = 0
+(b) gia = -1000
+(c) gia = 10000001
+(d) gia = 1500.5
+(e) gia = "35000"
+(f) gia = null</t>
+  </si>
+  <si>
+    <t>Giao diện: Báo lỗi "Giá phải là số nguyên từ 1 đến 10.000.000 đồng" dưới ô giá.
+API: HTTP 400 Bad Request, success=false, maLoi=GIA_KHONG_HOP_LE. Không lưu vào CSDL.</t>
+  </si>
+  <si>
+    <t>TC-22-08</t>
+  </si>
+  <si>
+    <t>Sửa giá món có sẵn trong thực đơn (AF-1)</t>
+  </si>
+  <si>
+    <t>Black-box theo UC Spec (AF-1)</t>
+  </si>
+  <si>
+    <t>UC22 AF-1; PATCH /api/menu-items/:id; capNhatGia</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Món "Cà phê đen" (mon-01) đang có giá 25.000đ.</t>
+  </si>
+  <si>
+    <t>PATCH /api/menu-items/mon-01; body: { gia: 28000 }</t>
+  </si>
+  <si>
+    <t>HTTP 200 OK. CSDL cập nhật mon_an.gia = 28000, trạng thái giữ nguyên. Giao diện thông báo: "Đã đổi giá \"Cà phê đen\" thành 28.000đ." và cập nhật giá hiển thị.</t>
+  </si>
+  <si>
+    <t>TC-22-09</t>
+  </si>
+  <si>
+    <t>Tắt bán (chuyển Tạm hết) và Bật bán lại (chuyển Đang bán) (AF-2)</t>
+  </si>
+  <si>
+    <t>Black-box theo UC Spec (AF-2)</t>
+  </si>
+  <si>
+    <t>UC22 AF-2; PATCH /api/menu-items/:id; capNhatTrangThai</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). mon-01 đang "CON_HANG", mon-03 đang "TAM_HET".</t>
+  </si>
+  <si>
+    <t>(a) PATCH /api/menu-items/mon-01 với { trangThai: "TAM_HET" }
+(b) PATCH /api/menu-items/mon-03 với { trangThai: "CON_HANG" }</t>
+  </si>
+  <si>
+    <t>HTTP 200 OK cho cả 2 thao tác:
+(a) mon-01 chuyển sang TAM_HET, nhãn đổi "Tạm hết", nút đổi "Bật bán". Màn hình Phục vụ hiện món màu xám, nút "+ Thêm" bị vô hiệu hóa.
+(b) mon-03 chuyển sang CON_HANG, nhãn đổi "Đang bán", nút đổi "Tắt bán". Màn hình Phục vụ cho phép gọi món bình thường.</t>
+  </si>
+  <si>
+    <t>TC-22-10</t>
+  </si>
+  <si>
+    <t>Sửa món không tồn tại trong hệ thống (EF-5)</t>
+  </si>
+  <si>
+    <t>EP (invalid class: monId không tồn tại)</t>
+  </si>
+  <si>
+    <t>UC22 EF-5; PATCH /api/menu-items/:id; mã lỗi MON_KHONG_TON_TAI</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Mã mon-99 không tồn tại trong CSDL.</t>
+  </si>
+  <si>
+    <t>PATCH /api/menu-items/mon-99; body: { gia: 28000 }</t>
+  </si>
+  <si>
+    <t>HTTP 404 Not Found, success=false, maLoi=MON_KHONG_TON_TAI, message="Không tìm thấy món". Giao diện thông báo lỗi và tự động tải lại danh sách thực đơn.</t>
+  </si>
+  <si>
+    <t>TC-22-11</t>
+  </si>
+  <si>
+    <t>Sửa món với dữ liệu rỗng hoặc trạng thái không hợp lệ</t>
+  </si>
+  <si>
+    <t>EP (invalid class: trạng thái ngoài ENUM / payload rỗng)</t>
+  </si>
+  <si>
+    <t>UC22; PATCH /api/menu-items/:id; mã lỗi TRANG_THAI_KHONG_HOP_LE / DU_LIEU_KHONG_HOP_LE</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Món mon-01 đang tồn tại.</t>
+  </si>
+  <si>
+    <t>(a) PATCH /api/menu-items/mon-01; body: { gia: 28000, trangThai: "HET_HANG" }
+(b) PATCH /api/menu-items/mon-01; body: {}</t>
+  </si>
+  <si>
+    <t>(a) HTTP 400 Bad Request, maLoi=TRANG_THAI_KHONG_HOP_LE. Không sửa bất kỳ trường nào (kể cả giá gửi kèm).
+(b) HTTP 400 Bad Request, maLoi=DU_LIEU_KHONG_HOP_LE, message="Không có thông tin cần sửa".</t>
+  </si>
+  <si>
+    <t>TC-22-12</t>
+  </si>
+  <si>
+    <t>Gọi API Quản lý menu khi chưa đăng nhập (EF-6 Security)</t>
+  </si>
+  <si>
+    <t>EP (invalid class: thiếu Authorization header)</t>
+  </si>
+  <si>
+    <t>UC22 EF-6; NFR-Security; middleware verifyToken; mã lỗi CHUA_DANG_NHAP</t>
+  </si>
+  <si>
+    <t>Chưa đăng nhập, không có token Authorization.</t>
+  </si>
+  <si>
+    <t>Gọi GET /api/menu-items, POST /api/menu-items, PATCH /api/menu-items/mon-01 không gửi header Authorization</t>
+  </si>
+  <si>
+    <t>HTTP 401 Unauthorized, success=false, maLoi=CHUA_DANG_NHAP, message="Vui lòng đăng nhập". Hệ thống từ chối mọi yêu cầu và không thay đổi dữ liệu.</t>
+  </si>
+  <si>
+    <t>TC-22-13</t>
+  </si>
+  <si>
+    <t>Sai vai trò (Phục vụ, Barista, Thu ngân) gọi API Quản lý menu bị từ chối (EF-6 Security)</t>
+  </si>
+  <si>
+    <t>EP (invalid class: vai trò không phải CHU_QUAN)</t>
+  </si>
+  <si>
+    <t>UC22 EF-6; NFR-Security; middleware requireRole('CHU_QUAN'); mã lỗi KHONG_CO_QUYEN</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập với tài khoản vai trò PHUC_VU, BARISTA hoặc THU_NGAN (có token hợp lệ nhưng sai quyền).</t>
+  </si>
+  <si>
+    <t>Dùng token PHUC_VU / BARISTA / THU_NGAN gọi GET, POST, PATCH /api/menu-items</t>
+  </si>
+  <si>
+    <t>HTTP 403 Forbidden, success=false, maLoi=KHONG_CO_QUYEN, message="Bạn không có quyền thực hiện thao tác này". Không thêm/sửa món ăn.</t>
+  </si>
+  <si>
+    <t>TC-22-14</t>
+  </si>
+  <si>
+    <t>Tìm kiếm món ăn trong thực đơn bằng tiếng Việt không dấu (AF-3)</t>
+  </si>
+  <si>
+    <t>Black-box theo UC Spec (AF-3)</t>
+  </si>
+  <si>
+    <t>UC22 AF-3; hàm boDau() trên giao diện quan-ly-menu.js</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Thực đơn có món "Trà đào", "Cà phê sữa", "Bạc xỉu".</t>
+  </si>
+  <si>
+    <t>Nhập vào ô "Tìm món": "tra dao", sau đó đổi thành "bac xiu"</t>
+  </si>
+  <si>
+    <t>Giao diện lọc món tức thì: gõ "tra dao" hiển thị món "Trà đào", gõ "bac xiu" hiển thị món "Bạc xỉu". Món không khớp bị ẩn. Khi xóa ô tìm kiếm thì bảng hiển thị lại đầy đủ thực đơn.</t>
+  </si>
+  <si>
+    <t>TC-24-01</t>
+  </si>
+  <si>
+    <t>Xem báo cáo doanh thu theo khoảng ngày hợp lệ</t>
+  </si>
+  <si>
+    <t>UC24 Main Flow (bước 1-6); GET /api/reports/revenue</t>
+  </si>
+  <si>
+    <t>Đã nạp lại schema.sql rồi seed.sql; đã đăng nhập tài khoản chutquan01 (vai trò CHU_QUAN). Trong khoảng ngày chọn có các đơn hàng thanh toán thành công.</t>
+  </si>
+  <si>
+    <t>GET /api/reports/revenue?tuNgay=2026-10-10&amp;denNgay=2026-10-12 với Bearer token của chutquan01</t>
+  </si>
+  <si>
+    <t>HTTP 200 OK. data trả về gồm: tuNgay, denNgay, soDon, doanhThu, trungBinhDon (làm tròn đến đồng); theoPhuongThuc gồm đủ 2 phương thức TIEN_MAT và QR (kể cả phương thức có doanh thu = 0); theoNgay gồm doanh thu từng ngày; topMon gồm tối đa 5 món bán chạy nhất (không tính món đã hủy).</t>
+  </si>
+  <si>
+    <t>TC-24-02</t>
+  </si>
+  <si>
+    <t>Truy vấn dữ liệu tính trọn vẹn mốc thời gian từ 00:00:00 ngày đầu đến trước 00:00:00 ngày sau ngày cuối</t>
+  </si>
+  <si>
+    <t>Functional / Boundary</t>
+  </si>
+  <si>
+    <t>UC24 Main Flow (bước 5); BaoCaoService.layBaoCao</t>
+  </si>
+  <si>
+    <t>GET /api/reports/revenue?tuNgay=2026-10-10&amp;denNgay=2026-10-12</t>
+  </si>
+  <si>
+    <t>Các hàm trong BaoCaoRepository được gọi với khoảng mốc thời gian chuẩn: tuLuc = "2026-10-10 00:00:00" đến denTruoc = "2026-10-13 00:00:00", đảm bảo tính trọn vẹn tất cả giao dịch đến 23:59:59 của ngày kết thúc.</t>
+  </si>
+  <si>
+    <t>TC-24-03</t>
+  </si>
+  <si>
+    <t>Biên ngày cuối tháng hoặc cuối năm vẫn cộng mốc giờ chính xác</t>
+  </si>
+  <si>
+    <t>BVA (ranh giới ngày cuối năm 31/12)</t>
+  </si>
+  <si>
+    <t>UC24; BaoCaoService.vietNgay; BVA ngày</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN).</t>
+  </si>
+  <si>
+    <t>GET /api/reports/revenue?tuNgay=2026-12-31 (xem báo cáo ngày cuối năm)</t>
+  </si>
+  <si>
+    <t>HTTP 200 OK. Mốc giờ denTruoc được tính chính xác sang năm mới: "2026-12-31 00:00:00" đến "2027-01-01 00:00:00" (không bị tràn tháng hay lỗi ngày phi lý).</t>
+  </si>
+  <si>
+    <t>TC-24-04</t>
+  </si>
+  <si>
+    <t>Không truyền tham số ngày -&gt; Mặc định xem báo cáo ngày hôm nay (AF-2 / Main Flow bước 1)</t>
+  </si>
+  <si>
+    <t>Functional (mặc định / AF-2)</t>
+  </si>
+  <si>
+    <t>UC24 Main Flow (bước 1) &amp; AF-2; GET /api/reports/revenue</t>
+  </si>
+  <si>
+    <t>GET /api/reports/revenue (không truyền query param tuNgay, denNgay)</t>
+  </si>
+  <si>
+    <t>HTTP 200 OK. Hệ thống tự động điền tuNgay = denNgay = ngày hiện tại của máy chủ dạng YYYY-MM-DD và trả về báo cáo của ngày hôm nay.</t>
+  </si>
+  <si>
+    <t>TC-24-05</t>
+  </si>
+  <si>
+    <t>Khoảng ngày không có giao dịch thanh toán thành công (AF-3)</t>
+  </si>
+  <si>
+    <t>UC24 AF-3; BaoCaoService; xử lý Division by Zero</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Ngày 2026-10-13 chưa có giao dịch nào thành công.</t>
+  </si>
+  <si>
+    <t>GET /api/reports/revenue?tuNgay=2026-10-13&amp;denNgay=2026-10-13</t>
+  </si>
+  <si>
+    <t>HTTP 200 OK. soDon = 0, doanhThu = 0, trungBinhDon = 0 (tránh chia cho 0), theoNgay = [], topMon = []. Giao diện hiển thị: doanh thu 0đ, 0 đơn; các bảng báo "Chưa có món nào được bán trong khoảng này." và "Chưa có doanh thu trong khoảng này."</t>
+  </si>
+  <si>
+    <t>TC-24-06</t>
+  </si>
+  <si>
+    <t>Ngày sai định dạng hoặc là ngày không có thật trong lịch (EF-4)</t>
+  </si>
+  <si>
+    <t>EP (invalid class: định dạng ngày sai / ngày phi lý)</t>
+  </si>
+  <si>
+    <t>UC24 EF-4; GET /api/reports/revenue; mã lỗi NGAY_KHONG_HOP_LE</t>
+  </si>
+  <si>
+    <t>Thử các giá trị tuNgay:
+(a) tuNgay = "10/10/2026" (sai format DD/MM/YYYY)
+(b) tuNgay = "2026-02-30" (ngày 30/02 không tồn tại)
+(c) tuNgay = "2026-13-01" (tháng 13 không tồn tại)
+(d) tuNgay = "abc" (chuỗi ký tự chữ)</t>
+  </si>
+  <si>
+    <t>HTTP 400 Bad Request, success=false, maLoi=NGAY_KHONG_HOP_LE, message="Ngày phải có dạng YYYY-MM-DD và là ngày có thật". Hệ thống không thực hiện truy vấn SQL vào CSDL.</t>
+  </si>
+  <si>
+    <t>TC-24-07</t>
+  </si>
+  <si>
+    <t>"Từ ngày" sau "Đến ngày" hoặc khoảng ngày vượt quá 366 ngày (EF-2, EF-3, Boundary 366 ngày)</t>
+  </si>
+  <si>
+    <t>BVA (ngưỡng 366 ngày) + EP (khoảng ngày ngược)</t>
+  </si>
+  <si>
+    <t>UC24 EF-2 &amp; EF-3; GET /api/reports/revenue; mã lỗi KHOANG_NGAY_KHONG_HOP_LE</t>
+  </si>
+  <si>
+    <t>(a) tuNgay = "2026-10-13", denNgay = "2026-10-01" ("Từ ngày" sau "Đến ngày")
+(b) tuNgay = "2025-01-01", denNgay = "2026-10-13" (651 ngày &gt; 366 ngày)
+(c) tuNgay = "2025-10-14", denNgay = "2026-10-14" (đúng 366 ngày - biên trên hợp lệ)</t>
+  </si>
+  <si>
+    <t>(a) HTTP 400 Bad Request, maLoi=KHOANG_NGAY_KHONG_HOP_LE, message="\"Từ ngày\" không được sau \"Đến ngày\"".
+(b) HTTP 400 Bad Request, maLoi=KHOANG_NGAY_KHONG_HOP_LE, message="Chỉ xem tối đa 366 ngày mỗi lần".
+(c) HTTP 200 OK (biên đúng 366 ngày được chấp nhận).</t>
+  </si>
+  <si>
+    <t>TC-24-08</t>
+  </si>
+  <si>
+    <t>Phân quyền truy cập báo cáo doanh thu: chưa đăng nhập hoặc sai vai trò bị từ chối (EF-5 Security)</t>
+  </si>
+  <si>
+    <t>EP (invalid class: thiếu token / sai vai trò)</t>
+  </si>
+  <si>
+    <t>UC24 EF-5; NFR-Security; middleware verifyToken &amp; requireRole('CHU_QUAN'); mã lỗi CHUA_DANG_NHAP / KHONG_CO_QUYEN</t>
+  </si>
+  <si>
+    <t>Server đang chạy.</t>
+  </si>
+  <si>
+    <t>(a) GET /api/reports/revenue không gửi kèm token Authorization
+(b) GET /api/reports/revenue với token của tài khoản vai trò PHUC_VU, BARISTA hoặc THU_NGAN</t>
+  </si>
+  <si>
+    <t>(a) HTTP 401 Unauthorized, maLoi=CHUA_DANG_NHAP, message="Vui lòng đăng nhập".
+(b) HTTP 403 Forbidden, maLoi=KHONG_CO_QUYEN, message="Bạn không có quyền thực hiện thao tác này". Không để lộ dữ liệu kinh doanh của quán cho vai trò khác.</t>
+  </si>
+  <si>
+    <t>TC-24-09</t>
+  </si>
+  <si>
+    <t>Chọn nhanh khoảng ngày ("Hôm nay", "7 ngày qua", "Tháng này") trên giao diện (AF-1)</t>
+  </si>
+  <si>
+    <t>UC24 AF-1; nút [data-nhanh] trên giao diện bao-cao.html</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Mở trang Báo cáo doanh thu (bao-cao.html).</t>
+  </si>
+  <si>
+    <t>Lần lượt click các nút:
+(a) Nút "Hôm nay"
+(b) Nút "7 ngày qua"
+(c) Nút "Tháng này"</t>
+  </si>
+  <si>
+    <t>Hệ thống tự động tính toán và điền chính xác vào 2 ô "Từ ngày" và "Đến ngày", đồng thời gọi API tải lại báo cáo ngay:
+(a) "Hôm nay": Từ ngày = Đến ngày = ngày hiện tại
+(b) "7 ngày qua": Từ ngày = ngày hiện tại - 6 ngày; Đến ngày = ngày hiện tại
+(c) "Tháng này": Từ ngày = ngày 01 của tháng hiện tại; Đến ngày = ngày hiện tại</t>
+  </si>
+  <si>
+    <t>TC-24-10</t>
+  </si>
+  <si>
+    <t>Bỏ trống "Từ ngày" khi xem báo cáo trên giao diện (EF-1)</t>
+  </si>
+  <si>
+    <t>EP (invalid class: thiếu trường bắt buộc trên UI)</t>
+  </si>
+  <si>
+    <t>UC24 EF-1; hàm taiBaoCao() trong bao-cao.js</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Mở trang Báo cáo doanh thu.</t>
+  </si>
+  <si>
+    <t>Xóa trống giá trị ở ô "Từ ngày", nhấn nút "Xem báo cáo"</t>
+  </si>
+  <si>
+    <t>Giao diện chặn không gửi request lên server. Hiển thị thông báo lỗi màu đỏ: "Vui lòng chọn \"Từ ngày\"." ngay dưới hàng bộ lọc và tự động focus vào ô "Từ ngày".</t>
   </si>
 </sst>
 </file>
@@ -1625,7 +2138,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1674,6 +2187,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1736,7 +2260,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1782,12 +2306,95 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="FF7F7F7F"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF7F7F7F"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF7F7F7F"/>
@@ -2089,7 +2696,7 @@
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N91"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2152,7 +2759,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>120</v>
       </c>
@@ -2236,7 +2843,7 @@
       </c>
       <c r="N3" s="1"/>
     </row>
-    <row r="4" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>132</v>
       </c>
@@ -2318,7 +2925,7 @@
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
     </row>
-    <row r="6" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>143</v>
       </c>
@@ -2358,7 +2965,7 @@
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
     </row>
-    <row r="7" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>148</v>
       </c>
@@ -2442,7 +3049,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>162</v>
       </c>
@@ -2568,7 +3175,7 @@
       </c>
       <c r="N11" s="1"/>
     </row>
-    <row r="12" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>181</v>
       </c>
@@ -2610,7 +3217,7 @@
       </c>
       <c r="N12" s="1"/>
     </row>
-    <row r="13" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>187</v>
       </c>
@@ -2652,7 +3259,7 @@
       </c>
       <c r="N13" s="1"/>
     </row>
-    <row r="14" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>193</v>
       </c>
@@ -2694,7 +3301,7 @@
       </c>
       <c r="N14" s="1"/>
     </row>
-    <row r="15" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>198</v>
       </c>
@@ -2734,7 +3341,7 @@
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>203</v>
       </c>
@@ -2774,7 +3381,7 @@
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
     </row>
-    <row r="17" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>207</v>
       </c>
@@ -2854,7 +3461,7 @@
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>216</v>
       </c>
@@ -3064,7 +3671,7 @@
       </c>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>390</v>
       </c>
@@ -3102,7 +3709,7 @@
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
     </row>
-    <row r="25" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>396</v>
       </c>
@@ -3140,7 +3747,7 @@
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>402</v>
       </c>
@@ -3178,7 +3785,7 @@
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
     </row>
-    <row r="27" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>407</v>
       </c>
@@ -3216,7 +3823,7 @@
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
     </row>
-    <row r="28" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>413</v>
       </c>
@@ -3254,7 +3861,7 @@
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
     </row>
-    <row r="29" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>419</v>
       </c>
@@ -3292,7 +3899,7 @@
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>246</v>
       </c>
@@ -3336,7 +3943,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>253</v>
       </c>
@@ -3380,7 +3987,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>258</v>
       </c>
@@ -3422,7 +4029,7 @@
       </c>
       <c r="N32" s="1"/>
     </row>
-    <row r="33" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>264</v>
       </c>
@@ -3462,7 +4069,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>271</v>
       </c>
@@ -3500,7 +4107,7 @@
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>277</v>
       </c>
@@ -3780,7 +4387,7 @@
       <c r="M41" s="1"/>
       <c r="N41" s="1"/>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>322</v>
       </c>
@@ -3818,7 +4425,7 @@
       <c r="M42" s="1"/>
       <c r="N42" s="1"/>
     </row>
-    <row r="43" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>327</v>
       </c>
@@ -3894,7 +4501,7 @@
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
     </row>
-    <row r="45" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>339</v>
       </c>
@@ -3932,7 +4539,7 @@
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
     </row>
-    <row r="46" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>343</v>
       </c>
@@ -3970,7 +4577,7 @@
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
     </row>
-    <row r="47" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>348</v>
       </c>
@@ -4010,7 +4617,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>353</v>
       </c>
@@ -4086,7 +4693,7 @@
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
     </row>
-    <row r="50" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>362</v>
       </c>
@@ -4124,7 +4731,7 @@
       <c r="M50" s="1"/>
       <c r="N50" s="1"/>
     </row>
-    <row r="51" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>367</v>
       </c>
@@ -4164,7 +4771,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>373</v>
       </c>
@@ -4202,7 +4809,7 @@
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
     </row>
-    <row r="53" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>378</v>
       </c>
@@ -4240,7 +4847,7 @@
       <c r="M53" s="1"/>
       <c r="N53" s="1"/>
     </row>
-    <row r="54" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>383</v>
       </c>
@@ -4280,7 +4887,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>35</v>
       </c>
@@ -4322,7 +4929,7 @@
       </c>
       <c r="N55" s="1"/>
     </row>
-    <row r="56" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>45</v>
       </c>
@@ -4366,7 +4973,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>52</v>
       </c>
@@ -4494,7 +5101,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>72</v>
       </c>
@@ -4538,7 +5145,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>80</v>
       </c>
@@ -4626,7 +5233,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>96</v>
       </c>
@@ -4757,6 +5364,882 @@
       <c r="N65" s="1" t="s">
         <v>119</v>
       </c>
+    </row>
+    <row r="66" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A66" s="17" t="s">
+        <v>520</v>
+      </c>
+      <c r="B66" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C66" s="18" t="s">
+        <v>521</v>
+      </c>
+      <c r="D66" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E66" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F66" s="18" t="s">
+        <v>522</v>
+      </c>
+      <c r="G66" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H66" s="18" t="s">
+        <v>523</v>
+      </c>
+      <c r="I66" s="18" t="s">
+        <v>524</v>
+      </c>
+      <c r="J66" s="18" t="s">
+        <v>525</v>
+      </c>
+      <c r="K66" s="18" t="s">
+        <v>526</v>
+      </c>
+      <c r="L66" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="M66" s="18"/>
+      <c r="N66" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A67" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="B67" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C67" s="18" t="s">
+        <v>529</v>
+      </c>
+      <c r="D67" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E67" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F67" s="18" t="s">
+        <v>530</v>
+      </c>
+      <c r="G67" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H67" s="18" t="s">
+        <v>531</v>
+      </c>
+      <c r="I67" s="18" t="s">
+        <v>532</v>
+      </c>
+      <c r="J67" s="18" t="s">
+        <v>533</v>
+      </c>
+      <c r="K67" s="18"/>
+      <c r="L67" s="17"/>
+      <c r="M67" s="18"/>
+      <c r="N67" s="18"/>
+    </row>
+    <row r="68" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A68" s="17" t="s">
+        <v>534</v>
+      </c>
+      <c r="B68" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C68" s="18" t="s">
+        <v>535</v>
+      </c>
+      <c r="D68" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E68" s="18" t="s">
+        <v>536</v>
+      </c>
+      <c r="F68" s="18" t="s">
+        <v>537</v>
+      </c>
+      <c r="G68" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H68" s="18" t="s">
+        <v>538</v>
+      </c>
+      <c r="I68" s="18" t="s">
+        <v>539</v>
+      </c>
+      <c r="J68" s="18" t="s">
+        <v>540</v>
+      </c>
+      <c r="K68" s="18"/>
+      <c r="L68" s="17"/>
+      <c r="M68" s="18"/>
+      <c r="N68" s="18"/>
+    </row>
+    <row r="69" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A69" s="17" t="s">
+        <v>541</v>
+      </c>
+      <c r="B69" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C69" s="18" t="s">
+        <v>542</v>
+      </c>
+      <c r="D69" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E69" s="18" t="s">
+        <v>543</v>
+      </c>
+      <c r="F69" s="18" t="s">
+        <v>544</v>
+      </c>
+      <c r="G69" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="H69" s="18" t="s">
+        <v>538</v>
+      </c>
+      <c r="I69" s="18" t="s">
+        <v>545</v>
+      </c>
+      <c r="J69" s="18" t="s">
+        <v>546</v>
+      </c>
+      <c r="K69" s="18"/>
+      <c r="L69" s="17"/>
+      <c r="M69" s="18"/>
+      <c r="N69" s="18"/>
+    </row>
+    <row r="70" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A70" s="17" t="s">
+        <v>547</v>
+      </c>
+      <c r="B70" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C70" s="18" t="s">
+        <v>548</v>
+      </c>
+      <c r="D70" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E70" s="18" t="s">
+        <v>549</v>
+      </c>
+      <c r="F70" s="18" t="s">
+        <v>550</v>
+      </c>
+      <c r="G70" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H70" s="18" t="s">
+        <v>551</v>
+      </c>
+      <c r="I70" s="18" t="s">
+        <v>552</v>
+      </c>
+      <c r="J70" s="18" t="s">
+        <v>553</v>
+      </c>
+      <c r="K70" s="18"/>
+      <c r="L70" s="17"/>
+      <c r="M70" s="18"/>
+      <c r="N70" s="18"/>
+    </row>
+    <row r="71" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A71" s="17" t="s">
+        <v>554</v>
+      </c>
+      <c r="B71" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C71" s="18" t="s">
+        <v>555</v>
+      </c>
+      <c r="D71" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E71" s="18" t="s">
+        <v>556</v>
+      </c>
+      <c r="F71" s="18" t="s">
+        <v>557</v>
+      </c>
+      <c r="G71" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H71" s="18" t="s">
+        <v>538</v>
+      </c>
+      <c r="I71" s="18" t="s">
+        <v>558</v>
+      </c>
+      <c r="J71" s="18" t="s">
+        <v>559</v>
+      </c>
+      <c r="K71" s="18"/>
+      <c r="L71" s="17"/>
+      <c r="M71" s="18"/>
+      <c r="N71" s="18"/>
+    </row>
+    <row r="72" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A72" s="17" t="s">
+        <v>560</v>
+      </c>
+      <c r="B72" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C72" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="D72" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E72" s="18" t="s">
+        <v>562</v>
+      </c>
+      <c r="F72" s="18" t="s">
+        <v>563</v>
+      </c>
+      <c r="G72" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H72" s="18" t="s">
+        <v>538</v>
+      </c>
+      <c r="I72" s="18" t="s">
+        <v>564</v>
+      </c>
+      <c r="J72" s="18" t="s">
+        <v>565</v>
+      </c>
+      <c r="K72" s="18"/>
+      <c r="L72" s="17"/>
+      <c r="M72" s="18"/>
+      <c r="N72" s="18"/>
+    </row>
+    <row r="73" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A73" s="17" t="s">
+        <v>566</v>
+      </c>
+      <c r="B73" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C73" s="18" t="s">
+        <v>567</v>
+      </c>
+      <c r="D73" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E73" s="18" t="s">
+        <v>568</v>
+      </c>
+      <c r="F73" s="18" t="s">
+        <v>569</v>
+      </c>
+      <c r="G73" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H73" s="18" t="s">
+        <v>570</v>
+      </c>
+      <c r="I73" s="18" t="s">
+        <v>571</v>
+      </c>
+      <c r="J73" s="18" t="s">
+        <v>572</v>
+      </c>
+      <c r="K73" s="18"/>
+      <c r="L73" s="17"/>
+      <c r="M73" s="18"/>
+      <c r="N73" s="18"/>
+    </row>
+    <row r="74" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A74" s="17" t="s">
+        <v>573</v>
+      </c>
+      <c r="B74" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C74" s="18" t="s">
+        <v>574</v>
+      </c>
+      <c r="D74" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E74" s="18" t="s">
+        <v>575</v>
+      </c>
+      <c r="F74" s="18" t="s">
+        <v>576</v>
+      </c>
+      <c r="G74" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H74" s="18" t="s">
+        <v>577</v>
+      </c>
+      <c r="I74" s="18" t="s">
+        <v>578</v>
+      </c>
+      <c r="J74" s="18" t="s">
+        <v>579</v>
+      </c>
+      <c r="K74" s="18"/>
+      <c r="L74" s="17"/>
+      <c r="M74" s="18"/>
+      <c r="N74" s="18"/>
+    </row>
+    <row r="75" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A75" s="17" t="s">
+        <v>580</v>
+      </c>
+      <c r="B75" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C75" s="18" t="s">
+        <v>581</v>
+      </c>
+      <c r="D75" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E75" s="18" t="s">
+        <v>582</v>
+      </c>
+      <c r="F75" s="18" t="s">
+        <v>583</v>
+      </c>
+      <c r="G75" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="H75" s="18" t="s">
+        <v>584</v>
+      </c>
+      <c r="I75" s="18" t="s">
+        <v>585</v>
+      </c>
+      <c r="J75" s="18" t="s">
+        <v>586</v>
+      </c>
+      <c r="K75" s="18"/>
+      <c r="L75" s="17"/>
+      <c r="M75" s="18"/>
+      <c r="N75" s="18"/>
+    </row>
+    <row r="76" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A76" s="17" t="s">
+        <v>587</v>
+      </c>
+      <c r="B76" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C76" s="18" t="s">
+        <v>588</v>
+      </c>
+      <c r="D76" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E76" s="18" t="s">
+        <v>589</v>
+      </c>
+      <c r="F76" s="18" t="s">
+        <v>590</v>
+      </c>
+      <c r="G76" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="H76" s="18" t="s">
+        <v>591</v>
+      </c>
+      <c r="I76" s="18" t="s">
+        <v>592</v>
+      </c>
+      <c r="J76" s="18" t="s">
+        <v>593</v>
+      </c>
+      <c r="K76" s="18"/>
+      <c r="L76" s="17"/>
+      <c r="M76" s="18"/>
+      <c r="N76" s="18"/>
+    </row>
+    <row r="77" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A77" s="17" t="s">
+        <v>594</v>
+      </c>
+      <c r="B77" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C77" s="18" t="s">
+        <v>595</v>
+      </c>
+      <c r="D77" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E77" s="18" t="s">
+        <v>596</v>
+      </c>
+      <c r="F77" s="18" t="s">
+        <v>597</v>
+      </c>
+      <c r="G77" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H77" s="18" t="s">
+        <v>598</v>
+      </c>
+      <c r="I77" s="18" t="s">
+        <v>599</v>
+      </c>
+      <c r="J77" s="18" t="s">
+        <v>600</v>
+      </c>
+      <c r="K77" s="18"/>
+      <c r="L77" s="17"/>
+      <c r="M77" s="18"/>
+      <c r="N77" s="18"/>
+    </row>
+    <row r="78" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A78" s="17" t="s">
+        <v>601</v>
+      </c>
+      <c r="B78" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C78" s="18" t="s">
+        <v>602</v>
+      </c>
+      <c r="D78" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E78" s="18" t="s">
+        <v>603</v>
+      </c>
+      <c r="F78" s="18" t="s">
+        <v>604</v>
+      </c>
+      <c r="G78" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H78" s="18" t="s">
+        <v>605</v>
+      </c>
+      <c r="I78" s="18" t="s">
+        <v>606</v>
+      </c>
+      <c r="J78" s="18" t="s">
+        <v>607</v>
+      </c>
+      <c r="K78" s="18"/>
+      <c r="L78" s="17"/>
+      <c r="M78" s="18"/>
+      <c r="N78" s="18"/>
+    </row>
+    <row r="79" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A79" s="17" t="s">
+        <v>608</v>
+      </c>
+      <c r="B79" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="C79" s="18" t="s">
+        <v>609</v>
+      </c>
+      <c r="D79" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E79" s="18" t="s">
+        <v>610</v>
+      </c>
+      <c r="F79" s="18" t="s">
+        <v>611</v>
+      </c>
+      <c r="G79" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="H79" s="18" t="s">
+        <v>612</v>
+      </c>
+      <c r="I79" s="18" t="s">
+        <v>613</v>
+      </c>
+      <c r="J79" s="18" t="s">
+        <v>614</v>
+      </c>
+      <c r="K79" s="18"/>
+      <c r="L79" s="17"/>
+      <c r="M79" s="18"/>
+      <c r="N79" s="18"/>
+    </row>
+    <row r="80" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A80" s="17" t="s">
+        <v>615</v>
+      </c>
+      <c r="B80" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C80" s="18" t="s">
+        <v>616</v>
+      </c>
+      <c r="D80" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E80" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F80" s="18" t="s">
+        <v>617</v>
+      </c>
+      <c r="G80" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H80" s="18" t="s">
+        <v>618</v>
+      </c>
+      <c r="I80" s="18" t="s">
+        <v>619</v>
+      </c>
+      <c r="J80" s="18" t="s">
+        <v>620</v>
+      </c>
+      <c r="K80" s="18"/>
+      <c r="L80" s="17"/>
+      <c r="M80" s="18"/>
+      <c r="N80" s="18"/>
+    </row>
+    <row r="81" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+      <c r="A81" s="17" t="s">
+        <v>621</v>
+      </c>
+      <c r="B81" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C81" s="18" t="s">
+        <v>622</v>
+      </c>
+      <c r="D81" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E81" s="18" t="s">
+        <v>623</v>
+      </c>
+      <c r="F81" s="18" t="s">
+        <v>624</v>
+      </c>
+      <c r="G81" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H81" s="18" t="s">
+        <v>538</v>
+      </c>
+      <c r="I81" s="18" t="s">
+        <v>625</v>
+      </c>
+      <c r="J81" s="18" t="s">
+        <v>626</v>
+      </c>
+      <c r="K81" s="18"/>
+      <c r="L81" s="17"/>
+      <c r="M81" s="18"/>
+      <c r="N81" s="18"/>
+    </row>
+    <row r="82" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A82" s="17" t="s">
+        <v>627</v>
+      </c>
+      <c r="B82" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C82" s="18" t="s">
+        <v>628</v>
+      </c>
+      <c r="D82" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E82" s="18" t="s">
+        <v>629</v>
+      </c>
+      <c r="F82" s="18" t="s">
+        <v>630</v>
+      </c>
+      <c r="G82" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="H82" s="18" t="s">
+        <v>631</v>
+      </c>
+      <c r="I82" s="18" t="s">
+        <v>632</v>
+      </c>
+      <c r="J82" s="18" t="s">
+        <v>633</v>
+      </c>
+      <c r="K82" s="18"/>
+      <c r="L82" s="17"/>
+      <c r="M82" s="18"/>
+      <c r="N82" s="18"/>
+    </row>
+    <row r="83" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A83" s="17" t="s">
+        <v>634</v>
+      </c>
+      <c r="B83" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C83" s="18" t="s">
+        <v>635</v>
+      </c>
+      <c r="D83" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E83" s="18" t="s">
+        <v>636</v>
+      </c>
+      <c r="F83" s="18" t="s">
+        <v>637</v>
+      </c>
+      <c r="G83" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H83" s="18" t="s">
+        <v>631</v>
+      </c>
+      <c r="I83" s="18" t="s">
+        <v>638</v>
+      </c>
+      <c r="J83" s="18" t="s">
+        <v>639</v>
+      </c>
+      <c r="K83" s="18"/>
+      <c r="L83" s="17"/>
+      <c r="M83" s="18"/>
+      <c r="N83" s="18"/>
+    </row>
+    <row r="84" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A84" s="17" t="s">
+        <v>640</v>
+      </c>
+      <c r="B84" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C84" s="18" t="s">
+        <v>641</v>
+      </c>
+      <c r="D84" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E84" s="18" t="s">
+        <v>610</v>
+      </c>
+      <c r="F84" s="18" t="s">
+        <v>642</v>
+      </c>
+      <c r="G84" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H84" s="18" t="s">
+        <v>643</v>
+      </c>
+      <c r="I84" s="18" t="s">
+        <v>644</v>
+      </c>
+      <c r="J84" s="18" t="s">
+        <v>645</v>
+      </c>
+      <c r="K84" s="18"/>
+      <c r="L84" s="17"/>
+      <c r="M84" s="18"/>
+      <c r="N84" s="18"/>
+    </row>
+    <row r="85" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+      <c r="A85" s="17" t="s">
+        <v>646</v>
+      </c>
+      <c r="B85" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C85" s="18" t="s">
+        <v>647</v>
+      </c>
+      <c r="D85" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E85" s="18" t="s">
+        <v>648</v>
+      </c>
+      <c r="F85" s="18" t="s">
+        <v>649</v>
+      </c>
+      <c r="G85" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H85" s="18" t="s">
+        <v>538</v>
+      </c>
+      <c r="I85" s="18" t="s">
+        <v>650</v>
+      </c>
+      <c r="J85" s="18" t="s">
+        <v>651</v>
+      </c>
+      <c r="K85" s="18"/>
+      <c r="L85" s="17"/>
+      <c r="M85" s="18"/>
+      <c r="N85" s="18"/>
+    </row>
+    <row r="86" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+      <c r="A86" s="17" t="s">
+        <v>652</v>
+      </c>
+      <c r="B86" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C86" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D86" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E86" s="18" t="s">
+        <v>654</v>
+      </c>
+      <c r="F86" s="18" t="s">
+        <v>655</v>
+      </c>
+      <c r="G86" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H86" s="18" t="s">
+        <v>538</v>
+      </c>
+      <c r="I86" s="18" t="s">
+        <v>656</v>
+      </c>
+      <c r="J86" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="K86" s="18"/>
+      <c r="L86" s="17"/>
+      <c r="M86" s="18"/>
+      <c r="N86" s="18"/>
+    </row>
+    <row r="87" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A87" s="17" t="s">
+        <v>658</v>
+      </c>
+      <c r="B87" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C87" s="18" t="s">
+        <v>659</v>
+      </c>
+      <c r="D87" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E87" s="18" t="s">
+        <v>660</v>
+      </c>
+      <c r="F87" s="18" t="s">
+        <v>661</v>
+      </c>
+      <c r="G87" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H87" s="18" t="s">
+        <v>662</v>
+      </c>
+      <c r="I87" s="18" t="s">
+        <v>663</v>
+      </c>
+      <c r="J87" s="18" t="s">
+        <v>664</v>
+      </c>
+      <c r="K87" s="18"/>
+      <c r="L87" s="17"/>
+      <c r="M87" s="18"/>
+      <c r="N87" s="18"/>
+    </row>
+    <row r="88" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+      <c r="A88" s="17" t="s">
+        <v>665</v>
+      </c>
+      <c r="B88" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C88" s="18" t="s">
+        <v>666</v>
+      </c>
+      <c r="D88" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E88" s="18" t="s">
+        <v>568</v>
+      </c>
+      <c r="F88" s="18" t="s">
+        <v>667</v>
+      </c>
+      <c r="G88" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="H88" s="18" t="s">
+        <v>668</v>
+      </c>
+      <c r="I88" s="18" t="s">
+        <v>669</v>
+      </c>
+      <c r="J88" s="18" t="s">
+        <v>670</v>
+      </c>
+      <c r="K88" s="18"/>
+      <c r="L88" s="17"/>
+      <c r="M88" s="18"/>
+      <c r="N88" s="18"/>
+    </row>
+    <row r="89" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A89" s="17" t="s">
+        <v>671</v>
+      </c>
+      <c r="B89" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C89" s="18" t="s">
+        <v>672</v>
+      </c>
+      <c r="D89" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E89" s="18" t="s">
+        <v>673</v>
+      </c>
+      <c r="F89" s="18" t="s">
+        <v>674</v>
+      </c>
+      <c r="G89" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="H89" s="18" t="s">
+        <v>675</v>
+      </c>
+      <c r="I89" s="18" t="s">
+        <v>676</v>
+      </c>
+      <c r="J89" s="18" t="s">
+        <v>677</v>
+      </c>
+      <c r="K89" s="18"/>
+      <c r="L89" s="17"/>
+      <c r="M89" s="18"/>
+      <c r="N89" s="18"/>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A90" s="19"/>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A91" s="19"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N65" xr:uid="{00000000-0009-0000-0000-000003000000}">
@@ -4764,14 +6247,37 @@
       <sortCondition ref="A1:A65"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="L2:L395">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+  <phoneticPr fontId="7" type="noConversion"/>
+  <conditionalFormatting sqref="L2:L65 L90:L395">
+    <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
       <formula>"PASS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
       <formula>"FAIL"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="10" operator="equal">
+      <formula>"Chưa chạy"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L66">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>"PASS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>"FAIL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
+      <formula>"Chưa chạy"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L67:L89">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"PASS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"FAIL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"Chưa chạy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5370,11 +6876,11 @@
       <c r="C16" s="1"/>
       <c r="D16" s="6">
         <f>COUNTIF('Test Case'!$D:$D,$A16)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"PASS")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"FAIL")</f>
@@ -5389,7 +6895,7 @@
       <c r="C17" s="1"/>
       <c r="D17" s="6">
         <f>COUNTIF('Test Case'!$D:$D,$A17)</f>
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="E17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"PASS")</f>
@@ -5408,7 +6914,7 @@
       <c r="C18" s="1"/>
       <c r="D18" s="6">
         <f>COUNTIF('Test Case'!$D:$D,$A18)</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"PASS")</f>
@@ -5427,7 +6933,7 @@
       <c r="C19" s="1"/>
       <c r="D19" s="6">
         <f>COUNTIF('Test Case'!$D:$D,$A19)</f>
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"PASS")</f>

</xml_diff>

<commit_message>
Chạy testcase TC-22-02 và TC-22-03 thành công
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7589E0B-DD8E-480C-B14B-67FF0ED23B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24447F51-0FD0-4321-A778-A573BE4BAEB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="680">
   <si>
     <t>UC</t>
   </si>
@@ -2129,6 +2129,12 @@
   </si>
   <si>
     <t>Giao diện chặn không gửi request lên server. Hiển thị thông báo lỗi màu đỏ: "Vui lòng chọn \"Từ ngày\"." ngay dưới hàng bộ lọc và tự động focus vào ô "Từ ngày".</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-22-02.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-22-03.png</t>
   </si>
 </sst>
 </file>
@@ -2260,7 +2266,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2300,101 +2306,24 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <font>
-        <color rgb="FF7F7F7F"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDEDED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF7F7F7F"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDEDED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF7F7F7F"/>
@@ -2696,7 +2625,7 @@
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
   </sheetPr>
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N89"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -5366,880 +5295,886 @@
       </c>
     </row>
     <row r="66" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A66" s="17" t="s">
+      <c r="A66" s="15" t="s">
         <v>520</v>
       </c>
-      <c r="B66" s="17" t="s">
+      <c r="B66" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C66" s="18" t="s">
+      <c r="C66" s="16" t="s">
         <v>521</v>
       </c>
-      <c r="D66" s="18" t="s">
+      <c r="D66" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="E66" s="18" t="s">
+      <c r="E66" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F66" s="18" t="s">
+      <c r="F66" s="16" t="s">
         <v>522</v>
       </c>
-      <c r="G66" s="17" t="s">
+      <c r="G66" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H66" s="18" t="s">
+      <c r="H66" s="16" t="s">
         <v>523</v>
       </c>
-      <c r="I66" s="18" t="s">
+      <c r="I66" s="16" t="s">
         <v>524</v>
       </c>
-      <c r="J66" s="18" t="s">
+      <c r="J66" s="16" t="s">
         <v>525</v>
       </c>
-      <c r="K66" s="18" t="s">
+      <c r="K66" s="16" t="s">
         <v>526</v>
       </c>
-      <c r="L66" s="17" t="s">
+      <c r="L66" s="15" t="s">
         <v>459</v>
       </c>
-      <c r="M66" s="18"/>
-      <c r="N66" s="18" t="s">
+      <c r="M66" s="16"/>
+      <c r="N66" s="16" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A67" s="17" t="s">
+    <row r="67" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A67" s="15" t="s">
         <v>528</v>
       </c>
-      <c r="B67" s="17" t="s">
+      <c r="B67" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C67" s="18" t="s">
+      <c r="C67" s="16" t="s">
         <v>529</v>
       </c>
-      <c r="D67" s="18" t="s">
+      <c r="D67" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="E67" s="18" t="s">
+      <c r="E67" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F67" s="18" t="s">
+      <c r="F67" s="16" t="s">
         <v>530</v>
       </c>
-      <c r="G67" s="17" t="s">
+      <c r="G67" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H67" s="18" t="s">
+      <c r="H67" s="16" t="s">
         <v>531</v>
       </c>
-      <c r="I67" s="18" t="s">
+      <c r="I67" s="16" t="s">
         <v>532</v>
       </c>
-      <c r="J67" s="18" t="s">
+      <c r="J67" s="16" t="s">
         <v>533</v>
       </c>
-      <c r="K67" s="18"/>
-      <c r="L67" s="17"/>
-      <c r="M67" s="18"/>
-      <c r="N67" s="18"/>
-    </row>
-    <row r="68" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A68" s="17" t="s">
+      <c r="K67" s="16" t="s">
+        <v>529</v>
+      </c>
+      <c r="L67" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="M67" s="14" t="s">
+        <v>678</v>
+      </c>
+      <c r="N67" s="16"/>
+    </row>
+    <row r="68" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A68" s="15" t="s">
         <v>534</v>
       </c>
-      <c r="B68" s="17" t="s">
+      <c r="B68" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C68" s="18" t="s">
+      <c r="C68" s="16" t="s">
         <v>535</v>
       </c>
-      <c r="D68" s="18" t="s">
+      <c r="D68" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E68" s="18" t="s">
+      <c r="E68" s="16" t="s">
         <v>536</v>
       </c>
-      <c r="F68" s="18" t="s">
+      <c r="F68" s="16" t="s">
         <v>537</v>
       </c>
-      <c r="G68" s="17" t="s">
+      <c r="G68" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H68" s="18" t="s">
+      <c r="H68" s="16" t="s">
         <v>538</v>
       </c>
-      <c r="I68" s="18" t="s">
+      <c r="I68" s="16" t="s">
         <v>539</v>
       </c>
-      <c r="J68" s="18" t="s">
+      <c r="J68" s="16" t="s">
         <v>540</v>
       </c>
-      <c r="K68" s="18"/>
-      <c r="L68" s="17"/>
-      <c r="M68" s="18"/>
-      <c r="N68" s="18"/>
+      <c r="K68" s="16" t="s">
+        <v>540</v>
+      </c>
+      <c r="L68" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="M68" s="14" t="s">
+        <v>679</v>
+      </c>
+      <c r="N68" s="16"/>
     </row>
     <row r="69" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A69" s="17" t="s">
+      <c r="A69" s="15" t="s">
         <v>541</v>
       </c>
-      <c r="B69" s="17" t="s">
+      <c r="B69" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C69" s="18" t="s">
+      <c r="C69" s="16" t="s">
         <v>542</v>
       </c>
-      <c r="D69" s="18" t="s">
+      <c r="D69" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="E69" s="18" t="s">
+      <c r="E69" s="16" t="s">
         <v>543</v>
       </c>
-      <c r="F69" s="18" t="s">
+      <c r="F69" s="16" t="s">
         <v>544</v>
       </c>
-      <c r="G69" s="17" t="s">
+      <c r="G69" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="H69" s="18" t="s">
+      <c r="H69" s="16" t="s">
         <v>538</v>
       </c>
-      <c r="I69" s="18" t="s">
+      <c r="I69" s="16" t="s">
         <v>545</v>
       </c>
-      <c r="J69" s="18" t="s">
+      <c r="J69" s="16" t="s">
         <v>546</v>
       </c>
-      <c r="K69" s="18"/>
-      <c r="L69" s="17"/>
-      <c r="M69" s="18"/>
-      <c r="N69" s="18"/>
+      <c r="K69" s="16"/>
+      <c r="L69" s="15"/>
+      <c r="M69" s="16"/>
+      <c r="N69" s="16"/>
     </row>
     <row r="70" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A70" s="17" t="s">
+      <c r="A70" s="15" t="s">
         <v>547</v>
       </c>
-      <c r="B70" s="17" t="s">
+      <c r="B70" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C70" s="18" t="s">
+      <c r="C70" s="16" t="s">
         <v>548</v>
       </c>
-      <c r="D70" s="18" t="s">
+      <c r="D70" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E70" s="18" t="s">
+      <c r="E70" s="16" t="s">
         <v>549</v>
       </c>
-      <c r="F70" s="18" t="s">
+      <c r="F70" s="16" t="s">
         <v>550</v>
       </c>
-      <c r="G70" s="17" t="s">
+      <c r="G70" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H70" s="18" t="s">
+      <c r="H70" s="16" t="s">
         <v>551</v>
       </c>
-      <c r="I70" s="18" t="s">
+      <c r="I70" s="16" t="s">
         <v>552</v>
       </c>
-      <c r="J70" s="18" t="s">
+      <c r="J70" s="16" t="s">
         <v>553</v>
       </c>
-      <c r="K70" s="18"/>
-      <c r="L70" s="17"/>
-      <c r="M70" s="18"/>
-      <c r="N70" s="18"/>
+      <c r="K70" s="16"/>
+      <c r="L70" s="15"/>
+      <c r="M70" s="16"/>
+      <c r="N70" s="16"/>
     </row>
     <row r="71" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A71" s="17" t="s">
+      <c r="A71" s="15" t="s">
         <v>554</v>
       </c>
-      <c r="B71" s="17" t="s">
+      <c r="B71" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C71" s="18" t="s">
+      <c r="C71" s="16" t="s">
         <v>555</v>
       </c>
-      <c r="D71" s="18" t="s">
+      <c r="D71" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="E71" s="18" t="s">
+      <c r="E71" s="16" t="s">
         <v>556</v>
       </c>
-      <c r="F71" s="18" t="s">
+      <c r="F71" s="16" t="s">
         <v>557</v>
       </c>
-      <c r="G71" s="17" t="s">
+      <c r="G71" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H71" s="18" t="s">
+      <c r="H71" s="16" t="s">
         <v>538</v>
       </c>
-      <c r="I71" s="18" t="s">
+      <c r="I71" s="16" t="s">
         <v>558</v>
       </c>
-      <c r="J71" s="18" t="s">
+      <c r="J71" s="16" t="s">
         <v>559</v>
       </c>
-      <c r="K71" s="18"/>
-      <c r="L71" s="17"/>
-      <c r="M71" s="18"/>
-      <c r="N71" s="18"/>
+      <c r="K71" s="16"/>
+      <c r="L71" s="15"/>
+      <c r="M71" s="16"/>
+      <c r="N71" s="16"/>
     </row>
     <row r="72" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A72" s="17" t="s">
+      <c r="A72" s="15" t="s">
         <v>560</v>
       </c>
-      <c r="B72" s="17" t="s">
+      <c r="B72" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C72" s="18" t="s">
+      <c r="C72" s="16" t="s">
         <v>561</v>
       </c>
-      <c r="D72" s="18" t="s">
+      <c r="D72" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E72" s="18" t="s">
+      <c r="E72" s="16" t="s">
         <v>562</v>
       </c>
-      <c r="F72" s="18" t="s">
+      <c r="F72" s="16" t="s">
         <v>563</v>
       </c>
-      <c r="G72" s="17" t="s">
+      <c r="G72" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H72" s="18" t="s">
+      <c r="H72" s="16" t="s">
         <v>538</v>
       </c>
-      <c r="I72" s="18" t="s">
+      <c r="I72" s="16" t="s">
         <v>564</v>
       </c>
-      <c r="J72" s="18" t="s">
+      <c r="J72" s="16" t="s">
         <v>565</v>
       </c>
-      <c r="K72" s="18"/>
-      <c r="L72" s="17"/>
-      <c r="M72" s="18"/>
-      <c r="N72" s="18"/>
+      <c r="K72" s="16"/>
+      <c r="L72" s="15"/>
+      <c r="M72" s="16"/>
+      <c r="N72" s="16"/>
     </row>
     <row r="73" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A73" s="17" t="s">
+      <c r="A73" s="15" t="s">
         <v>566</v>
       </c>
-      <c r="B73" s="17" t="s">
+      <c r="B73" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C73" s="18" t="s">
+      <c r="C73" s="16" t="s">
         <v>567</v>
       </c>
-      <c r="D73" s="18" t="s">
+      <c r="D73" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E73" s="18" t="s">
+      <c r="E73" s="16" t="s">
         <v>568</v>
       </c>
-      <c r="F73" s="18" t="s">
+      <c r="F73" s="16" t="s">
         <v>569</v>
       </c>
-      <c r="G73" s="17" t="s">
+      <c r="G73" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H73" s="18" t="s">
+      <c r="H73" s="16" t="s">
         <v>570</v>
       </c>
-      <c r="I73" s="18" t="s">
+      <c r="I73" s="16" t="s">
         <v>571</v>
       </c>
-      <c r="J73" s="18" t="s">
+      <c r="J73" s="16" t="s">
         <v>572</v>
       </c>
-      <c r="K73" s="18"/>
-      <c r="L73" s="17"/>
-      <c r="M73" s="18"/>
-      <c r="N73" s="18"/>
+      <c r="K73" s="16"/>
+      <c r="L73" s="15"/>
+      <c r="M73" s="16"/>
+      <c r="N73" s="16"/>
     </row>
     <row r="74" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A74" s="17" t="s">
+      <c r="A74" s="15" t="s">
         <v>573</v>
       </c>
-      <c r="B74" s="17" t="s">
+      <c r="B74" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C74" s="18" t="s">
+      <c r="C74" s="16" t="s">
         <v>574</v>
       </c>
-      <c r="D74" s="18" t="s">
+      <c r="D74" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E74" s="18" t="s">
+      <c r="E74" s="16" t="s">
         <v>575</v>
       </c>
-      <c r="F74" s="18" t="s">
+      <c r="F74" s="16" t="s">
         <v>576</v>
       </c>
-      <c r="G74" s="17" t="s">
+      <c r="G74" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H74" s="18" t="s">
+      <c r="H74" s="16" t="s">
         <v>577</v>
       </c>
-      <c r="I74" s="18" t="s">
+      <c r="I74" s="16" t="s">
         <v>578</v>
       </c>
-      <c r="J74" s="18" t="s">
+      <c r="J74" s="16" t="s">
         <v>579</v>
       </c>
-      <c r="K74" s="18"/>
-      <c r="L74" s="17"/>
-      <c r="M74" s="18"/>
-      <c r="N74" s="18"/>
+      <c r="K74" s="16"/>
+      <c r="L74" s="15"/>
+      <c r="M74" s="16"/>
+      <c r="N74" s="16"/>
     </row>
     <row r="75" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A75" s="17" t="s">
+      <c r="A75" s="15" t="s">
         <v>580</v>
       </c>
-      <c r="B75" s="17" t="s">
+      <c r="B75" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C75" s="18" t="s">
+      <c r="C75" s="16" t="s">
         <v>581</v>
       </c>
-      <c r="D75" s="18" t="s">
+      <c r="D75" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E75" s="18" t="s">
+      <c r="E75" s="16" t="s">
         <v>582</v>
       </c>
-      <c r="F75" s="18" t="s">
+      <c r="F75" s="16" t="s">
         <v>583</v>
       </c>
-      <c r="G75" s="17" t="s">
+      <c r="G75" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="H75" s="18" t="s">
+      <c r="H75" s="16" t="s">
         <v>584</v>
       </c>
-      <c r="I75" s="18" t="s">
+      <c r="I75" s="16" t="s">
         <v>585</v>
       </c>
-      <c r="J75" s="18" t="s">
+      <c r="J75" s="16" t="s">
         <v>586</v>
       </c>
-      <c r="K75" s="18"/>
-      <c r="L75" s="17"/>
-      <c r="M75" s="18"/>
-      <c r="N75" s="18"/>
+      <c r="K75" s="16"/>
+      <c r="L75" s="15"/>
+      <c r="M75" s="16"/>
+      <c r="N75" s="16"/>
     </row>
     <row r="76" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A76" s="17" t="s">
+      <c r="A76" s="15" t="s">
         <v>587</v>
       </c>
-      <c r="B76" s="17" t="s">
+      <c r="B76" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C76" s="18" t="s">
+      <c r="C76" s="16" t="s">
         <v>588</v>
       </c>
-      <c r="D76" s="18" t="s">
+      <c r="D76" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E76" s="18" t="s">
+      <c r="E76" s="16" t="s">
         <v>589</v>
       </c>
-      <c r="F76" s="18" t="s">
+      <c r="F76" s="16" t="s">
         <v>590</v>
       </c>
-      <c r="G76" s="17" t="s">
+      <c r="G76" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="H76" s="18" t="s">
+      <c r="H76" s="16" t="s">
         <v>591</v>
       </c>
-      <c r="I76" s="18" t="s">
+      <c r="I76" s="16" t="s">
         <v>592</v>
       </c>
-      <c r="J76" s="18" t="s">
+      <c r="J76" s="16" t="s">
         <v>593</v>
       </c>
-      <c r="K76" s="18"/>
-      <c r="L76" s="17"/>
-      <c r="M76" s="18"/>
-      <c r="N76" s="18"/>
+      <c r="K76" s="16"/>
+      <c r="L76" s="15"/>
+      <c r="M76" s="16"/>
+      <c r="N76" s="16"/>
     </row>
     <row r="77" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A77" s="17" t="s">
+      <c r="A77" s="15" t="s">
         <v>594</v>
       </c>
-      <c r="B77" s="17" t="s">
+      <c r="B77" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C77" s="18" t="s">
+      <c r="C77" s="16" t="s">
         <v>595</v>
       </c>
-      <c r="D77" s="18" t="s">
+      <c r="D77" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E77" s="18" t="s">
+      <c r="E77" s="16" t="s">
         <v>596</v>
       </c>
-      <c r="F77" s="18" t="s">
+      <c r="F77" s="16" t="s">
         <v>597</v>
       </c>
-      <c r="G77" s="17" t="s">
+      <c r="G77" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H77" s="18" t="s">
+      <c r="H77" s="16" t="s">
         <v>598</v>
       </c>
-      <c r="I77" s="18" t="s">
+      <c r="I77" s="16" t="s">
         <v>599</v>
       </c>
-      <c r="J77" s="18" t="s">
+      <c r="J77" s="16" t="s">
         <v>600</v>
       </c>
-      <c r="K77" s="18"/>
-      <c r="L77" s="17"/>
-      <c r="M77" s="18"/>
-      <c r="N77" s="18"/>
+      <c r="K77" s="16"/>
+      <c r="L77" s="15"/>
+      <c r="M77" s="16"/>
+      <c r="N77" s="16"/>
     </row>
     <row r="78" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A78" s="17" t="s">
+      <c r="A78" s="15" t="s">
         <v>601</v>
       </c>
-      <c r="B78" s="17" t="s">
+      <c r="B78" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C78" s="18" t="s">
+      <c r="C78" s="16" t="s">
         <v>602</v>
       </c>
-      <c r="D78" s="18" t="s">
+      <c r="D78" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E78" s="18" t="s">
+      <c r="E78" s="16" t="s">
         <v>603</v>
       </c>
-      <c r="F78" s="18" t="s">
+      <c r="F78" s="16" t="s">
         <v>604</v>
       </c>
-      <c r="G78" s="17" t="s">
+      <c r="G78" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H78" s="18" t="s">
+      <c r="H78" s="16" t="s">
         <v>605</v>
       </c>
-      <c r="I78" s="18" t="s">
+      <c r="I78" s="16" t="s">
         <v>606</v>
       </c>
-      <c r="J78" s="18" t="s">
+      <c r="J78" s="16" t="s">
         <v>607</v>
       </c>
-      <c r="K78" s="18"/>
-      <c r="L78" s="17"/>
-      <c r="M78" s="18"/>
-      <c r="N78" s="18"/>
+      <c r="K78" s="16"/>
+      <c r="L78" s="15"/>
+      <c r="M78" s="16"/>
+      <c r="N78" s="16"/>
     </row>
     <row r="79" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A79" s="17" t="s">
+      <c r="A79" s="15" t="s">
         <v>608</v>
       </c>
-      <c r="B79" s="17" t="s">
+      <c r="B79" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="C79" s="18" t="s">
+      <c r="C79" s="16" t="s">
         <v>609</v>
       </c>
-      <c r="D79" s="18" t="s">
+      <c r="D79" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E79" s="18" t="s">
+      <c r="E79" s="16" t="s">
         <v>610</v>
       </c>
-      <c r="F79" s="18" t="s">
+      <c r="F79" s="16" t="s">
         <v>611</v>
       </c>
-      <c r="G79" s="17" t="s">
+      <c r="G79" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="H79" s="18" t="s">
+      <c r="H79" s="16" t="s">
         <v>612</v>
       </c>
-      <c r="I79" s="18" t="s">
+      <c r="I79" s="16" t="s">
         <v>613</v>
       </c>
-      <c r="J79" s="18" t="s">
+      <c r="J79" s="16" t="s">
         <v>614</v>
       </c>
-      <c r="K79" s="18"/>
-      <c r="L79" s="17"/>
-      <c r="M79" s="18"/>
-      <c r="N79" s="18"/>
+      <c r="K79" s="16"/>
+      <c r="L79" s="15"/>
+      <c r="M79" s="16"/>
+      <c r="N79" s="16"/>
     </row>
     <row r="80" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A80" s="17" t="s">
+      <c r="A80" s="15" t="s">
         <v>615</v>
       </c>
-      <c r="B80" s="17" t="s">
+      <c r="B80" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C80" s="18" t="s">
+      <c r="C80" s="16" t="s">
         <v>616</v>
       </c>
-      <c r="D80" s="18" t="s">
+      <c r="D80" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="E80" s="18" t="s">
+      <c r="E80" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F80" s="18" t="s">
+      <c r="F80" s="16" t="s">
         <v>617</v>
       </c>
-      <c r="G80" s="17" t="s">
+      <c r="G80" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H80" s="18" t="s">
+      <c r="H80" s="16" t="s">
         <v>618</v>
       </c>
-      <c r="I80" s="18" t="s">
+      <c r="I80" s="16" t="s">
         <v>619</v>
       </c>
-      <c r="J80" s="18" t="s">
+      <c r="J80" s="16" t="s">
         <v>620</v>
       </c>
-      <c r="K80" s="18"/>
-      <c r="L80" s="17"/>
-      <c r="M80" s="18"/>
-      <c r="N80" s="18"/>
+      <c r="K80" s="16"/>
+      <c r="L80" s="15"/>
+      <c r="M80" s="16"/>
+      <c r="N80" s="16"/>
     </row>
     <row r="81" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A81" s="17" t="s">
+      <c r="A81" s="15" t="s">
         <v>621</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B81" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C81" s="18" t="s">
+      <c r="C81" s="16" t="s">
         <v>622</v>
       </c>
-      <c r="D81" s="18" t="s">
+      <c r="D81" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E81" s="18" t="s">
+      <c r="E81" s="16" t="s">
         <v>623</v>
       </c>
-      <c r="F81" s="18" t="s">
+      <c r="F81" s="16" t="s">
         <v>624</v>
       </c>
-      <c r="G81" s="17" t="s">
+      <c r="G81" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H81" s="18" t="s">
+      <c r="H81" s="16" t="s">
         <v>538</v>
       </c>
-      <c r="I81" s="18" t="s">
+      <c r="I81" s="16" t="s">
         <v>625</v>
       </c>
-      <c r="J81" s="18" t="s">
+      <c r="J81" s="16" t="s">
         <v>626</v>
       </c>
-      <c r="K81" s="18"/>
-      <c r="L81" s="17"/>
-      <c r="M81" s="18"/>
-      <c r="N81" s="18"/>
+      <c r="K81" s="16"/>
+      <c r="L81" s="15"/>
+      <c r="M81" s="16"/>
+      <c r="N81" s="16"/>
     </row>
     <row r="82" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A82" s="17" t="s">
+      <c r="A82" s="15" t="s">
         <v>627</v>
       </c>
-      <c r="B82" s="17" t="s">
+      <c r="B82" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C82" s="18" t="s">
+      <c r="C82" s="16" t="s">
         <v>628</v>
       </c>
-      <c r="D82" s="18" t="s">
+      <c r="D82" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="E82" s="18" t="s">
+      <c r="E82" s="16" t="s">
         <v>629</v>
       </c>
-      <c r="F82" s="18" t="s">
+      <c r="F82" s="16" t="s">
         <v>630</v>
       </c>
-      <c r="G82" s="17" t="s">
+      <c r="G82" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="H82" s="18" t="s">
+      <c r="H82" s="16" t="s">
         <v>631</v>
       </c>
-      <c r="I82" s="18" t="s">
+      <c r="I82" s="16" t="s">
         <v>632</v>
       </c>
-      <c r="J82" s="18" t="s">
+      <c r="J82" s="16" t="s">
         <v>633</v>
       </c>
-      <c r="K82" s="18"/>
-      <c r="L82" s="17"/>
-      <c r="M82" s="18"/>
-      <c r="N82" s="18"/>
+      <c r="K82" s="16"/>
+      <c r="L82" s="15"/>
+      <c r="M82" s="16"/>
+      <c r="N82" s="16"/>
     </row>
     <row r="83" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A83" s="17" t="s">
+      <c r="A83" s="15" t="s">
         <v>634</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B83" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C83" s="18" t="s">
+      <c r="C83" s="16" t="s">
         <v>635</v>
       </c>
-      <c r="D83" s="18" t="s">
+      <c r="D83" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E83" s="18" t="s">
+      <c r="E83" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="F83" s="18" t="s">
+      <c r="F83" s="16" t="s">
         <v>637</v>
       </c>
-      <c r="G83" s="17" t="s">
+      <c r="G83" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H83" s="18" t="s">
+      <c r="H83" s="16" t="s">
         <v>631</v>
       </c>
-      <c r="I83" s="18" t="s">
+      <c r="I83" s="16" t="s">
         <v>638</v>
       </c>
-      <c r="J83" s="18" t="s">
+      <c r="J83" s="16" t="s">
         <v>639</v>
       </c>
-      <c r="K83" s="18"/>
-      <c r="L83" s="17"/>
-      <c r="M83" s="18"/>
-      <c r="N83" s="18"/>
+      <c r="K83" s="16"/>
+      <c r="L83" s="15"/>
+      <c r="M83" s="16"/>
+      <c r="N83" s="16"/>
     </row>
     <row r="84" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A84" s="17" t="s">
+      <c r="A84" s="15" t="s">
         <v>640</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B84" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C84" s="18" t="s">
+      <c r="C84" s="16" t="s">
         <v>641</v>
       </c>
-      <c r="D84" s="18" t="s">
+      <c r="D84" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E84" s="18" t="s">
+      <c r="E84" s="16" t="s">
         <v>610</v>
       </c>
-      <c r="F84" s="18" t="s">
+      <c r="F84" s="16" t="s">
         <v>642</v>
       </c>
-      <c r="G84" s="17" t="s">
+      <c r="G84" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H84" s="18" t="s">
+      <c r="H84" s="16" t="s">
         <v>643</v>
       </c>
-      <c r="I84" s="18" t="s">
+      <c r="I84" s="16" t="s">
         <v>644</v>
       </c>
-      <c r="J84" s="18" t="s">
+      <c r="J84" s="16" t="s">
         <v>645</v>
       </c>
-      <c r="K84" s="18"/>
-      <c r="L84" s="17"/>
-      <c r="M84" s="18"/>
-      <c r="N84" s="18"/>
+      <c r="K84" s="16"/>
+      <c r="L84" s="15"/>
+      <c r="M84" s="16"/>
+      <c r="N84" s="16"/>
     </row>
     <row r="85" spans="1:14" ht="102" x14ac:dyDescent="0.25">
-      <c r="A85" s="17" t="s">
+      <c r="A85" s="15" t="s">
         <v>646</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B85" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C85" s="18" t="s">
+      <c r="C85" s="16" t="s">
         <v>647</v>
       </c>
-      <c r="D85" s="18" t="s">
+      <c r="D85" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E85" s="18" t="s">
+      <c r="E85" s="16" t="s">
         <v>648</v>
       </c>
-      <c r="F85" s="18" t="s">
+      <c r="F85" s="16" t="s">
         <v>649</v>
       </c>
-      <c r="G85" s="17" t="s">
+      <c r="G85" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H85" s="18" t="s">
+      <c r="H85" s="16" t="s">
         <v>538</v>
       </c>
-      <c r="I85" s="18" t="s">
+      <c r="I85" s="16" t="s">
         <v>650</v>
       </c>
-      <c r="J85" s="18" t="s">
+      <c r="J85" s="16" t="s">
         <v>651</v>
       </c>
-      <c r="K85" s="18"/>
-      <c r="L85" s="17"/>
-      <c r="M85" s="18"/>
-      <c r="N85" s="18"/>
+      <c r="K85" s="16"/>
+      <c r="L85" s="15"/>
+      <c r="M85" s="16"/>
+      <c r="N85" s="16"/>
     </row>
     <row r="86" spans="1:14" ht="102" x14ac:dyDescent="0.25">
-      <c r="A86" s="17" t="s">
+      <c r="A86" s="15" t="s">
         <v>652</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B86" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C86" s="18" t="s">
+      <c r="C86" s="16" t="s">
         <v>653</v>
       </c>
-      <c r="D86" s="18" t="s">
+      <c r="D86" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="E86" s="18" t="s">
+      <c r="E86" s="16" t="s">
         <v>654</v>
       </c>
-      <c r="F86" s="18" t="s">
+      <c r="F86" s="16" t="s">
         <v>655</v>
       </c>
-      <c r="G86" s="17" t="s">
+      <c r="G86" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H86" s="18" t="s">
+      <c r="H86" s="16" t="s">
         <v>538</v>
       </c>
-      <c r="I86" s="18" t="s">
+      <c r="I86" s="16" t="s">
         <v>656</v>
       </c>
-      <c r="J86" s="18" t="s">
+      <c r="J86" s="16" t="s">
         <v>657</v>
       </c>
-      <c r="K86" s="18"/>
-      <c r="L86" s="17"/>
-      <c r="M86" s="18"/>
-      <c r="N86" s="18"/>
+      <c r="K86" s="16"/>
+      <c r="L86" s="15"/>
+      <c r="M86" s="16"/>
+      <c r="N86" s="16"/>
     </row>
     <row r="87" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A87" s="17" t="s">
+      <c r="A87" s="15" t="s">
         <v>658</v>
       </c>
-      <c r="B87" s="17" t="s">
+      <c r="B87" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C87" s="18" t="s">
+      <c r="C87" s="16" t="s">
         <v>659</v>
       </c>
-      <c r="D87" s="18" t="s">
+      <c r="D87" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E87" s="18" t="s">
+      <c r="E87" s="16" t="s">
         <v>660</v>
       </c>
-      <c r="F87" s="18" t="s">
+      <c r="F87" s="16" t="s">
         <v>661</v>
       </c>
-      <c r="G87" s="17" t="s">
+      <c r="G87" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H87" s="18" t="s">
+      <c r="H87" s="16" t="s">
         <v>662</v>
       </c>
-      <c r="I87" s="18" t="s">
+      <c r="I87" s="16" t="s">
         <v>663</v>
       </c>
-      <c r="J87" s="18" t="s">
+      <c r="J87" s="16" t="s">
         <v>664</v>
       </c>
-      <c r="K87" s="18"/>
-      <c r="L87" s="17"/>
-      <c r="M87" s="18"/>
-      <c r="N87" s="18"/>
+      <c r="K87" s="16"/>
+      <c r="L87" s="15"/>
+      <c r="M87" s="16"/>
+      <c r="N87" s="16"/>
     </row>
     <row r="88" spans="1:14" ht="102" x14ac:dyDescent="0.25">
-      <c r="A88" s="17" t="s">
+      <c r="A88" s="15" t="s">
         <v>665</v>
       </c>
-      <c r="B88" s="17" t="s">
+      <c r="B88" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C88" s="18" t="s">
+      <c r="C88" s="16" t="s">
         <v>666</v>
       </c>
-      <c r="D88" s="18" t="s">
+      <c r="D88" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E88" s="18" t="s">
+      <c r="E88" s="16" t="s">
         <v>568</v>
       </c>
-      <c r="F88" s="18" t="s">
+      <c r="F88" s="16" t="s">
         <v>667</v>
       </c>
-      <c r="G88" s="17" t="s">
+      <c r="G88" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="H88" s="18" t="s">
+      <c r="H88" s="16" t="s">
         <v>668</v>
       </c>
-      <c r="I88" s="18" t="s">
+      <c r="I88" s="16" t="s">
         <v>669</v>
       </c>
-      <c r="J88" s="18" t="s">
+      <c r="J88" s="16" t="s">
         <v>670</v>
       </c>
-      <c r="K88" s="18"/>
-      <c r="L88" s="17"/>
-      <c r="M88" s="18"/>
-      <c r="N88" s="18"/>
+      <c r="K88" s="16"/>
+      <c r="L88" s="15"/>
+      <c r="M88" s="16"/>
+      <c r="N88" s="16"/>
     </row>
     <row r="89" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A89" s="17" t="s">
+      <c r="A89" s="15" t="s">
         <v>671</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="B89" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="C89" s="18" t="s">
+      <c r="C89" s="16" t="s">
         <v>672</v>
       </c>
-      <c r="D89" s="18" t="s">
+      <c r="D89" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E89" s="18" t="s">
+      <c r="E89" s="16" t="s">
         <v>673</v>
       </c>
-      <c r="F89" s="18" t="s">
+      <c r="F89" s="16" t="s">
         <v>674</v>
       </c>
-      <c r="G89" s="17" t="s">
+      <c r="G89" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="H89" s="18" t="s">
+      <c r="H89" s="16" t="s">
         <v>675</v>
       </c>
-      <c r="I89" s="18" t="s">
+      <c r="I89" s="16" t="s">
         <v>676</v>
       </c>
-      <c r="J89" s="18" t="s">
+      <c r="J89" s="16" t="s">
         <v>677</v>
       </c>
-      <c r="K89" s="18"/>
-      <c r="L89" s="17"/>
-      <c r="M89" s="18"/>
-      <c r="N89" s="18"/>
-    </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A90" s="19"/>
-    </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A91" s="19"/>
+      <c r="K89" s="16"/>
+      <c r="L89" s="15"/>
+      <c r="M89" s="16"/>
+      <c r="N89" s="16"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N65" xr:uid="{00000000-0009-0000-0000-000003000000}">
@@ -6248,29 +6183,7 @@
     </sortState>
   </autoFilter>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="L2:L65 L90:L395">
-    <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
-      <formula>"PASS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
-      <formula>"FAIL"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="10" operator="equal">
-      <formula>"Chưa chạy"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L66">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
-      <formula>"PASS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
-      <formula>"FAIL"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
-      <formula>"Chưa chạy"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L67:L89">
+  <conditionalFormatting sqref="L2:L395">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"PASS"</formula>
     </cfRule>
@@ -6325,6 +6238,8 @@
     <hyperlink ref="M62" r:id="rId27" xr:uid="{3AA3DDD4-7123-4057-8041-CF1B902A3E1C}"/>
     <hyperlink ref="M64" r:id="rId28" xr:uid="{9606907E-556D-4CCC-82F8-9F50D0A02BF1}"/>
     <hyperlink ref="M65" r:id="rId29" xr:uid="{06E98682-1678-4789-922C-833F9D2B116B}"/>
+    <hyperlink ref="M67" r:id="rId30" xr:uid="{EA70FFB8-7920-41C8-A0FA-18B4BE4C3BAD}"/>
+    <hyperlink ref="M68" r:id="rId31" xr:uid="{4E4579C3-CEB9-40D9-A997-8179236FB2AF}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6880,7 +6795,7 @@
       </c>
       <c r="E16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"PASS")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F16" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A16,'Test Case'!$L:$L,"FAIL")</f>
@@ -6899,7 +6814,7 @@
       </c>
       <c r="E17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"PASS")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"FAIL")</f>
@@ -7069,74 +6984,74 @@
       <c r="A31" s="3" t="s">
         <v>453</v>
       </c>
-      <c r="B31" s="15" t="str">
+      <c r="B31" s="17" t="str">
         <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
         <v>Đã chạy 38 / 64 TC; PASS 38; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="15"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="17"/>
     </row>
     <row r="32" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>454</v>
       </c>
-      <c r="B32" s="16"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16"/>
-      <c r="J32" s="16"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
+      <c r="J32" s="18"/>
     </row>
     <row r="33" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>455</v>
       </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
-      <c r="J33" s="16"/>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="18"/>
     </row>
     <row r="34" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>456</v>
       </c>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="16"/>
-      <c r="J34" s="16"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
+      <c r="J34" s="18"/>
     </row>
     <row r="35" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="B35" s="16"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
+      <c r="B35" s="18"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
+      <c r="J35" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Hoàn tất kiểm thử testcase TC-22-04
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24447F51-0FD0-4321-A778-A573BE4BAEB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E3E0E9-027F-47B3-8A86-68D84AF27B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,15 +31,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="680">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1129" uniqueCount="683">
   <si>
     <t>UC</t>
   </si>
@@ -1908,22 +1905,7 @@
     <t>TC-22-14</t>
   </si>
   <si>
-    <t>Tìm kiếm món ăn trong thực đơn bằng tiếng Việt không dấu (AF-3)</t>
-  </si>
-  <si>
     <t>Black-box theo UC Spec (AF-3)</t>
-  </si>
-  <si>
-    <t>UC22 AF-3; hàm boDau() trên giao diện quan-ly-menu.js</t>
-  </si>
-  <si>
-    <t>Đã đăng nhập chutquan01 (vai trò CHU_QUAN). Thực đơn có món "Trà đào", "Cà phê sữa", "Bạc xỉu".</t>
-  </si>
-  <si>
-    <t>Nhập vào ô "Tìm món": "tra dao", sau đó đổi thành "bac xiu"</t>
-  </si>
-  <si>
-    <t>Giao diện lọc món tức thì: gõ "tra dao" hiển thị món "Trà đào", gõ "bac xiu" hiển thị món "Bạc xỉu". Món không khớp bị ẩn. Khi xóa ô tìm kiếm thì bảng hiển thị lại đầy đủ thực đơn.</t>
   </si>
   <si>
     <t>TC-24-01</t>
@@ -2135,6 +2117,32 @@
   </si>
   <si>
     <t>KQ-test\TC-22-03.png</t>
+  </si>
+  <si>
+    <t>Kiểm tra giữ nguyên trạng thái món khi Chủ quán đã chủ động "Tắt bán"</t>
+  </si>
+  <si>
+    <t>Integration Testing (Business Logic Conflict)</t>
+  </si>
+  <si>
+    <t>UC18 &amp; UC22; POST /api/inventory/:id/restock; KhoHangRepository.js (hàm dongBoTrangThaiMonAn)</t>
+  </si>
+  <si>
+    <t>- Món "Cà phê đen" có công thức gồm nguyên liệu "Hạt cà phê Robusta" (tồn kho &gt; 0).
+- Chủ quán vào trang Quản lý menu, bấm "Tắt bán" món "Cà phê đen" (chuyển sang TAM_HET do quán tạm ngưng phục vụ).</t>
+  </si>
+  <si>
+    <t>1. Barista thực hiện nhập thêm kho cho nguyên liệu "Hạt cà phê Robusta": POST /api/inventory/nl-01/restock với { soLuong: 10 }.
+2. Kiểm tra lại trạng thái của món "Cà phê đen" trong bảng mon_an và trên menu Phục vụ.</t>
+  </si>
+  <si>
+    <t>Món "Cà phê đen" vẫn phải giữ nguyên trạng thái TAM_HET vì Chủ quán đã chủ động tắt bán.</t>
+  </si>
+  <si>
+    <t>Giao diện chỉ cho phép người dùng nhập giới hạn 100 ký tự không cho nhập hơn.</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-22-04.png</t>
   </si>
 </sst>
 </file>
@@ -2144,13 +2152,20 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -2205,8 +2220,25 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2237,6 +2269,12 @@
         <bgColor rgb="FFED7D31"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -2262,66 +2300,80 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{5FAD4E6F-4F20-44E1-AD8C-2B89C9EDDB5E}"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
@@ -2688,7 +2740,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>120</v>
       </c>
@@ -3828,7 +3880,7 @@
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>246</v>
       </c>
@@ -4700,7 +4752,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>373</v>
       </c>
@@ -4986,7 +5038,7 @@
       </c>
       <c r="N58" s="1"/>
     </row>
-    <row r="59" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
         <v>66</v>
       </c>
@@ -5074,7 +5126,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>80</v>
       </c>
@@ -5374,7 +5426,7 @@
         <v>459</v>
       </c>
       <c r="M67" s="14" t="s">
-        <v>678</v>
+        <v>673</v>
       </c>
       <c r="N67" s="16"/>
     </row>
@@ -5416,7 +5468,7 @@
         <v>459</v>
       </c>
       <c r="M68" s="14" t="s">
-        <v>679</v>
+        <v>674</v>
       </c>
       <c r="N68" s="16"/>
     </row>
@@ -5451,9 +5503,15 @@
       <c r="J69" s="16" t="s">
         <v>546</v>
       </c>
-      <c r="K69" s="16"/>
-      <c r="L69" s="15"/>
-      <c r="M69" s="16"/>
+      <c r="K69" s="16" t="s">
+        <v>681</v>
+      </c>
+      <c r="L69" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="M69" s="14" t="s">
+        <v>682</v>
+      </c>
       <c r="N69" s="16"/>
     </row>
     <row r="70" spans="1:14" ht="51" x14ac:dyDescent="0.25">
@@ -5492,7 +5550,7 @@
       <c r="M70" s="16"/>
       <c r="N70" s="16"/>
     </row>
-    <row r="71" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A71" s="15" t="s">
         <v>554</v>
       </c>
@@ -5780,51 +5838,51 @@
       <c r="M78" s="16"/>
       <c r="N78" s="16"/>
     </row>
-    <row r="79" spans="1:14" ht="51" x14ac:dyDescent="0.25">
-      <c r="A79" s="15" t="s">
+    <row r="79" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A79" s="21" t="s">
         <v>608</v>
       </c>
-      <c r="B79" s="15" t="s">
+      <c r="B79" s="19" t="s">
         <v>518</v>
       </c>
-      <c r="C79" s="16" t="s">
-        <v>609</v>
-      </c>
-      <c r="D79" s="16" t="s">
+      <c r="C79" s="20" t="s">
+        <v>675</v>
+      </c>
+      <c r="D79" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="E79" s="16" t="s">
-        <v>610</v>
-      </c>
-      <c r="F79" s="16" t="s">
-        <v>611</v>
-      </c>
-      <c r="G79" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="H79" s="16" t="s">
-        <v>612</v>
-      </c>
-      <c r="I79" s="16" t="s">
-        <v>613</v>
-      </c>
-      <c r="J79" s="16" t="s">
-        <v>614</v>
-      </c>
-      <c r="K79" s="16"/>
-      <c r="L79" s="15"/>
-      <c r="M79" s="16"/>
-      <c r="N79" s="16"/>
+      <c r="E79" s="20" t="s">
+        <v>676</v>
+      </c>
+      <c r="F79" s="20" t="s">
+        <v>677</v>
+      </c>
+      <c r="G79" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="H79" s="20" t="s">
+        <v>678</v>
+      </c>
+      <c r="I79" s="20" t="s">
+        <v>679</v>
+      </c>
+      <c r="J79" s="20" t="s">
+        <v>680</v>
+      </c>
+      <c r="K79" s="20"/>
+      <c r="L79" s="22"/>
+      <c r="M79" s="20"/>
+      <c r="N79" s="20"/>
     </row>
     <row r="80" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A80" s="15" t="s">
-        <v>615</v>
+        <v>610</v>
       </c>
       <c r="B80" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C80" s="16" t="s">
-        <v>616</v>
+        <v>611</v>
       </c>
       <c r="D80" s="16" t="s">
         <v>37</v>
@@ -5833,19 +5891,19 @@
         <v>38</v>
       </c>
       <c r="F80" s="16" t="s">
-        <v>617</v>
+        <v>612</v>
       </c>
       <c r="G80" s="15" t="s">
         <v>40</v>
       </c>
       <c r="H80" s="16" t="s">
-        <v>618</v>
+        <v>613</v>
       </c>
       <c r="I80" s="16" t="s">
-        <v>619</v>
+        <v>614</v>
       </c>
       <c r="J80" s="16" t="s">
-        <v>620</v>
+        <v>615</v>
       </c>
       <c r="K80" s="16"/>
       <c r="L80" s="15"/>
@@ -5854,22 +5912,22 @@
     </row>
     <row r="81" spans="1:14" ht="51" x14ac:dyDescent="0.25">
       <c r="A81" s="15" t="s">
-        <v>621</v>
+        <v>616</v>
       </c>
       <c r="B81" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C81" s="16" t="s">
-        <v>622</v>
+        <v>617</v>
       </c>
       <c r="D81" s="16" t="s">
         <v>20</v>
       </c>
       <c r="E81" s="16" t="s">
-        <v>623</v>
+        <v>618</v>
       </c>
       <c r="F81" s="16" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
       <c r="G81" s="15" t="s">
         <v>40</v>
@@ -5878,10 +5936,10 @@
         <v>538</v>
       </c>
       <c r="I81" s="16" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="J81" s="16" t="s">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="K81" s="16"/>
       <c r="L81" s="15"/>
@@ -5890,34 +5948,34 @@
     </row>
     <row r="82" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A82" s="15" t="s">
-        <v>627</v>
+        <v>622</v>
       </c>
       <c r="B82" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C82" s="16" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="D82" s="16" t="s">
         <v>74</v>
       </c>
       <c r="E82" s="16" t="s">
-        <v>629</v>
+        <v>624</v>
       </c>
       <c r="F82" s="16" t="s">
-        <v>630</v>
+        <v>625</v>
       </c>
       <c r="G82" s="15" t="s">
         <v>63</v>
       </c>
       <c r="H82" s="16" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="I82" s="16" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="J82" s="16" t="s">
-        <v>633</v>
+        <v>628</v>
       </c>
       <c r="K82" s="16"/>
       <c r="L82" s="15"/>
@@ -5926,34 +5984,34 @@
     </row>
     <row r="83" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="B83" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C83" s="16" t="s">
-        <v>635</v>
+        <v>630</v>
       </c>
       <c r="D83" s="16" t="s">
         <v>20</v>
       </c>
       <c r="E83" s="16" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="F83" s="16" t="s">
-        <v>637</v>
+        <v>632</v>
       </c>
       <c r="G83" s="15" t="s">
         <v>40</v>
       </c>
       <c r="H83" s="16" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="I83" s="16" t="s">
-        <v>638</v>
+        <v>633</v>
       </c>
       <c r="J83" s="16" t="s">
-        <v>639</v>
+        <v>634</v>
       </c>
       <c r="K83" s="16"/>
       <c r="L83" s="15"/>
@@ -5962,34 +6020,34 @@
     </row>
     <row r="84" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
-        <v>640</v>
+        <v>635</v>
       </c>
       <c r="B84" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C84" s="16" t="s">
-        <v>641</v>
+        <v>636</v>
       </c>
       <c r="D84" s="16" t="s">
         <v>20</v>
       </c>
       <c r="E84" s="16" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F84" s="16" t="s">
-        <v>642</v>
+        <v>637</v>
       </c>
       <c r="G84" s="15" t="s">
         <v>40</v>
       </c>
       <c r="H84" s="16" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
       <c r="I84" s="16" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
       <c r="J84" s="16" t="s">
-        <v>645</v>
+        <v>640</v>
       </c>
       <c r="K84" s="16"/>
       <c r="L84" s="15"/>
@@ -5998,22 +6056,22 @@
     </row>
     <row r="85" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A85" s="15" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
       <c r="B85" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C85" s="16" t="s">
-        <v>647</v>
+        <v>642</v>
       </c>
       <c r="D85" s="16" t="s">
         <v>54</v>
       </c>
       <c r="E85" s="16" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
       <c r="F85" s="16" t="s">
-        <v>649</v>
+        <v>644</v>
       </c>
       <c r="G85" s="15" t="s">
         <v>40</v>
@@ -6022,10 +6080,10 @@
         <v>538</v>
       </c>
       <c r="I85" s="16" t="s">
-        <v>650</v>
+        <v>645</v>
       </c>
       <c r="J85" s="16" t="s">
-        <v>651</v>
+        <v>646</v>
       </c>
       <c r="K85" s="16"/>
       <c r="L85" s="15"/>
@@ -6034,22 +6092,22 @@
     </row>
     <row r="86" spans="1:14" ht="102" x14ac:dyDescent="0.25">
       <c r="A86" s="15" t="s">
-        <v>652</v>
+        <v>647</v>
       </c>
       <c r="B86" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C86" s="16" t="s">
-        <v>653</v>
+        <v>648</v>
       </c>
       <c r="D86" s="16" t="s">
         <v>74</v>
       </c>
       <c r="E86" s="16" t="s">
-        <v>654</v>
+        <v>649</v>
       </c>
       <c r="F86" s="16" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
       <c r="G86" s="15" t="s">
         <v>40</v>
@@ -6058,10 +6116,10 @@
         <v>538</v>
       </c>
       <c r="I86" s="16" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
       <c r="J86" s="16" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="K86" s="16"/>
       <c r="L86" s="15"/>
@@ -6070,49 +6128,49 @@
     </row>
     <row r="87" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A87" s="15" t="s">
-        <v>658</v>
+        <v>653</v>
       </c>
       <c r="B87" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C87" s="16" t="s">
-        <v>659</v>
+        <v>654</v>
       </c>
       <c r="D87" s="16" t="s">
         <v>54</v>
       </c>
       <c r="E87" s="16" t="s">
-        <v>660</v>
+        <v>655</v>
       </c>
       <c r="F87" s="16" t="s">
-        <v>661</v>
+        <v>656</v>
       </c>
       <c r="G87" s="15" t="s">
         <v>40</v>
       </c>
       <c r="H87" s="16" t="s">
-        <v>662</v>
+        <v>657</v>
       </c>
       <c r="I87" s="16" t="s">
-        <v>663</v>
+        <v>658</v>
       </c>
       <c r="J87" s="16" t="s">
-        <v>664</v>
+        <v>659</v>
       </c>
       <c r="K87" s="16"/>
       <c r="L87" s="15"/>
       <c r="M87" s="16"/>
       <c r="N87" s="16"/>
     </row>
-    <row r="88" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A88" s="15" t="s">
-        <v>665</v>
+        <v>660</v>
       </c>
       <c r="B88" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C88" s="16" t="s">
-        <v>666</v>
+        <v>661</v>
       </c>
       <c r="D88" s="16" t="s">
         <v>20</v>
@@ -6121,19 +6179,19 @@
         <v>568</v>
       </c>
       <c r="F88" s="16" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="G88" s="15" t="s">
         <v>63</v>
       </c>
       <c r="H88" s="16" t="s">
-        <v>668</v>
+        <v>663</v>
       </c>
       <c r="I88" s="16" t="s">
-        <v>669</v>
+        <v>664</v>
       </c>
       <c r="J88" s="16" t="s">
-        <v>670</v>
+        <v>665</v>
       </c>
       <c r="K88" s="16"/>
       <c r="L88" s="15"/>
@@ -6142,34 +6200,34 @@
     </row>
     <row r="89" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A89" s="15" t="s">
-        <v>671</v>
+        <v>666</v>
       </c>
       <c r="B89" s="15" t="s">
         <v>519</v>
       </c>
       <c r="C89" s="16" t="s">
-        <v>672</v>
+        <v>667</v>
       </c>
       <c r="D89" s="16" t="s">
         <v>54</v>
       </c>
       <c r="E89" s="16" t="s">
-        <v>673</v>
+        <v>668</v>
       </c>
       <c r="F89" s="16" t="s">
-        <v>674</v>
+        <v>669</v>
       </c>
       <c r="G89" s="15" t="s">
         <v>63</v>
       </c>
       <c r="H89" s="16" t="s">
-        <v>675</v>
+        <v>670</v>
       </c>
       <c r="I89" s="16" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="J89" s="16" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="K89" s="16"/>
       <c r="L89" s="15"/>
@@ -6182,7 +6240,7 @@
       <sortCondition ref="A1:A65"/>
     </sortState>
   </autoFilter>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="L2:L395">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"PASS"</formula>
@@ -6240,6 +6298,7 @@
     <hyperlink ref="M65" r:id="rId29" xr:uid="{06E98682-1678-4789-922C-833F9D2B116B}"/>
     <hyperlink ref="M67" r:id="rId30" xr:uid="{EA70FFB8-7920-41C8-A0FA-18B4BE4C3BAD}"/>
     <hyperlink ref="M68" r:id="rId31" xr:uid="{4E4579C3-CEB9-40D9-A997-8179236FB2AF}"/>
+    <hyperlink ref="M69" r:id="rId32" xr:uid="{84857B41-0C15-485C-A885-F39B7D4FBC60}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6833,7 +6892,7 @@
       </c>
       <c r="E18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"PASS")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"FAIL")</f>

</xml_diff>

<commit_message>
Hoàn thành kiểm thử testcase TC-22-05
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E3E0E9-027F-47B3-8A86-68D84AF27B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B84A02-9499-4C55-A3CD-DE734DE10976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1129" uniqueCount="683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="684">
   <si>
     <t>UC</t>
   </si>
@@ -2143,6 +2143,9 @@
   </si>
   <si>
     <t>KQ-test\TC-22-04.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-22-05.png</t>
   </si>
 </sst>
 </file>
@@ -2172,34 +2175,34 @@
       <sz val="14"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -2224,12 +2227,14 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF9C0006"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2351,12 +2356,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2368,6 +2367,12 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -5545,9 +5550,15 @@
       <c r="J70" s="16" t="s">
         <v>553</v>
       </c>
-      <c r="K70" s="16"/>
-      <c r="L70" s="15"/>
-      <c r="M70" s="16"/>
+      <c r="K70" s="16" t="s">
+        <v>553</v>
+      </c>
+      <c r="L70" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="M70" s="14" t="s">
+        <v>683</v>
+      </c>
       <c r="N70" s="16"/>
     </row>
     <row r="71" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
@@ -5839,40 +5850,40 @@
       <c r="N78" s="16"/>
     </row>
     <row r="79" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A79" s="21" t="s">
+      <c r="A79" s="19" t="s">
         <v>608</v>
       </c>
-      <c r="B79" s="19" t="s">
+      <c r="B79" s="17" t="s">
         <v>518</v>
       </c>
-      <c r="C79" s="20" t="s">
+      <c r="C79" s="18" t="s">
         <v>675</v>
       </c>
-      <c r="D79" s="20" t="s">
+      <c r="D79" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E79" s="20" t="s">
+      <c r="E79" s="18" t="s">
         <v>676</v>
       </c>
-      <c r="F79" s="20" t="s">
+      <c r="F79" s="18" t="s">
         <v>677</v>
       </c>
-      <c r="G79" s="19" t="s">
+      <c r="G79" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="H79" s="20" t="s">
+      <c r="H79" s="18" t="s">
         <v>678</v>
       </c>
-      <c r="I79" s="20" t="s">
+      <c r="I79" s="18" t="s">
         <v>679</v>
       </c>
-      <c r="J79" s="20" t="s">
+      <c r="J79" s="18" t="s">
         <v>680</v>
       </c>
-      <c r="K79" s="20"/>
-      <c r="L79" s="22"/>
-      <c r="M79" s="20"/>
-      <c r="N79" s="20"/>
+      <c r="K79" s="18"/>
+      <c r="L79" s="20"/>
+      <c r="M79" s="18"/>
+      <c r="N79" s="18"/>
     </row>
     <row r="80" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A80" s="15" t="s">
@@ -6299,6 +6310,7 @@
     <hyperlink ref="M67" r:id="rId30" xr:uid="{EA70FFB8-7920-41C8-A0FA-18B4BE4C3BAD}"/>
     <hyperlink ref="M68" r:id="rId31" xr:uid="{4E4579C3-CEB9-40D9-A997-8179236FB2AF}"/>
     <hyperlink ref="M69" r:id="rId32" xr:uid="{84857B41-0C15-485C-A885-F39B7D4FBC60}"/>
+    <hyperlink ref="M70" r:id="rId33" xr:uid="{7E380299-08A2-47C2-B4E7-DEBC1C8EA036}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6911,7 +6923,7 @@
       </c>
       <c r="E19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"PASS")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"FAIL")</f>
@@ -7043,74 +7055,74 @@
       <c r="A31" s="3" t="s">
         <v>453</v>
       </c>
-      <c r="B31" s="17" t="str">
+      <c r="B31" s="21" t="str">
         <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
         <v>Đã chạy 38 / 64 TC; PASS 38; FAIL 0; tỉ lệ pass 100.0%</v>
       </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
     </row>
     <row r="32" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>454</v>
       </c>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="22"/>
     </row>
     <row r="33" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>455</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
-      <c r="J33" s="18"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="22"/>
+      <c r="J33" s="22"/>
     </row>
     <row r="34" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>456</v>
       </c>
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="18"/>
-      <c r="H34" s="18"/>
-      <c r="I34" s="18"/>
-      <c r="J34" s="18"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="I34" s="22"/>
+      <c r="J34" s="22"/>
     </row>
     <row r="35" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="B35" s="18"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
-      <c r="J35" s="18"/>
+      <c r="B35" s="22"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="I35" s="22"/>
+      <c r="J35" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Hoàn tất kiểm thử testcase TC-22-06
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B84A02-9499-4C55-A3CD-DE734DE10976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778DA7DB-01EF-4A0E-A33A-C66F5D7850EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="684">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="685">
   <si>
     <t>UC</t>
   </si>
@@ -2146,6 +2146,9 @@
   </si>
   <si>
     <t>KQ-test\TC-22-05.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-22-06.png</t>
   </si>
 </sst>
 </file>
@@ -5592,9 +5595,15 @@
       <c r="J71" s="16" t="s">
         <v>559</v>
       </c>
-      <c r="K71" s="16"/>
-      <c r="L71" s="15"/>
-      <c r="M71" s="16"/>
+      <c r="K71" s="16" t="s">
+        <v>559</v>
+      </c>
+      <c r="L71" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="M71" s="14" t="s">
+        <v>684</v>
+      </c>
       <c r="N71" s="16"/>
     </row>
     <row r="72" spans="1:14" ht="89.25" x14ac:dyDescent="0.25">
@@ -6311,6 +6320,7 @@
     <hyperlink ref="M68" r:id="rId31" xr:uid="{4E4579C3-CEB9-40D9-A997-8179236FB2AF}"/>
     <hyperlink ref="M69" r:id="rId32" xr:uid="{84857B41-0C15-485C-A885-F39B7D4FBC60}"/>
     <hyperlink ref="M70" r:id="rId33" xr:uid="{7E380299-08A2-47C2-B4E7-DEBC1C8EA036}"/>
+    <hyperlink ref="M71" r:id="rId34" xr:uid="{4A9FFBFF-EF0A-42D6-99E7-396BFFC02102}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6904,7 +6914,7 @@
       </c>
       <c r="E18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"PASS")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F18" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A18,'Test Case'!$L:$L,"FAIL")</f>

</xml_diff>

<commit_message>
hoàn thành kiểm thử TC-22-07
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778DA7DB-01EF-4A0E-A33A-C66F5D7850EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9014F1C4-2A17-4826-8388-2ED5D5948132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="685">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="685">
   <si>
     <t>UC</t>
   </si>
@@ -5637,8 +5637,12 @@
       <c r="J72" s="16" t="s">
         <v>565</v>
       </c>
-      <c r="K72" s="16"/>
-      <c r="L72" s="15"/>
+      <c r="K72" s="16" t="s">
+        <v>565</v>
+      </c>
+      <c r="L72" s="15" t="s">
+        <v>459</v>
+      </c>
       <c r="M72" s="16"/>
       <c r="N72" s="16"/>
     </row>
@@ -6895,7 +6899,7 @@
       </c>
       <c r="E17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"PASS")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"FAIL")</f>

</xml_diff>

<commit_message>
Hoàn thành kiểm thử TC-22-08
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34173532-182C-42B7-82DA-65086EF86AB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD721C06-4026-4C64-8CCE-EDFB1DA62D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1140" uniqueCount="686">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="687">
   <si>
     <t>UC</t>
   </si>
@@ -2152,6 +2152,9 @@
   </si>
   <si>
     <t>KQ-test\TC-22-08.png</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-22-09.png</t>
   </si>
 </sst>
 </file>
@@ -5722,9 +5725,15 @@
       <c r="J74" s="16" t="s">
         <v>579</v>
       </c>
-      <c r="K74" s="16"/>
-      <c r="L74" s="15"/>
-      <c r="M74" s="16"/>
+      <c r="K74" s="16" t="s">
+        <v>579</v>
+      </c>
+      <c r="L74" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="M74" s="14" t="s">
+        <v>686</v>
+      </c>
       <c r="N74" s="16"/>
     </row>
     <row r="75" spans="1:14" ht="51" x14ac:dyDescent="0.25">
@@ -6335,6 +6344,7 @@
     <hyperlink ref="M70" r:id="rId33" xr:uid="{7E380299-08A2-47C2-B4E7-DEBC1C8EA036}"/>
     <hyperlink ref="M71" r:id="rId34" xr:uid="{4A9FFBFF-EF0A-42D6-99E7-396BFFC02102}"/>
     <hyperlink ref="M73" r:id="rId35" xr:uid="{8122B6D1-AB2E-453D-ABBD-90F259A7ACE0}"/>
+    <hyperlink ref="M74" r:id="rId36" xr:uid="{7A37FDCC-E43E-42FA-8644-5B26D127DEC4}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6947,7 +6957,7 @@
       </c>
       <c r="E19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"PASS")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"FAIL")</f>

</xml_diff>

<commit_message>
(test): có bug ở TC-22-14
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5470D3-6258-4A1A-9070-52C061369865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9F45F49-5E1B-48F3-8204-4B1922BA647D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="690">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1157" uniqueCount="693">
   <si>
     <t>UC</t>
   </si>
@@ -2164,6 +2164,15 @@
   </si>
   <si>
     <t>KQ-test\TC-22-13.png</t>
+  </si>
+  <si>
+    <t>Món cà phê đen sau khi được nhập nguyên liệu thì tự động đổi qua trạng thái còn hàng.</t>
+  </si>
+  <si>
+    <t>fail</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-22-14.png</t>
   </si>
 </sst>
 </file>
@@ -2328,7 +2337,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2394,6 +2403,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -5945,9 +5960,15 @@
       <c r="J79" s="18" t="s">
         <v>680</v>
       </c>
-      <c r="K79" s="18"/>
-      <c r="L79" s="20"/>
-      <c r="M79" s="18"/>
+      <c r="K79" s="24" t="s">
+        <v>690</v>
+      </c>
+      <c r="L79" s="20" t="s">
+        <v>691</v>
+      </c>
+      <c r="M79" s="25" t="s">
+        <v>692</v>
+      </c>
       <c r="N79" s="18"/>
     </row>
     <row r="80" spans="1:14" ht="76.5" x14ac:dyDescent="0.25">
@@ -6382,6 +6403,7 @@
     <hyperlink ref="M75" r:id="rId37" xr:uid="{457EC74B-61C4-4210-8AF2-CCA84EBCDB64}"/>
     <hyperlink ref="M77" r:id="rId38" xr:uid="{0B302733-E9E0-470F-8B09-8E1EBA4EB82D}"/>
     <hyperlink ref="M78" r:id="rId39" xr:uid="{1DF0E4BB-591D-41B6-9EE3-1EFAE674C8A9}"/>
+    <hyperlink ref="M79" r:id="rId40" xr:uid="{F4F6776F-A5F1-4B24-A139-49EE3D1A8F59}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6998,7 +7020,7 @@
       </c>
       <c r="F19" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A19,'Test Case'!$L:$L,"FAIL")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Hoàn thành test TC-24-08
</commit_message>
<xml_diff>
--- a/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
+++ b/tests/Kiểm thử Phần Mềm/TestCases_Nhom5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\project\lan-may-cafe\tests\Kiểm thử Phần Mềm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E7C9ED-CA48-45FE-88E7-087565CA7BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F40F9D69-3DE8-4A86-AFF4-4BEBCC9F95A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="706">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="709">
   <si>
     <t>UC</t>
   </si>
@@ -2242,6 +2242,15 @@
   </si>
   <si>
     <t>KQ-test\TC-24-07.png</t>
+  </si>
+  <si>
+    <t>Hậu</t>
+  </si>
+  <si>
+    <t>đã fix bug</t>
+  </si>
+  <si>
+    <t>KQ-test\TC-24-08.png</t>
   </si>
 </sst>
 </file>
@@ -6351,7 +6360,7 @@
       </c>
       <c r="N86" s="16"/>
     </row>
-    <row r="87" spans="1:14" ht="63.75">
+    <row r="87" spans="1:14" ht="89.25">
       <c r="A87" s="15" t="s">
         <v>653</v>
       </c>
@@ -6382,9 +6391,15 @@
       <c r="J87" s="16" t="s">
         <v>659</v>
       </c>
-      <c r="K87" s="16"/>
-      <c r="L87" s="15"/>
-      <c r="M87" s="16"/>
+      <c r="K87" s="16" t="s">
+        <v>659</v>
+      </c>
+      <c r="L87" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="M87" s="14" t="s">
+        <v>708</v>
+      </c>
       <c r="N87" s="16"/>
     </row>
     <row r="88" spans="1:14" ht="102">
@@ -6539,6 +6554,7 @@
     <hyperlink ref="M84" r:id="rId45" xr:uid="{2B372E0F-1D46-483B-A426-880ABEAADA1E}"/>
     <hyperlink ref="M85" r:id="rId46" xr:uid="{9CA04E1C-9F53-4E68-B0A0-AA1245523970}"/>
     <hyperlink ref="M86" r:id="rId47" xr:uid="{97256925-AE2F-479D-93CF-1CB71939B69B}"/>
+    <hyperlink ref="M87" r:id="rId48" xr:uid="{DF37A6BE-D995-47E3-91B8-7FE1E6D3C4ED}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6617,11 +6633,15 @@
       <c r="G2" t="s">
         <v>433</v>
       </c>
-      <c r="H2" s="1"/>
+      <c r="H2" s="1" t="s">
+        <v>706</v>
+      </c>
       <c r="I2" s="1" t="s">
         <v>698</v>
       </c>
-      <c r="J2" s="1"/>
+      <c r="J2" s="1" t="s">
+        <v>707</v>
+      </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="1"/>
@@ -7129,7 +7149,7 @@
       </c>
       <c r="E17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"PASS")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F17" s="6">
         <f>COUNTIFS('Test Case'!$D:$D,$A17,'Test Case'!$L:$L,"FAIL")</f>

</xml_diff>